<commit_message>
Atualização automática: 2026-09-15 13:03
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U881" headerRowCount="1">
-  <autoFilter ref="A1:U881"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U879" headerRowCount="1">
+  <autoFilter ref="A1:U879"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U881"/>
+  <dimension ref="A1:U879"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="L137" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M137" s="1" t="inlineStr">
@@ -11977,12 +11977,23 @@
       </c>
       <c r="N137" s="1" t="n"/>
       <c r="O137" s="1" t="n"/>
-      <c r="P137" s="1" t="n"/>
-      <c r="Q137" s="1" t="inlineStr"/>
-      <c r="R137" s="1" t="inlineStr"/>
+      <c r="P137" s="2" t="n">
+        <v>46280.51998788195</v>
+      </c>
+      <c r="Q137" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
+      <c r="R137" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde,
+Para regularizar, precisamos retificar os períodos, entretanto, o cliente não paga taxa eletrônica. Por favor, verificar com o cliente sobre o pagamento da taxa.</t>
+        </is>
+      </c>
       <c r="S137" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T137" s="1" t="n"/>
@@ -15765,7 +15776,7 @@
       </c>
       <c r="N182" s="1" t="n"/>
       <c r="O182" s="2" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="P182" s="1" t="n"/>
       <c r="Q182" s="1" t="inlineStr"/>
@@ -52055,69 +52066,59 @@
     </row>
     <row r="680">
       <c r="A680" s="1" t="n">
-        <v>81296</v>
+        <v>84022</v>
       </c>
       <c r="B680" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C680" s="1" t="inlineStr">
         <is>
-          <t>Outras Cláusulas</t>
+          <t xml:space="preserve">Novo </t>
         </is>
       </c>
       <c r="D680" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E680" s="1" t="inlineStr">
         <is>
-          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
+          <t>Estou tentando usar a ferramenta de fechamento e está com a mensagem: Falta informação de contato de endereço Comercial no cadastro do clienteEmpresa: 6977 - PROTECTION SHIELD LTDA</t>
         </is>
       </c>
       <c r="F680" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G680" s="1" t="n"/>
-      <c r="H680" s="1" t="inlineStr">
-        <is>
-          <t>Edson Silva</t>
-        </is>
-      </c>
+      <c r="H680" s="1" t="n"/>
       <c r="I680" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J680" s="2" t="n">
-        <v>46225.4866127662</v>
+        <v>46280.50560975695</v>
       </c>
       <c r="K680" s="2" t="n">
-        <v>46255</v>
+        <v>46281</v>
       </c>
       <c r="L680" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M680" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N680" s="2" t="n">
-        <v>46253.38738584491</v>
-      </c>
+          <t>Gisele Rodrigues</t>
+        </is>
+      </c>
+      <c r="N680" s="1" t="n"/>
       <c r="O680" s="1" t="n"/>
       <c r="P680" s="1" t="n"/>
       <c r="Q680" s="1" t="inlineStr"/>
-      <c r="R680" s="1" t="inlineStr">
-        <is>
-          <t>Raisa, para esse processo, será necessário o envio do IPTU e também que seja informado quem será o responsável tecnico perante o CREMESP, enviando-nos inclusive a carteira do CREMESP do responsável.</t>
-        </is>
-      </c>
+      <c r="R680" s="1" t="n"/>
       <c r="S680" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52128,59 +52129,69 @@
     </row>
     <row r="681">
       <c r="A681" s="1" t="n">
-        <v>83981</v>
+        <v>81296</v>
       </c>
       <c r="B681" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C681" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Outras Cláusulas</t>
         </is>
       </c>
       <c r="D681" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E681" s="1" t="inlineStr">
         <is>
-          <t>3262 - JCV - GNRE de ALPEC - AlagoasConforme solicitação no e-mail anexo, é necessário providenciar o preenchimento do REDAR, emissão da taxa e protocolar do processo junto à SEFAZ/AL.</t>
+          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
         </is>
       </c>
       <c r="F681" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G681" s="1" t="n"/>
-      <c r="H681" s="1" t="n"/>
+      <c r="H681" s="1" t="inlineStr">
+        <is>
+          <t>Edson Silva</t>
+        </is>
+      </c>
       <c r="I681" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J681" s="2" t="n">
-        <v>46280.38897322916</v>
+        <v>46225.4866127662</v>
       </c>
       <c r="K681" s="2" t="n">
-        <v>46282</v>
+        <v>46255</v>
       </c>
       <c r="L681" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M681" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
-      <c r="N681" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N681" s="2" t="n">
+        <v>46253.38738584491</v>
+      </c>
       <c r="O681" s="1" t="n"/>
       <c r="P681" s="1" t="n"/>
       <c r="Q681" s="1" t="inlineStr"/>
-      <c r="R681" s="1" t="n"/>
+      <c r="R681" s="1" t="inlineStr">
+        <is>
+          <t>Raisa, para esse processo, será necessário o envio do IPTU e também que seja informado quem será o responsável tecnico perante o CREMESP, enviando-nos inclusive a carteira do CREMESP do responsável.</t>
+        </is>
+      </c>
       <c r="S681" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52191,16 +52202,16 @@
     </row>
     <row r="682">
       <c r="A682" s="1" t="n">
-        <v>83985</v>
+        <v>83981</v>
       </c>
       <c r="B682" s="1" t="inlineStr">
         <is>
-          <t>Procuração</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C682" s="1" t="inlineStr">
         <is>
-          <t>Fiscalização Federal</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="D682" s="1" t="inlineStr">
@@ -52210,7 +52221,7 @@
       </c>
       <c r="E682" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, preciso que vincule a empresa 7041 - PROMOTORAS GYN ao certificado da SDD</t>
+          <t>3262 - JCV - GNRE de ALPEC - AlagoasConforme solicitação no e-mail anexo, é necessário providenciar o preenchimento do REDAR, emissão da taxa e protocolar do processo junto à SEFAZ/AL.</t>
         </is>
       </c>
       <c r="F682" s="1" t="n">
@@ -52224,7 +52235,7 @@
         </is>
       </c>
       <c r="J682" s="2" t="n">
-        <v>46280.41337118056</v>
+        <v>46280.38897322916</v>
       </c>
       <c r="K682" s="2" t="n">
         <v>46282</v>
@@ -52236,7 +52247,7 @@
       </c>
       <c r="M682" s="1" t="inlineStr">
         <is>
-          <t>Gisele Rodrigues</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="N682" s="1" t="n"/>
@@ -59833,7 +59844,7 @@
       </c>
       <c r="I782" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J782" s="2" t="n">
@@ -59844,7 +59855,7 @@
       </c>
       <c r="L782" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M782" s="1" t="inlineStr">
@@ -59852,9 +59863,7 @@
           <t>Ricardo Ferreira</t>
         </is>
       </c>
-      <c r="N782" s="2" t="n">
-        <v>46268.41803993056</v>
-      </c>
+      <c r="N782" s="1" t="n"/>
       <c r="O782" s="1" t="n"/>
       <c r="P782" s="1" t="n"/>
       <c r="Q782" s="1" t="inlineStr"/>
@@ -59868,7 +59877,11 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T782" s="1" t="n"/>
+      <c r="T782" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
       <c r="U782" s="1" t="inlineStr"/>
     </row>
     <row r="783">
@@ -63246,7 +63259,7 @@
       </c>
       <c r="L828" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M828" s="1" t="inlineStr">
@@ -63254,7 +63267,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N828" s="1" t="n"/>
+      <c r="N828" s="2" t="n">
+        <v>46267.54541188657</v>
+      </c>
       <c r="O828" s="2" t="n">
         <v>46283</v>
       </c>
@@ -64898,7 +64913,7 @@
       </c>
       <c r="L849" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M849" s="1" t="inlineStr">
@@ -64906,7 +64921,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N849" s="1" t="n"/>
+      <c r="N849" s="2" t="n">
+        <v>46255.4431121875</v>
+      </c>
       <c r="O849" s="2" t="n">
         <v>46283</v>
       </c>
@@ -65198,7 +65215,7 @@
       </c>
       <c r="L853" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M853" s="1" t="inlineStr">
@@ -65206,7 +65223,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N853" s="1" t="n"/>
+      <c r="N853" s="2" t="n">
+        <v>46255.48540517361</v>
+      </c>
       <c r="O853" s="1" t="n"/>
       <c r="P853" s="1" t="n"/>
       <c r="Q853" s="1" t="inlineStr"/>
@@ -65298,7 +65317,7 @@
     </row>
     <row r="855">
       <c r="A855" s="1" t="n">
-        <v>81052</v>
+        <v>81055</v>
       </c>
       <c r="B855" s="1" t="inlineStr">
         <is>
@@ -65317,7 +65336,7 @@
       </c>
       <c r="E855" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F855" s="1" t="n">
@@ -65335,7 +65354,7 @@
         </is>
       </c>
       <c r="J855" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K855" s="2" t="n">
         <v>46219</v>
@@ -65351,7 +65370,7 @@
         </is>
       </c>
       <c r="N855" s="2" t="n">
-        <v>46219.50471747686</v>
+        <v>46219.50607847222</v>
       </c>
       <c r="O855" s="2" t="n">
         <v>46283</v>
@@ -65360,7 +65379,7 @@
       <c r="Q855" s="1" t="inlineStr"/>
       <c r="R855" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t>Aguardando retorno dos dados do contador</t>
         </is>
       </c>
       <c r="S855" s="1" t="inlineStr">
@@ -65373,74 +65392,83 @@
     </row>
     <row r="856">
       <c r="A856" s="1" t="n">
-        <v>81055</v>
+        <v>82881</v>
       </c>
       <c r="B856" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Produtos</t>
         </is>
       </c>
       <c r="C856" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Cadastro de produtos</t>
         </is>
       </c>
       <c r="D856" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>RJ - GC ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E856" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t xml:space="preserve">Prezados, bom dia.Estou formalizando, via chamado, a solicitação de revisão do cadastro de produtos da empresa.Em anexo, encaminho o e-mail com a tratativa referente ao assunto. </t>
         </is>
       </c>
       <c r="F856" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G856" s="1" t="n"/>
+        <v>6336</v>
+      </c>
+      <c r="G856" s="1" t="inlineStr">
+        <is>
+          <t>BEL LINE COMERCIO DE COSMETICOS LTDA</t>
+        </is>
+      </c>
       <c r="H856" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Fernanda Bertunes</t>
         </is>
       </c>
       <c r="I856" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>CADASTRO DE PRODUTOS</t>
         </is>
       </c>
       <c r="J856" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46258.42822939815</v>
       </c>
       <c r="K856" s="2" t="n">
-        <v>46219</v>
+        <v>46288</v>
       </c>
       <c r="L856" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M856" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N856" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N856" s="1" t="n"/>
       <c r="O856" s="2" t="n">
-        <v>46283</v>
-      </c>
-      <c r="P856" s="1" t="n"/>
-      <c r="Q856" s="1" t="inlineStr"/>
+        <v>46269</v>
+      </c>
+      <c r="P856" s="2" t="n">
+        <v>46265.43684837963</v>
+      </c>
+      <c r="Q856" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
       <c r="R856" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t>Bom dia 
+Cadastro analisado e enviado por email</t>
         </is>
       </c>
       <c r="S856" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T856" s="1" t="n"/>
@@ -65448,69 +65476,72 @@
     </row>
     <row r="857">
       <c r="A857" s="1" t="n">
-        <v>82430</v>
+        <v>81757</v>
       </c>
       <c r="B857" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Produtos</t>
         </is>
       </c>
       <c r="C857" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Cadastro de produtos</t>
         </is>
       </c>
       <c r="D857" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E857" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia!Segue checklist atualizado da empresa 7007 - SANTOS&amp;DIAN Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>6945 - BRASIL DISTRIBUIDORA DE PEÇAS - CADASTRO DE INTENS, PARA INCLUSÃO DE INFORMAÇÕES TRIBUTÁRIAS.Por favor dar início na inclusão das informações tributarias no cadastro de itens do clienteAtt.Vander</t>
         </is>
       </c>
       <c r="F857" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G857" s="1" t="n"/>
+        <v>6945</v>
+      </c>
+      <c r="G857" s="1" t="inlineStr">
+        <is>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+        </is>
+      </c>
       <c r="H857" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Fernanda Bertunes</t>
         </is>
       </c>
       <c r="I857" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>CADASTRO DE PRODUTOS</t>
         </is>
       </c>
       <c r="J857" s="2" t="n">
-        <v>46248.47311612269</v>
+        <v>46237.52224869213</v>
       </c>
       <c r="K857" s="2" t="n">
-        <v>46251</v>
+        <v>46267</v>
       </c>
       <c r="L857" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M857" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N857" s="2" t="n">
-        <v>46253.38669748843</v>
-      </c>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N857" s="1" t="n"/>
       <c r="O857" s="2" t="n">
-        <v>46283</v>
+        <v>46267</v>
       </c>
       <c r="P857" s="1" t="n"/>
       <c r="Q857" s="1" t="inlineStr"/>
       <c r="R857" s="1" t="inlineStr">
         <is>
-          <t>cobramos novamente o antigo contador</t>
+          <t xml:space="preserve">Por favor , enviar a planilha de cadastro no layout padrão para analise 
+Enviar a planilha no layout correto e abrir novo chamado anexando email </t>
         </is>
       </c>
       <c r="S857" s="1" t="inlineStr">
@@ -65523,7 +65554,7 @@
     </row>
     <row r="858">
       <c r="A858" s="1" t="n">
-        <v>82881</v>
+        <v>82777</v>
       </c>
       <c r="B858" s="1" t="inlineStr">
         <is>
@@ -65537,20 +65568,20 @@
       </c>
       <c r="D858" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>RJ - GC</t>
         </is>
       </c>
       <c r="E858" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, bom dia.Estou formalizando, via chamado, a solicitação de revisão do cadastro de produtos da empresa.Em anexo, encaminho o e-mail com a tratativa referente ao assunto. </t>
+          <t>Prezados, bom dia!Enviei um e-mail sobre a solicitação da Jéssica sobre o cliente JEM TRUCK.Por favor verificar e validar se chegam a mesma conclusão antes de envio ao cliente.</t>
         </is>
       </c>
       <c r="F858" s="1" t="n">
-        <v>6336</v>
+        <v>6979</v>
       </c>
       <c r="G858" s="1" t="inlineStr">
         <is>
-          <t>BEL LINE COMERCIO DE COSMETICOS LTDA</t>
+          <t xml:space="preserve">JEM TRUCK TRANSPORTE DE CARGAS E TERRAPLANAGEM LTDA </t>
         </is>
       </c>
       <c r="H858" s="1" t="inlineStr">
@@ -65564,10 +65595,10 @@
         </is>
       </c>
       <c r="J858" s="2" t="n">
-        <v>46258.42822939815</v>
+        <v>46255.4226837963</v>
       </c>
       <c r="K858" s="2" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L858" s="1" t="inlineStr">
         <is>
@@ -65576,15 +65607,15 @@
       </c>
       <c r="M858" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
+          <t>Maicon Costa</t>
         </is>
       </c>
       <c r="N858" s="1" t="n"/>
       <c r="O858" s="2" t="n">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="P858" s="2" t="n">
-        <v>46265.43684837963</v>
+        <v>46262.63475393518</v>
       </c>
       <c r="Q858" s="1" t="inlineStr">
         <is>
@@ -65592,174 +65623,181 @@
         </is>
       </c>
       <c r="R858" s="1" t="inlineStr">
-        <is>
-          <t>Bom dia 
-Cadastro analisado e enviado por email</t>
-        </is>
-      </c>
-      <c r="S858" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T858" s="1" t="n"/>
-      <c r="U858" s="1" t="inlineStr"/>
-    </row>
-    <row r="859">
-      <c r="A859" s="1" t="n">
-        <v>81757</v>
-      </c>
-      <c r="B859" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de Produtos</t>
-        </is>
-      </c>
-      <c r="C859" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de produtos</t>
-        </is>
-      </c>
-      <c r="D859" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E859" s="1" t="inlineStr">
-        <is>
-          <t>6945 - BRASIL DISTRIBUIDORA DE PEÇAS - CADASTRO DE INTENS, PARA INCLUSÃO DE INFORMAÇÕES TRIBUTÁRIAS.Por favor dar início na inclusão das informações tributarias no cadastro de itens do clienteAtt.Vander</t>
-        </is>
-      </c>
-      <c r="F859" s="1" t="n">
-        <v>6945</v>
-      </c>
-      <c r="G859" s="1" t="inlineStr">
-        <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
-        </is>
-      </c>
-      <c r="H859" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="I859" s="1" t="inlineStr">
-        <is>
-          <t>CADASTRO DE PRODUTOS</t>
-        </is>
-      </c>
-      <c r="J859" s="2" t="n">
-        <v>46237.52224869213</v>
-      </c>
-      <c r="K859" s="2" t="n">
-        <v>46267</v>
-      </c>
-      <c r="L859" s="1" t="inlineStr">
-        <is>
-          <t>Devolvido</t>
-        </is>
-      </c>
-      <c r="M859" s="1" t="inlineStr">
-        <is>
-          <t>Vander Silva</t>
-        </is>
-      </c>
-      <c r="N859" s="1" t="n"/>
-      <c r="O859" s="2" t="n">
-        <v>46267</v>
-      </c>
-      <c r="P859" s="1" t="n"/>
-      <c r="Q859" s="1" t="inlineStr"/>
-      <c r="R859" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Por favor , enviar a planilha de cadastro no layout padrão para analise 
-Enviar a planilha no layout correto e abrir novo chamado anexando email </t>
-        </is>
-      </c>
-      <c r="S859" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T859" s="1" t="n"/>
-      <c r="U859" s="1" t="inlineStr"/>
-    </row>
-    <row r="860">
-      <c r="A860" s="1" t="n">
-        <v>82777</v>
-      </c>
-      <c r="B860" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de Produtos</t>
-        </is>
-      </c>
-      <c r="C860" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de produtos</t>
-        </is>
-      </c>
-      <c r="D860" s="1" t="inlineStr">
-        <is>
-          <t>RJ - GC</t>
-        </is>
-      </c>
-      <c r="E860" s="1" t="inlineStr">
-        <is>
-          <t>Prezados, bom dia!Enviei um e-mail sobre a solicitação da Jéssica sobre o cliente JEM TRUCK.Por favor verificar e validar se chegam a mesma conclusão antes de envio ao cliente.</t>
-        </is>
-      </c>
-      <c r="F860" s="1" t="n">
-        <v>6979</v>
-      </c>
-      <c r="G860" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JEM TRUCK TRANSPORTE DE CARGAS E TERRAPLANAGEM LTDA </t>
-        </is>
-      </c>
-      <c r="H860" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="I860" s="1" t="inlineStr">
-        <is>
-          <t>CADASTRO DE PRODUTOS</t>
-        </is>
-      </c>
-      <c r="J860" s="2" t="n">
-        <v>46255.4226837963</v>
-      </c>
-      <c r="K860" s="2" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L860" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M860" s="1" t="inlineStr">
-        <is>
-          <t>Maicon Costa</t>
-        </is>
-      </c>
-      <c r="N860" s="1" t="n"/>
-      <c r="O860" s="2" t="n">
-        <v>46267</v>
-      </c>
-      <c r="P860" s="2" t="n">
-        <v>46262.63475393518</v>
-      </c>
-      <c r="Q860" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="R860" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Boa tarde 
 Informação já respondida por email
 Assuntos sobre duvidas tributarias, não deve ser aberto chamado </t>
         </is>
       </c>
+      <c r="S858" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T858" s="1" t="n"/>
+      <c r="U858" s="1" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" s="1" t="n">
+        <v>82815</v>
+      </c>
+      <c r="B859" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C859" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D859" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E859" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F859" s="1" t="n">
+        <v>5789</v>
+      </c>
+      <c r="G859" s="1" t="inlineStr">
+        <is>
+          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
+        </is>
+      </c>
+      <c r="H859" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I859" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J859" s="2" t="n">
+        <v>46255.67638510417</v>
+      </c>
+      <c r="K859" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L859" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M859" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N859" s="2" t="n">
+        <v>46262.65963637731</v>
+      </c>
+      <c r="O859" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P859" s="2" t="n">
+        <v>46266.5932252662</v>
+      </c>
+      <c r="Q859" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R859" s="1" t="inlineStr">
+        <is>
+          <t>Em fila para atendimento</t>
+        </is>
+      </c>
+      <c r="S859" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T859" s="1" t="n"/>
+      <c r="U859" s="1" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" s="1" t="n">
+        <v>82817</v>
+      </c>
+      <c r="B860" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C860" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D860" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E860" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F860" s="1" t="n">
+        <v>3808</v>
+      </c>
+      <c r="G860" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mercearia Doce Bom Ltda. </t>
+        </is>
+      </c>
+      <c r="H860" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I860" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J860" s="2" t="n">
+        <v>46255.6791724537</v>
+      </c>
+      <c r="K860" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L860" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M860" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N860" s="1" t="n"/>
+      <c r="O860" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P860" s="2" t="n">
+        <v>46262.65880697917</v>
+      </c>
+      <c r="Q860" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R860" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde
+Cadastro analisado e devolvido por email em 24/08</t>
+        </is>
+      </c>
       <c r="S860" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -65770,7 +65808,7 @@
     </row>
     <row r="861">
       <c r="A861" s="1" t="n">
-        <v>82815</v>
+        <v>82818</v>
       </c>
       <c r="B861" s="1" t="inlineStr">
         <is>
@@ -65793,11 +65831,11 @@
         </is>
       </c>
       <c r="F861" s="1" t="n">
-        <v>5789</v>
+        <v>4222</v>
       </c>
       <c r="G861" s="1" t="inlineStr">
         <is>
-          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
+          <t>STOCK FRANGO DISTRIBUIDORA DE GÊNEROS ALIMENTÍCIOS E TRANSPORTE LTDA</t>
         </is>
       </c>
       <c r="H861" s="1" t="inlineStr">
@@ -65811,7 +65849,7 @@
         </is>
       </c>
       <c r="J861" s="2" t="n">
-        <v>46255.67638510417</v>
+        <v>46255.67973850694</v>
       </c>
       <c r="K861" s="2" t="n">
         <v>46287</v>
@@ -65826,14 +65864,12 @@
           <t>Lohany Martins</t>
         </is>
       </c>
-      <c r="N861" s="2" t="n">
-        <v>46262.65963637731</v>
-      </c>
+      <c r="N861" s="1" t="n"/>
       <c r="O861" s="2" t="n">
         <v>46269</v>
       </c>
       <c r="P861" s="2" t="n">
-        <v>46266.5932252662</v>
+        <v>46262.65957361111</v>
       </c>
       <c r="Q861" s="1" t="inlineStr">
         <is>
@@ -65842,7 +65878,8 @@
       </c>
       <c r="R861" s="1" t="inlineStr">
         <is>
-          <t>Em fila para atendimento</t>
+          <t>Boa tarde 
+Cadastro analisado e enviado por email em 24/08</t>
         </is>
       </c>
       <c r="S861" s="1" t="inlineStr">
@@ -65855,7 +65892,7 @@
     </row>
     <row r="862">
       <c r="A862" s="1" t="n">
-        <v>82817</v>
+        <v>82819</v>
       </c>
       <c r="B862" s="1" t="inlineStr">
         <is>
@@ -65878,11 +65915,11 @@
         </is>
       </c>
       <c r="F862" s="1" t="n">
-        <v>3808</v>
+        <v>6529</v>
       </c>
       <c r="G862" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mercearia Doce Bom Ltda. </t>
+          <t>VALLEMAR MERCADO LTDA</t>
         </is>
       </c>
       <c r="H862" s="1" t="inlineStr">
@@ -65896,7 +65933,7 @@
         </is>
       </c>
       <c r="J862" s="2" t="n">
-        <v>46255.6791724537</v>
+        <v>46255.68034375</v>
       </c>
       <c r="K862" s="2" t="n">
         <v>46287</v>
@@ -65916,7 +65953,7 @@
         <v>46269</v>
       </c>
       <c r="P862" s="2" t="n">
-        <v>46262.65880697917</v>
+        <v>46262.66115917824</v>
       </c>
       <c r="Q862" s="1" t="inlineStr">
         <is>
@@ -65925,7 +65962,7 @@
       </c>
       <c r="R862" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde
+          <t>Boa tarde 
 Cadastro analisado e devolvido por email em 24/08</t>
         </is>
       </c>
@@ -65939,7 +65976,7 @@
     </row>
     <row r="863">
       <c r="A863" s="1" t="n">
-        <v>82818</v>
+        <v>82901</v>
       </c>
       <c r="B863" s="1" t="inlineStr">
         <is>
@@ -65962,11 +65999,11 @@
         </is>
       </c>
       <c r="F863" s="1" t="n">
-        <v>4222</v>
+        <v>4604</v>
       </c>
       <c r="G863" s="1" t="inlineStr">
         <is>
-          <t>STOCK FRANGO DISTRIBUIDORA DE GÊNEROS ALIMENTÍCIOS E TRANSPORTE LTDA</t>
+          <t>H P T COMERCIO E INDUSTRIA DE MÓVEIS LTDA</t>
         </is>
       </c>
       <c r="H863" s="1" t="inlineStr">
@@ -65980,10 +66017,10 @@
         </is>
       </c>
       <c r="J863" s="2" t="n">
-        <v>46255.67973850694</v>
+        <v>46258.64696304398</v>
       </c>
       <c r="K863" s="2" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="L863" s="1" t="inlineStr">
         <is>
@@ -65995,12 +66032,14 @@
           <t>Lohany Martins</t>
         </is>
       </c>
-      <c r="N863" s="1" t="n"/>
+      <c r="N863" s="2" t="n">
+        <v>46265.43650153935</v>
+      </c>
       <c r="O863" s="2" t="n">
         <v>46269</v>
       </c>
       <c r="P863" s="2" t="n">
-        <v>46262.65957361111</v>
+        <v>46266.6452650463</v>
       </c>
       <c r="Q863" s="1" t="inlineStr">
         <is>
@@ -66009,8 +66048,7 @@
       </c>
       <c r="R863" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde 
-Cadastro analisado e enviado por email em 24/08</t>
+          <t>Na fila para atendimento</t>
         </is>
       </c>
       <c r="S863" s="1" t="inlineStr">
@@ -66023,7 +66061,7 @@
     </row>
     <row r="864">
       <c r="A864" s="1" t="n">
-        <v>82819</v>
+        <v>82924</v>
       </c>
       <c r="B864" s="1" t="inlineStr">
         <is>
@@ -66046,11 +66084,11 @@
         </is>
       </c>
       <c r="F864" s="1" t="n">
-        <v>6529</v>
+        <v>5739</v>
       </c>
       <c r="G864" s="1" t="inlineStr">
         <is>
-          <t>VALLEMAR MERCADO LTDA</t>
+          <t>GOLD REAL MOVEIS LTDA</t>
         </is>
       </c>
       <c r="H864" s="1" t="inlineStr">
@@ -66064,10 +66102,10 @@
         </is>
       </c>
       <c r="J864" s="2" t="n">
-        <v>46255.68034375</v>
+        <v>46258.73919143518</v>
       </c>
       <c r="K864" s="2" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="L864" s="1" t="inlineStr">
         <is>
@@ -66079,12 +66117,14 @@
           <t>Lohany Martins</t>
         </is>
       </c>
-      <c r="N864" s="1" t="n"/>
+      <c r="N864" s="2" t="n">
+        <v>46265.44787318287</v>
+      </c>
       <c r="O864" s="2" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="P864" s="2" t="n">
-        <v>46262.66115917824</v>
+        <v>46266.64227896991</v>
       </c>
       <c r="Q864" s="1" t="inlineStr">
         <is>
@@ -66093,8 +66133,7 @@
       </c>
       <c r="R864" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde 
-Cadastro analisado e devolvido por email em 24/08</t>
+          <t xml:space="preserve">Em fila de atendimento </t>
         </is>
       </c>
       <c r="S864" s="1" t="inlineStr">
@@ -66107,7 +66146,7 @@
     </row>
     <row r="865">
       <c r="A865" s="1" t="n">
-        <v>82901</v>
+        <v>82951</v>
       </c>
       <c r="B865" s="1" t="inlineStr">
         <is>
@@ -66126,15 +66165,15 @@
       </c>
       <c r="E865" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+          <t>Bom dia, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
         </is>
       </c>
       <c r="F865" s="1" t="n">
-        <v>4604</v>
+        <v>3959</v>
       </c>
       <c r="G865" s="1" t="inlineStr">
         <is>
-          <t>H P T COMERCIO E INDUSTRIA DE MÓVEIS LTDA</t>
+          <t>ALDEBARAN DISTRIBUIDORA E COMÉRCIO DE MATERIAL MÉDICO E HOSPITALAR LTDA</t>
         </is>
       </c>
       <c r="H865" s="1" t="inlineStr">
@@ -66148,14 +66187,14 @@
         </is>
       </c>
       <c r="J865" s="2" t="n">
-        <v>46258.64696304398</v>
+        <v>46259.43735</v>
       </c>
       <c r="K865" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="L865" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M865" s="1" t="inlineStr">
@@ -66164,27 +66203,21 @@
         </is>
       </c>
       <c r="N865" s="2" t="n">
-        <v>46265.43650153935</v>
+        <v>46265.45876041667</v>
       </c>
       <c r="O865" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="P865" s="2" t="n">
-        <v>46266.6452650463</v>
-      </c>
-      <c r="Q865" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
+        <v>46273</v>
+      </c>
+      <c r="P865" s="1" t="n"/>
+      <c r="Q865" s="1" t="inlineStr"/>
       <c r="R865" s="1" t="inlineStr">
         <is>
-          <t>Na fila para atendimento</t>
+          <t xml:space="preserve">Em fila de atendimento </t>
         </is>
       </c>
       <c r="S865" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T865" s="1" t="n"/>
@@ -66192,7 +66225,7 @@
     </row>
     <row r="866">
       <c r="A866" s="1" t="n">
-        <v>82924</v>
+        <v>83005</v>
       </c>
       <c r="B866" s="1" t="inlineStr">
         <is>
@@ -66215,11 +66248,11 @@
         </is>
       </c>
       <c r="F866" s="1" t="n">
-        <v>5739</v>
+        <v>6523</v>
       </c>
       <c r="G866" s="1" t="inlineStr">
         <is>
-          <t>GOLD REAL MOVEIS LTDA</t>
+          <t>PARADA DOS PAES LTDA</t>
         </is>
       </c>
       <c r="H866" s="1" t="inlineStr">
@@ -66233,10 +66266,10 @@
         </is>
       </c>
       <c r="J866" s="2" t="n">
-        <v>46258.73919143518</v>
+        <v>46259.70646643519</v>
       </c>
       <c r="K866" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="L866" s="1" t="inlineStr">
         <is>
@@ -66249,13 +66282,13 @@
         </is>
       </c>
       <c r="N866" s="2" t="n">
-        <v>46265.44787318287</v>
+        <v>46265.51365540509</v>
       </c>
       <c r="O866" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="P866" s="2" t="n">
-        <v>46266.64227896991</v>
+        <v>46268.69805833334</v>
       </c>
       <c r="Q866" s="1" t="inlineStr">
         <is>
@@ -66264,7 +66297,7 @@
       </c>
       <c r="R866" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em fila de atendimento </t>
+          <t>Em fila de atendimento</t>
         </is>
       </c>
       <c r="S866" s="1" t="inlineStr">
@@ -66277,34 +66310,34 @@
     </row>
     <row r="867">
       <c r="A867" s="1" t="n">
-        <v>82951</v>
+        <v>82502</v>
       </c>
       <c r="B867" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Produtos</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C867" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de produtos</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D867" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E867" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+          <t>6070	MEGACAR	Cliente informou que já enviou o cadastro de produto, por favor verificar se já foi revisado e devolvido para o cliente. Como esta o andamento?</t>
         </is>
       </c>
       <c r="F867" s="1" t="n">
-        <v>3959</v>
+        <v>6070</v>
       </c>
       <c r="G867" s="1" t="inlineStr">
         <is>
-          <t>ALDEBARAN DISTRIBUIDORA E COMÉRCIO DE MATERIAL MÉDICO E HOSPITALAR LTDA</t>
+          <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
         </is>
       </c>
       <c r="H867" s="1" t="inlineStr">
@@ -66318,37 +66351,40 @@
         </is>
       </c>
       <c r="J867" s="2" t="n">
-        <v>46259.43735</v>
+        <v>46251.42708194444</v>
       </c>
       <c r="K867" s="2" t="n">
-        <v>46290</v>
+        <v>46258</v>
       </c>
       <c r="L867" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M867" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
-        </is>
-      </c>
-      <c r="N867" s="2" t="n">
-        <v>46265.45876041667</v>
-      </c>
-      <c r="O867" s="2" t="n">
-        <v>46273</v>
-      </c>
-      <c r="P867" s="1" t="n"/>
-      <c r="Q867" s="1" t="inlineStr"/>
+          <t>Leticia Queiroz</t>
+        </is>
+      </c>
+      <c r="N867" s="1" t="n"/>
+      <c r="O867" s="1" t="n"/>
+      <c r="P867" s="2" t="n">
+        <v>46261.54547850695</v>
+      </c>
+      <c r="Q867" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
       <c r="R867" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em fila de atendimento </t>
+          <t xml:space="preserve">Em 2026, não recebemos nenhuma solicitação referente a esse cliente 
+Por favor, solicitar o cadastro de produtos atualizado, enviar por email para @integracaocadastroechat e abrir novo chamado </t>
         </is>
       </c>
       <c r="S867" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T867" s="1" t="n"/>
@@ -66356,7 +66392,7 @@
     </row>
     <row r="868">
       <c r="A868" s="1" t="n">
-        <v>83005</v>
+        <v>83231</v>
       </c>
       <c r="B868" s="1" t="inlineStr">
         <is>
@@ -66370,20 +66406,20 @@
       </c>
       <c r="D868" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E868" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+          <t>Por gentileza, realizar a analise do cadastro dos produtos anexo.</t>
         </is>
       </c>
       <c r="F868" s="1" t="n">
-        <v>6523</v>
+        <v>4469</v>
       </c>
       <c r="G868" s="1" t="inlineStr">
         <is>
-          <t>PARADA DOS PAES LTDA</t>
+          <t xml:space="preserve">REI DOS GRÃOS LTDA </t>
         </is>
       </c>
       <c r="H868" s="1" t="inlineStr">
@@ -66397,10 +66433,10 @@
         </is>
       </c>
       <c r="J868" s="2" t="n">
-        <v>46259.70646643519</v>
+        <v>46262.59248885416</v>
       </c>
       <c r="K868" s="2" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="L868" s="1" t="inlineStr">
         <is>
@@ -66409,17 +66445,15 @@
       </c>
       <c r="M868" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N868" s="2" t="n">
-        <v>46265.51365540509</v>
-      </c>
-      <c r="O868" s="2" t="n">
-        <v>46273</v>
-      </c>
+        <v>46265.59963434028</v>
+      </c>
+      <c r="O868" s="1" t="n"/>
       <c r="P868" s="2" t="n">
-        <v>46268.69805833334</v>
+        <v>46269.6534278125</v>
       </c>
       <c r="Q868" s="1" t="inlineStr">
         <is>
@@ -66428,7 +66462,8 @@
       </c>
       <c r="R868" s="1" t="inlineStr">
         <is>
-          <t>Em fila de atendimento</t>
+          <t xml:space="preserve">Em fila de atendimento
+Por favor sempre anexar o email no chamado </t>
         </is>
       </c>
       <c r="S868" s="1" t="inlineStr">
@@ -66441,34 +66476,34 @@
     </row>
     <row r="869">
       <c r="A869" s="1" t="n">
-        <v>82502</v>
+        <v>83139</v>
       </c>
       <c r="B869" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Cadastro de Produtos</t>
         </is>
       </c>
       <c r="C869" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Cadastro de produtos</t>
         </is>
       </c>
       <c r="D869" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>RJ - GC ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E869" s="1" t="inlineStr">
         <is>
-          <t>6070	MEGACAR	Cliente informou que já enviou o cadastro de produto, por favor verificar se já foi revisado e devolvido para o cliente. Como esta o andamento?</t>
+          <t>Prezados, boa tarde! Segue anexo e-mail enviado com a planilha de cadastro de produtos da empresa.</t>
         </is>
       </c>
       <c r="F869" s="1" t="n">
-        <v>6070</v>
+        <v>6049</v>
       </c>
       <c r="G869" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
+          <t>ESTACAO DO PEIXE RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="H869" s="1" t="inlineStr">
@@ -66482,40 +66517,35 @@
         </is>
       </c>
       <c r="J869" s="2" t="n">
-        <v>46251.42708194444</v>
+        <v>46261.59434112268</v>
       </c>
       <c r="K869" s="2" t="n">
-        <v>46258</v>
+        <v>46294</v>
       </c>
       <c r="L869" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M869" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
-      <c r="N869" s="1" t="n"/>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N869" s="2" t="n">
+        <v>46265.60815690972</v>
+      </c>
       <c r="O869" s="1" t="n"/>
-      <c r="P869" s="2" t="n">
-        <v>46261.54547850695</v>
-      </c>
-      <c r="Q869" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
+      <c r="P869" s="1" t="n"/>
+      <c r="Q869" s="1" t="inlineStr"/>
       <c r="R869" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em 2026, não recebemos nenhuma solicitação referente a esse cliente 
-Por favor, solicitar o cadastro de produtos atualizado, enviar por email para @integracaocadastroechat e abrir novo chamado </t>
+          <t>Em fila de atendimento</t>
         </is>
       </c>
       <c r="S869" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T869" s="1" t="n"/>
@@ -66523,7 +66553,7 @@
     </row>
     <row r="870">
       <c r="A870" s="1" t="n">
-        <v>83231</v>
+        <v>83262</v>
       </c>
       <c r="B870" s="1" t="inlineStr">
         <is>
@@ -66537,20 +66567,20 @@
       </c>
       <c r="D870" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>RJ - GC ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E870" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, realizar a analise do cadastro dos produtos anexo.</t>
+          <t xml:space="preserve">Prezados, bom dia! Segue e-mail enviado com a planilha de cadastro de produtos. </t>
         </is>
       </c>
       <c r="F870" s="1" t="n">
-        <v>4469</v>
+        <v>6540</v>
       </c>
       <c r="G870" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">REI DOS GRÃOS LTDA </t>
+          <t>MERCADINHO BAMBINA LTDA</t>
         </is>
       </c>
       <c r="H870" s="1" t="inlineStr">
@@ -66564,10 +66594,10 @@
         </is>
       </c>
       <c r="J870" s="2" t="n">
-        <v>46262.59248885416</v>
+        <v>46265.4616653125</v>
       </c>
       <c r="K870" s="2" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="L870" s="1" t="inlineStr">
         <is>
@@ -66576,15 +66606,15 @@
       </c>
       <c r="M870" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Amanda Mesquita</t>
         </is>
       </c>
       <c r="N870" s="2" t="n">
-        <v>46265.59963434028</v>
+        <v>46265.62414548611</v>
       </c>
       <c r="O870" s="1" t="n"/>
       <c r="P870" s="2" t="n">
-        <v>46269.6534278125</v>
+        <v>46276.71389502315</v>
       </c>
       <c r="Q870" s="1" t="inlineStr">
         <is>
@@ -66593,8 +66623,7 @@
       </c>
       <c r="R870" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em fila de atendimento
-Por favor sempre anexar o email no chamado </t>
+          <t>Em fila de atendimento</t>
         </is>
       </c>
       <c r="S870" s="1" t="inlineStr">
@@ -66607,7 +66636,7 @@
     </row>
     <row r="871">
       <c r="A871" s="1" t="n">
-        <v>83139</v>
+        <v>83367</v>
       </c>
       <c r="B871" s="1" t="inlineStr">
         <is>
@@ -66626,15 +66655,15 @@
       </c>
       <c r="E871" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde! Segue anexo e-mail enviado com a planilha de cadastro de produtos da empresa.</t>
+          <t>Prezados, boa tarde!Segue em anexo cadastro de produtos da empresa 5789 – ACE FRUIT para validação do CBS/IBS.</t>
         </is>
       </c>
       <c r="F871" s="1" t="n">
-        <v>6049</v>
+        <v>5789</v>
       </c>
       <c r="G871" s="1" t="inlineStr">
         <is>
-          <t>ESTACAO DO PEIXE RESTAURANTE LTDA</t>
+          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
         </is>
       </c>
       <c r="H871" s="1" t="inlineStr">
@@ -66648,10 +66677,10 @@
         </is>
       </c>
       <c r="J871" s="2" t="n">
-        <v>46261.59434112268</v>
+        <v>46266.64626565972</v>
       </c>
       <c r="K871" s="2" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="L871" s="1" t="inlineStr">
         <is>
@@ -66660,18 +66689,18 @@
       </c>
       <c r="M871" s="1" t="inlineStr">
         <is>
-          <t>Amanda Mesquita</t>
+          <t>Lohany Martins</t>
         </is>
       </c>
       <c r="N871" s="2" t="n">
-        <v>46265.60815690972</v>
+        <v>46269.66462141203</v>
       </c>
       <c r="O871" s="1" t="n"/>
       <c r="P871" s="1" t="n"/>
       <c r="Q871" s="1" t="inlineStr"/>
       <c r="R871" s="1" t="inlineStr">
         <is>
-          <t>Em fila de atendimento</t>
+          <t>Em fila para atendimento</t>
         </is>
       </c>
       <c r="S871" s="1" t="inlineStr">
@@ -66684,7 +66713,7 @@
     </row>
     <row r="872">
       <c r="A872" s="1" t="n">
-        <v>83262</v>
+        <v>83429</v>
       </c>
       <c r="B872" s="1" t="inlineStr">
         <is>
@@ -66703,15 +66732,15 @@
       </c>
       <c r="E872" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, bom dia! Segue e-mail enviado com a planilha de cadastro de produtos. </t>
+          <t xml:space="preserve">Prezados, boa tarde!Segue novamente planilha de IBS/CBS da empresa 3965 - TUTTI DELI, ela já foi enviada anteriormente o número do chamado antigo é 82784, porém ela foi retornada mesmo estando completa. Na planilha consta NCM, Descrição e EAN. </t>
         </is>
       </c>
       <c r="F872" s="1" t="n">
-        <v>6540</v>
+        <v>3965</v>
       </c>
       <c r="G872" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO BAMBINA LTDA</t>
+          <t>TUTTI QUITUTE PRODUTOS ALIMENTICIOS LTDA</t>
         </is>
       </c>
       <c r="H872" s="1" t="inlineStr">
@@ -66725,41 +66754,29 @@
         </is>
       </c>
       <c r="J872" s="2" t="n">
-        <v>46265.4616653125</v>
+        <v>46266.75154699074</v>
       </c>
       <c r="K872" s="2" t="n">
         <v>46296</v>
       </c>
       <c r="L872" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M872" s="1" t="inlineStr">
         <is>
-          <t>Amanda Mesquita</t>
-        </is>
-      </c>
-      <c r="N872" s="2" t="n">
-        <v>46265.62414548611</v>
-      </c>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N872" s="1" t="n"/>
       <c r="O872" s="1" t="n"/>
-      <c r="P872" s="2" t="n">
-        <v>46276.71389502315</v>
-      </c>
-      <c r="Q872" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="R872" s="1" t="inlineStr">
-        <is>
-          <t>Em fila de atendimento</t>
-        </is>
-      </c>
+      <c r="P872" s="1" t="n"/>
+      <c r="Q872" s="1" t="inlineStr"/>
+      <c r="R872" s="1" t="inlineStr"/>
       <c r="S872" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T872" s="1" t="n"/>
@@ -66767,7 +66784,7 @@
     </row>
     <row r="873">
       <c r="A873" s="1" t="n">
-        <v>83367</v>
+        <v>83313</v>
       </c>
       <c r="B873" s="1" t="inlineStr">
         <is>
@@ -66786,15 +66803,15 @@
       </c>
       <c r="E873" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!Segue em anexo cadastro de produtos da empresa 5789 – ACE FRUIT para validação do CBS/IBS.</t>
+          <t xml:space="preserve">Prezados, bom dia.Segue e-mail enviado com a planilha de cadastro de produtos. Conforme falado com o gerente de contas Bruno, fica de acordo realizar a validação do cadastro de acordo com as informações enviadas ao cliente. Caso validação não seja realizada por completo iremos comunicar ao cliente. </t>
         </is>
       </c>
       <c r="F873" s="1" t="n">
-        <v>5789</v>
+        <v>6644</v>
       </c>
       <c r="G873" s="1" t="inlineStr">
         <is>
-          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
+          <t>MAPA DISTRIBUIDORA DE ALIMENTOS IMPORTACAO E EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="H873" s="1" t="inlineStr">
@@ -66808,32 +66825,26 @@
         </is>
       </c>
       <c r="J873" s="2" t="n">
-        <v>46266.64626565972</v>
+        <v>46266.41307797454</v>
       </c>
       <c r="K873" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="L873" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M873" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
-        </is>
-      </c>
-      <c r="N873" s="2" t="n">
-        <v>46269.66462141203</v>
-      </c>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N873" s="1" t="n"/>
       <c r="O873" s="1" t="n"/>
       <c r="P873" s="1" t="n"/>
       <c r="Q873" s="1" t="inlineStr"/>
-      <c r="R873" s="1" t="inlineStr">
-        <is>
-          <t>Em fila para atendimento</t>
-        </is>
-      </c>
+      <c r="R873" s="1" t="inlineStr"/>
       <c r="S873" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -66844,7 +66855,7 @@
     </row>
     <row r="874">
       <c r="A874" s="1" t="n">
-        <v>83429</v>
+        <v>83541</v>
       </c>
       <c r="B874" s="1" t="inlineStr">
         <is>
@@ -66863,15 +66874,15 @@
       </c>
       <c r="E874" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, boa tarde!Segue novamente planilha de IBS/CBS da empresa 3965 - TUTTI DELI, ela já foi enviada anteriormente o número do chamado antigo é 82784, porém ela foi retornada mesmo estando completa. Na planilha consta NCM, Descrição e EAN. </t>
+          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
         </is>
       </c>
       <c r="F874" s="1" t="n">
-        <v>3965</v>
+        <v>4411</v>
       </c>
       <c r="G874" s="1" t="inlineStr">
         <is>
-          <t>TUTTI QUITUTE PRODUTOS ALIMENTICIOS LTDA</t>
+          <t>JPS MATERIAIS DE CONSTRUÇÃO E DECORAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H874" s="1" t="inlineStr">
@@ -66885,14 +66896,14 @@
         </is>
       </c>
       <c r="J874" s="2" t="n">
-        <v>46266.75154699074</v>
+        <v>46268.43361015046</v>
       </c>
       <c r="K874" s="2" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L874" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M874" s="1" t="inlineStr">
@@ -66902,12 +66913,22 @@
       </c>
       <c r="N874" s="1" t="n"/>
       <c r="O874" s="1" t="n"/>
-      <c r="P874" s="1" t="n"/>
-      <c r="Q874" s="1" t="inlineStr"/>
-      <c r="R874" s="1" t="inlineStr"/>
+      <c r="P874" s="2" t="n">
+        <v>46273.43621866898</v>
+      </c>
+      <c r="Q874" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R874" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro analisado e enviado por email em 04/09</t>
+        </is>
+      </c>
       <c r="S874" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T874" s="1" t="n"/>
@@ -66915,7 +66936,7 @@
     </row>
     <row r="875">
       <c r="A875" s="1" t="n">
-        <v>83313</v>
+        <v>83542</v>
       </c>
       <c r="B875" s="1" t="inlineStr">
         <is>
@@ -66934,15 +66955,15 @@
       </c>
       <c r="E875" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, bom dia.Segue e-mail enviado com a planilha de cadastro de produtos. Conforme falado com o gerente de contas Bruno, fica de acordo realizar a validação do cadastro de acordo com as informações enviadas ao cliente. Caso validação não seja realizada por completo iremos comunicar ao cliente. </t>
+          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
         </is>
       </c>
       <c r="F875" s="1" t="n">
-        <v>6644</v>
+        <v>6412</v>
       </c>
       <c r="G875" s="1" t="inlineStr">
         <is>
-          <t>MAPA DISTRIBUIDORA DE ALIMENTOS IMPORTACAO E EXPORTACAO LTDA</t>
+          <t xml:space="preserve">SPJ MATERIAIS DE CONSTRUCAO LTDA </t>
         </is>
       </c>
       <c r="H875" s="1" t="inlineStr">
@@ -66956,29 +66977,39 @@
         </is>
       </c>
       <c r="J875" s="2" t="n">
-        <v>46266.41307797454</v>
+        <v>46268.43411693287</v>
       </c>
       <c r="K875" s="2" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L875" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M875" s="1" t="inlineStr">
         <is>
-          <t>Amanda Mesquita</t>
+          <t>Lohany Martins</t>
         </is>
       </c>
       <c r="N875" s="1" t="n"/>
       <c r="O875" s="1" t="n"/>
-      <c r="P875" s="1" t="n"/>
-      <c r="Q875" s="1" t="inlineStr"/>
-      <c r="R875" s="1" t="inlineStr"/>
+      <c r="P875" s="2" t="n">
+        <v>46273.43373032408</v>
+      </c>
+      <c r="Q875" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R875" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro analisado e enviado por email em 04/03</t>
+        </is>
+      </c>
       <c r="S875" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T875" s="1" t="n"/>
@@ -66986,7 +67017,7 @@
     </row>
     <row r="876">
       <c r="A876" s="1" t="n">
-        <v>83541</v>
+        <v>83562</v>
       </c>
       <c r="B876" s="1" t="inlineStr">
         <is>
@@ -67000,20 +67031,20 @@
       </c>
       <c r="D876" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E876" s="1" t="inlineStr">
         <is>
-          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
+          <t>6947 - F. MARQUES DE SA LTDA - PLANILHA DE INTENS Em anexo email enviado com a planilha.</t>
         </is>
       </c>
       <c r="F876" s="1" t="n">
-        <v>4411</v>
+        <v>6947</v>
       </c>
       <c r="G876" s="1" t="inlineStr">
         <is>
-          <t>JPS MATERIAIS DE CONSTRUÇÃO E DECORAÇÕES LTDA</t>
+          <t>F. MARQUES DE SA LTDA</t>
         </is>
       </c>
       <c r="H876" s="1" t="inlineStr">
@@ -67027,39 +67058,29 @@
         </is>
       </c>
       <c r="J876" s="2" t="n">
-        <v>46268.43361015046</v>
+        <v>46268.52269753473</v>
       </c>
       <c r="K876" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="L876" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M876" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N876" s="1" t="n"/>
       <c r="O876" s="1" t="n"/>
-      <c r="P876" s="2" t="n">
-        <v>46273.43621866898</v>
-      </c>
-      <c r="Q876" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="R876" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro analisado e enviado por email em 04/09</t>
-        </is>
-      </c>
+      <c r="P876" s="1" t="n"/>
+      <c r="Q876" s="1" t="inlineStr"/>
+      <c r="R876" s="1" t="inlineStr"/>
       <c r="S876" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T876" s="1" t="n"/>
@@ -67067,7 +67088,7 @@
     </row>
     <row r="877">
       <c r="A877" s="1" t="n">
-        <v>83542</v>
+        <v>83432</v>
       </c>
       <c r="B877" s="1" t="inlineStr">
         <is>
@@ -67081,20 +67102,20 @@
       </c>
       <c r="D877" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E877" s="1" t="inlineStr">
         <is>
-          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
+          <t>Revisão de cadastro de produtos da Ki-Preco</t>
         </is>
       </c>
       <c r="F877" s="1" t="n">
-        <v>6412</v>
+        <v>6442</v>
       </c>
       <c r="G877" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPJ MATERIAIS DE CONSTRUCAO LTDA </t>
+          <t>KI PRECO SERVICOS ADMINISTRATIVOS LTDA</t>
         </is>
       </c>
       <c r="H877" s="1" t="inlineStr">
@@ -67108,39 +67129,29 @@
         </is>
       </c>
       <c r="J877" s="2" t="n">
-        <v>46268.43411693287</v>
+        <v>46266.81141119213</v>
       </c>
       <c r="K877" s="2" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L877" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M877" s="1" t="inlineStr">
         <is>
-          <t>Lohany Martins</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N877" s="1" t="n"/>
       <c r="O877" s="1" t="n"/>
-      <c r="P877" s="2" t="n">
-        <v>46273.43373032408</v>
-      </c>
-      <c r="Q877" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="R877" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro analisado e enviado por email em 04/03</t>
-        </is>
-      </c>
+      <c r="P877" s="1" t="n"/>
+      <c r="Q877" s="1" t="inlineStr"/>
+      <c r="R877" s="1" t="inlineStr"/>
       <c r="S877" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T877" s="1" t="n"/>
@@ -67148,7 +67159,7 @@
     </row>
     <row r="878">
       <c r="A878" s="1" t="n">
-        <v>83562</v>
+        <v>83644</v>
       </c>
       <c r="B878" s="1" t="inlineStr">
         <is>
@@ -67167,15 +67178,15 @@
       </c>
       <c r="E878" s="1" t="inlineStr">
         <is>
-          <t>6947 - F. MARQUES DE SA LTDA - PLANILHA DE INTENS Em anexo email enviado com a planilha.</t>
+          <t>Prezadas, conforme solicitado pelo Nilton, segue:Abrir um chamado para esta empresa fazer a análise do cadastro de produtos dividido em 3 partes:1º - primeira parte analisar os produtos que estão com a exclusão a partir de primeiro de outubro fusão do ICMS – ST (que acho que não deve ter nenhum)2º - segunda parte fazer a classificação da alíquota teste do IBS e CBS3º - Classificação total das alíquotas atuais de ICMS PIS e COFINScadastro enviado no e-mail.</t>
         </is>
       </c>
       <c r="F878" s="1" t="n">
-        <v>6947</v>
+        <v>1603</v>
       </c>
       <c r="G878" s="1" t="inlineStr">
         <is>
-          <t>F. MARQUES DE SA LTDA</t>
+          <t>MERCADINHO KI PREÇO BAIXO LTDA</t>
         </is>
       </c>
       <c r="H878" s="1" t="inlineStr">
@@ -67189,10 +67200,10 @@
         </is>
       </c>
       <c r="J878" s="2" t="n">
-        <v>46268.52269753473</v>
+        <v>46273.47367033565</v>
       </c>
       <c r="K878" s="2" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="L878" s="1" t="inlineStr">
         <is>
@@ -67201,7 +67212,7 @@
       </c>
       <c r="M878" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N878" s="1" t="n"/>
@@ -67219,7 +67230,7 @@
     </row>
     <row r="879">
       <c r="A879" s="1" t="n">
-        <v>83432</v>
+        <v>83654</v>
       </c>
       <c r="B879" s="1" t="inlineStr">
         <is>
@@ -67233,20 +67244,20 @@
       </c>
       <c r="D879" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>RJ - GC ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E879" s="1" t="inlineStr">
         <is>
-          <t>Revisão de cadastro de produtos da Ki-Preco</t>
+          <t>Prezados, segue em anexo e-mail com planilha de cadastro de produtos da empresa.</t>
         </is>
       </c>
       <c r="F879" s="1" t="n">
-        <v>6442</v>
+        <v>5714</v>
       </c>
       <c r="G879" s="1" t="inlineStr">
         <is>
-          <t>KI PRECO SERVICOS ADMINISTRATIVOS LTDA</t>
+          <t>DIBRAMASUL MADEIRAS LTDA</t>
         </is>
       </c>
       <c r="H879" s="1" t="inlineStr">
@@ -67260,185 +67271,43 @@
         </is>
       </c>
       <c r="J879" s="2" t="n">
-        <v>46266.81141119213</v>
+        <v>46273.54331446759</v>
       </c>
       <c r="K879" s="2" t="n">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="L879" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M879" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Amanda Mesquita</t>
         </is>
       </c>
       <c r="N879" s="1" t="n"/>
       <c r="O879" s="1" t="n"/>
-      <c r="P879" s="1" t="n"/>
-      <c r="Q879" s="1" t="inlineStr"/>
-      <c r="R879" s="1" t="inlineStr"/>
+      <c r="P879" s="2" t="n">
+        <v>46276.69486894676</v>
+      </c>
+      <c r="Q879" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R879" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro analisado e devolvido por email em 10/09</t>
+        </is>
+      </c>
       <c r="S879" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T879" s="1" t="n"/>
       <c r="U879" s="1" t="inlineStr"/>
-    </row>
-    <row r="880">
-      <c r="A880" s="1" t="n">
-        <v>83644</v>
-      </c>
-      <c r="B880" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de Produtos</t>
-        </is>
-      </c>
-      <c r="C880" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de produtos</t>
-        </is>
-      </c>
-      <c r="D880" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E880" s="1" t="inlineStr">
-        <is>
-          <t>Prezadas, conforme solicitado pelo Nilton, segue:Abrir um chamado para esta empresa fazer a análise do cadastro de produtos dividido em 3 partes:1º - primeira parte analisar os produtos que estão com a exclusão a partir de primeiro de outubro fusão do ICMS – ST (que acho que não deve ter nenhum)2º - segunda parte fazer a classificação da alíquota teste do IBS e CBS3º - Classificação total das alíquotas atuais de ICMS PIS e COFINScadastro enviado no e-mail.</t>
-        </is>
-      </c>
-      <c r="F880" s="1" t="n">
-        <v>1603</v>
-      </c>
-      <c r="G880" s="1" t="inlineStr">
-        <is>
-          <t>MERCADINHO KI PREÇO BAIXO LTDA</t>
-        </is>
-      </c>
-      <c r="H880" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="I880" s="1" t="inlineStr">
-        <is>
-          <t>CADASTRO DE PRODUTOS</t>
-        </is>
-      </c>
-      <c r="J880" s="2" t="n">
-        <v>46273.47367033565</v>
-      </c>
-      <c r="K880" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L880" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M880" s="1" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N880" s="1" t="n"/>
-      <c r="O880" s="1" t="n"/>
-      <c r="P880" s="1" t="n"/>
-      <c r="Q880" s="1" t="inlineStr"/>
-      <c r="R880" s="1" t="inlineStr"/>
-      <c r="S880" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T880" s="1" t="n"/>
-      <c r="U880" s="1" t="inlineStr"/>
-    </row>
-    <row r="881">
-      <c r="A881" s="1" t="n">
-        <v>83654</v>
-      </c>
-      <c r="B881" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de Produtos</t>
-        </is>
-      </c>
-      <c r="C881" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de produtos</t>
-        </is>
-      </c>
-      <c r="D881" s="1" t="inlineStr">
-        <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E881" s="1" t="inlineStr">
-        <is>
-          <t>Prezados, segue em anexo e-mail com planilha de cadastro de produtos da empresa.</t>
-        </is>
-      </c>
-      <c r="F881" s="1" t="n">
-        <v>5714</v>
-      </c>
-      <c r="G881" s="1" t="inlineStr">
-        <is>
-          <t>DIBRAMASUL MADEIRAS LTDA</t>
-        </is>
-      </c>
-      <c r="H881" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="I881" s="1" t="inlineStr">
-        <is>
-          <t>CADASTRO DE PRODUTOS</t>
-        </is>
-      </c>
-      <c r="J881" s="2" t="n">
-        <v>46273.54331446759</v>
-      </c>
-      <c r="K881" s="2" t="n">
-        <v>46304</v>
-      </c>
-      <c r="L881" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M881" s="1" t="inlineStr">
-        <is>
-          <t>Amanda Mesquita</t>
-        </is>
-      </c>
-      <c r="N881" s="1" t="n"/>
-      <c r="O881" s="1" t="n"/>
-      <c r="P881" s="2" t="n">
-        <v>46276.69486894676</v>
-      </c>
-      <c r="Q881" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Bertunes</t>
-        </is>
-      </c>
-      <c r="R881" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro analisado e devolvido por email em 10/09</t>
-        </is>
-      </c>
-      <c r="S881" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T881" s="1" t="n"/>
-      <c r="U881" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-16 18:20
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -51865,7 +51865,7 @@
       </c>
       <c r="L678" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M678" s="1" t="inlineStr">
@@ -51873,11 +51873,17 @@
           <t>Yasmin Peixoto</t>
         </is>
       </c>
-      <c r="N678" s="1" t="n"/>
+      <c r="N678" s="2" t="n">
+        <v>46281.75651021991</v>
+      </c>
       <c r="O678" s="1" t="n"/>
       <c r="P678" s="1" t="n"/>
       <c r="Q678" s="1" t="inlineStr"/>
-      <c r="R678" s="1" t="inlineStr"/>
+      <c r="R678" s="1" t="inlineStr">
+        <is>
+          <t>Certidão/Levantamento solicitado, aguardando retorno.</t>
+        </is>
+      </c>
       <c r="S678" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52242,7 +52248,7 @@
       </c>
       <c r="L683" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M683" s="1" t="inlineStr">
@@ -52252,12 +52258,22 @@
       </c>
       <c r="N683" s="1" t="n"/>
       <c r="O683" s="1" t="n"/>
-      <c r="P683" s="1" t="n"/>
-      <c r="Q683" s="1" t="inlineStr"/>
-      <c r="R683" s="1" t="inlineStr"/>
+      <c r="P683" s="2" t="n">
+        <v>46281.76203364583</v>
+      </c>
+      <c r="Q683" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="R683" s="1" t="inlineStr">
+        <is>
+          <t>Empresa não possui inscrição municipal.</t>
+        </is>
+      </c>
       <c r="S683" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T683" s="1" t="n"/>
@@ -59473,7 +59489,7 @@
       </c>
       <c r="L776" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M776" s="1" t="inlineStr">
@@ -59483,12 +59499,27 @@
       </c>
       <c r="N776" s="1" t="n"/>
       <c r="O776" s="1" t="n"/>
-      <c r="P776" s="1" t="n"/>
-      <c r="Q776" s="1" t="inlineStr"/>
-      <c r="R776" s="1" t="inlineStr"/>
+      <c r="P776" s="2" t="n">
+        <v>46281.75655381945</v>
+      </c>
+      <c r="Q776" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="R776" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ricardo, boa tarde!
+Realizei as simulações considerando as opções atualmente disponíveis para adesão. Como a PGFN estabeleceu limites para os valores que podem ser incluídos em cada modalidade de transação, foi necessário realizar as simulações separadamente, de acordo com cada opção disponível.
+Encaminho as simulações em anexo para sua análise, contemplando os cenários com o número mínimo e máximo de parcelas permitido em cada modalidade.
+É importante destacar que o cliente já possui algumas transações em andamento. Entre elas, há uma transação referente aos débitos do Simples Nacional, atualmente parcelada em 145 parcelas. Essa condição, porém, não está mais disponível para novas adesões neste momento, uma vez que o limite atual para essa modalidade é de 60 parcelas.
+Dessa forma, as simulações anexas demonstram as condições que podem ser obtidas atualmente, permitindo uma comparação com as transações que o cliente já possui e a avaliação do cenário mais adequado.
+</t>
+        </is>
+      </c>
       <c r="S776" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T776" s="1" t="n"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-22 09:32
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U845" headerRowCount="1">
-  <autoFilter ref="A1:U845"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U842" headerRowCount="1">
+  <autoFilter ref="A1:U842"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U845"/>
+  <dimension ref="A1:U842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60278,7 +60278,7 @@
       </c>
       <c r="L782" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M782" s="1" t="inlineStr">
@@ -60288,12 +60288,23 @@
       </c>
       <c r="N782" s="1" t="n"/>
       <c r="O782" s="1" t="n"/>
-      <c r="P782" s="1" t="n"/>
-      <c r="Q782" s="1" t="inlineStr"/>
-      <c r="R782" s="1" t="inlineStr"/>
+      <c r="P782" s="2" t="n">
+        <v>46287.39302276621</v>
+      </c>
+      <c r="Q782" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia!
+Segue simulado e proposta. </t>
+        </is>
+      </c>
       <c r="S782" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T782" s="1" t="n"/>
@@ -61071,39 +61082,39 @@
     </row>
     <row r="793">
       <c r="A793" s="1" t="n">
-        <v>83897</v>
+        <v>83642</v>
       </c>
       <c r="B793" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Notificação</t>
         </is>
       </c>
       <c r="C793" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D793" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>MG EXPRESS - GC</t>
         </is>
       </c>
       <c r="E793" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t>Cliente recebeu notificação CRC, prazo de 15 dias de retorno.</t>
         </is>
       </c>
       <c r="F793" s="1" t="n">
-        <v>6973</v>
+        <v>6588</v>
       </c>
       <c r="G793" s="1" t="inlineStr">
         <is>
-          <t>SINDIFY TECNOLOGIA LTDA</t>
+          <t>ALM GESTAO TECH RETAIL LTDA</t>
         </is>
       </c>
       <c r="H793" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I793" s="1" t="inlineStr">
@@ -61112,10 +61123,10 @@
         </is>
       </c>
       <c r="J793" s="2" t="n">
-        <v>46279.39057037037</v>
+        <v>46273.44699390046</v>
       </c>
       <c r="K793" s="2" t="n">
-        <v>46281</v>
+        <v>46276</v>
       </c>
       <c r="L793" s="1" t="inlineStr">
         <is>
@@ -61124,7 +61135,7 @@
       </c>
       <c r="M793" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
+          <t>Romero Borges</t>
         </is>
       </c>
       <c r="N793" s="1" t="n"/>
@@ -61142,39 +61153,39 @@
     </row>
     <row r="794">
       <c r="A794" s="1" t="n">
-        <v>83642</v>
+        <v>84129</v>
       </c>
       <c r="B794" s="1" t="inlineStr">
         <is>
-          <t>Notificação</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C794" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D794" s="1" t="inlineStr">
         <is>
-          <t>MG EXPRESS - GC</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E794" s="1" t="inlineStr">
         <is>
-          <t>Cliente recebeu notificação CRC, prazo de 15 dias de retorno.</t>
+          <t>Por gentileza poderia me informar o login e a senha da prefeitura.</t>
         </is>
       </c>
       <c r="F794" s="1" t="n">
-        <v>6588</v>
+        <v>6608</v>
       </c>
       <c r="G794" s="1" t="inlineStr">
         <is>
-          <t>ALM GESTAO TECH RETAIL LTDA</t>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 4)</t>
         </is>
       </c>
       <c r="H794" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I794" s="1" t="inlineStr">
@@ -61183,10 +61194,10 @@
         </is>
       </c>
       <c r="J794" s="2" t="n">
-        <v>46273.44699390046</v>
+        <v>46282.74585570602</v>
       </c>
       <c r="K794" s="2" t="n">
-        <v>46276</v>
+        <v>46286</v>
       </c>
       <c r="L794" s="1" t="inlineStr">
         <is>
@@ -61195,7 +61206,7 @@
       </c>
       <c r="M794" s="1" t="inlineStr">
         <is>
-          <t>Romero Borges</t>
+          <t>Rafaella Macedo</t>
         </is>
       </c>
       <c r="N794" s="1" t="n"/>
@@ -61213,11 +61224,11 @@
     </row>
     <row r="795">
       <c r="A795" s="1" t="n">
-        <v>84129</v>
+        <v>82264</v>
       </c>
       <c r="B795" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C795" s="1" t="inlineStr">
@@ -61227,25 +61238,25 @@
       </c>
       <c r="D795" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E795" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza poderia me informar o login e a senha da prefeitura.</t>
+          <t>Por gentileza enviar a guia atualizada da TFEdas duas empresas do grupo BOMBEIROS 6621 E 6622</t>
         </is>
       </c>
       <c r="F795" s="1" t="n">
-        <v>6608</v>
+        <v>6621</v>
       </c>
       <c r="G795" s="1" t="inlineStr">
         <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 4)</t>
+          <t>BOMBEIROS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANÇA LTDA</t>
         </is>
       </c>
       <c r="H795" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I795" s="1" t="inlineStr">
@@ -61254,29 +61265,40 @@
         </is>
       </c>
       <c r="J795" s="2" t="n">
-        <v>46282.74585570602</v>
+        <v>46246.3872690162</v>
       </c>
       <c r="K795" s="2" t="n">
-        <v>46286</v>
+        <v>46248</v>
       </c>
       <c r="L795" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M795" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Macedo</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N795" s="1" t="n"/>
       <c r="O795" s="1" t="n"/>
-      <c r="P795" s="1" t="n"/>
-      <c r="Q795" s="1" t="inlineStr"/>
-      <c r="R795" s="1" t="inlineStr"/>
+      <c r="P795" s="2" t="n">
+        <v>46246.66841165509</v>
+      </c>
+      <c r="Q795" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde!
+Não há débitos em aberto, seguem certidões. </t>
+        </is>
+      </c>
       <c r="S795" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T795" s="1" t="n"/>
@@ -61284,39 +61306,39 @@
     </row>
     <row r="796">
       <c r="A796" s="1" t="n">
-        <v>82264</v>
+        <v>82915</v>
       </c>
       <c r="B796" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C796" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D796" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E796" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza enviar a guia atualizada da TFEdas duas empresas do grupo BOMBEIROS 6621 E 6622</t>
+          <t>Alteração contratual do CAPITAL SOCIAL, QSA, ADMINISTRADOR e ATIVIDADE/CNAE da empresa 6628-TSN TECHNICAL SERVICE NETWORK LTDAGrupo: GTG1- Alteração de Sócio:Saida da Sra. MARIA BARBOSA DOS SANTOS CLEMENTE, que sede e tranfere o total das cotas para o Sr. ALISSON BARBOSA DE SOUSA 2- Aumento do capital:será aumentado de 150.000, para 300.000, sendo a integralização de 50.000, através do registro de um carro, e o restante (100.000), a integralizar em 12 parcelas.3- Alteração de CNAEs, seram removidos  4 e temos e incluir 6, conforme abaixo:CNAEs RETIRAR: (OK)•	23.41-9-00 - Fabricação de produtos cerâmicos refratários •	61.10-8-01 - Serviços de telefonia fixa comutada - STFC •	61.10-8-03 - Serviços de comunicação multimídia - SCM•	62.02-3-00 - Desenvolvimento e licenciamento de programas de computador customizáveisINCLUIR: (OK)•	4686-9/02 — Comércio atacadista de embalagens;•	4789-0/99 — Comércio varejista de outros produtos não especificados anteriormente;•	4744-0/03 — Comércio varejista de materiais hidráulicos;•	4679-6/04 — Comércio atacadista especializado de materiais de construção não especificados anteriormente;•	4673-7/00 — Comércio atacadista de material elétrico.•	86.60-7-00 - Atividades de apoio à gestão de saúde</t>
         </is>
       </c>
       <c r="F796" s="1" t="n">
-        <v>6621</v>
+        <v>6628</v>
       </c>
       <c r="G796" s="1" t="inlineStr">
         <is>
-          <t>BOMBEIROS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANÇA LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="H796" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I796" s="1" t="inlineStr">
@@ -61325,119 +61347,120 @@
         </is>
       </c>
       <c r="J796" s="2" t="n">
-        <v>46246.3872690162</v>
+        <v>46258.70282021991</v>
       </c>
       <c r="K796" s="2" t="n">
-        <v>46248</v>
+        <v>46286</v>
       </c>
       <c r="L796" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M796" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
-      <c r="N796" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N796" s="2" t="n">
+        <v>46261.63173943287</v>
+      </c>
       <c r="O796" s="1" t="n"/>
-      <c r="P796" s="2" t="n">
-        <v>46246.66841165509</v>
-      </c>
-      <c r="Q796" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
+      <c r="P796" s="1" t="n"/>
+      <c r="Q796" s="1" t="inlineStr"/>
       <c r="R796" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Boa tarde!
-Não há débitos em aberto, seguem certidões. </t>
-        </is>
-      </c>
-      <c r="S796" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T796" s="1" t="n"/>
-      <c r="U796" s="1" t="inlineStr"/>
-    </row>
-    <row r="797">
-      <c r="A797" s="1" t="n">
-        <v>82915</v>
-      </c>
-      <c r="B797" s="1" t="inlineStr">
-        <is>
-          <t>Alteração Contratual</t>
-        </is>
-      </c>
-      <c r="C797" s="1" t="inlineStr">
-        <is>
-          <t>Sócios</t>
-        </is>
-      </c>
-      <c r="D797" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA MASTER</t>
-        </is>
-      </c>
-      <c r="E797" s="1" t="inlineStr">
-        <is>
-          <t>Alteração contratual do CAPITAL SOCIAL, QSA, ADMINISTRADOR e ATIVIDADE/CNAE da empresa 6628-TSN TECHNICAL SERVICE NETWORK LTDAGrupo: GTG1- Alteração de Sócio:Saida da Sra. MARIA BARBOSA DOS SANTOS CLEMENTE, que sede e tranfere o total das cotas para o Sr. ALISSON BARBOSA DE SOUSA 2- Aumento do capital:será aumentado de 150.000, para 300.000, sendo a integralização de 50.000, através do registro de um carro, e o restante (100.000), a integralizar em 12 parcelas.3- Alteração de CNAEs, seram removidos  4 e temos e incluir 6, conforme abaixo:CNAEs RETIRAR: (OK)•	23.41-9-00 - Fabricação de produtos cerâmicos refratários •	61.10-8-01 - Serviços de telefonia fixa comutada - STFC •	61.10-8-03 - Serviços de comunicação multimídia - SCM•	62.02-3-00 - Desenvolvimento e licenciamento de programas de computador customizáveisINCLUIR: (OK)•	4686-9/02 — Comércio atacadista de embalagens;•	4789-0/99 — Comércio varejista de outros produtos não especificados anteriormente;•	4744-0/03 — Comércio varejista de materiais hidráulicos;•	4679-6/04 — Comércio atacadista especializado de materiais de construção não especificados anteriormente;•	4673-7/00 — Comércio atacadista de material elétrico.•	86.60-7-00 - Atividades de apoio à gestão de saúde</t>
-        </is>
-      </c>
-      <c r="F797" s="1" t="n">
-        <v>6628</v>
-      </c>
-      <c r="G797" s="1" t="inlineStr">
-        <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
-        </is>
-      </c>
-      <c r="H797" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Ribeiro</t>
-        </is>
-      </c>
-      <c r="I797" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J797" s="2" t="n">
-        <v>46258.70282021991</v>
-      </c>
-      <c r="K797" s="2" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L797" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M797" s="1" t="inlineStr">
-        <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N797" s="2" t="n">
-        <v>46261.63173943287</v>
-      </c>
-      <c r="O797" s="1" t="n"/>
-      <c r="P797" s="1" t="n"/>
-      <c r="Q797" s="1" t="inlineStr"/>
-      <c r="R797" s="1" t="inlineStr">
         <is>
           <t>Prezados(as), boa tarde!
 Conforme solicitado, alteração contratual em andamento. 
 Atenciosamente,</t>
         </is>
       </c>
+      <c r="S796" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T796" s="1" t="n"/>
+      <c r="U796" s="1" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" s="1" t="n">
+        <v>84101</v>
+      </c>
+      <c r="B797" s="1" t="inlineStr">
+        <is>
+          <t>Parcelamento PGFN</t>
+        </is>
+      </c>
+      <c r="C797" s="1" t="inlineStr">
+        <is>
+          <t>Simples Nacional</t>
+        </is>
+      </c>
+      <c r="D797" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E797" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia! Por gentileza, poderiam emitir uma guia atualizada</t>
+        </is>
+      </c>
+      <c r="F797" s="1" t="n">
+        <v>6650</v>
+      </c>
+      <c r="G797" s="1" t="inlineStr">
+        <is>
+          <t>ACJ COMERCIO DE EMBALAGENS LTDA</t>
+        </is>
+      </c>
+      <c r="H797" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="I797" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J797" s="2" t="n">
+        <v>46282.47985864583</v>
+      </c>
+      <c r="K797" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L797" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M797" s="1" t="inlineStr">
+        <is>
+          <t>Sofia Souza</t>
+        </is>
+      </c>
+      <c r="N797" s="1" t="n"/>
+      <c r="O797" s="1" t="n"/>
+      <c r="P797" s="2" t="n">
+        <v>46283.70308052083</v>
+      </c>
+      <c r="Q797" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R797" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Qual parcela que voce deseja que seja emitida?
+Simples Nacional ou PGFN Simples Nacional?</t>
+        </is>
+      </c>
       <c r="S797" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T797" s="1" t="n"/>
@@ -61445,16 +61468,16 @@
     </row>
     <row r="798">
       <c r="A798" s="1" t="n">
-        <v>84101</v>
+        <v>81317</v>
       </c>
       <c r="B798" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento PGFN</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C798" s="1" t="inlineStr">
         <is>
-          <t>Simples Nacional</t>
+          <t xml:space="preserve">Inclusão de Ata </t>
         </is>
       </c>
       <c r="D798" s="1" t="inlineStr">
@@ -61464,20 +61487,20 @@
       </c>
       <c r="E798" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, poderiam emitir uma guia atualizada</t>
+          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
         </is>
       </c>
       <c r="F798" s="1" t="n">
-        <v>6650</v>
+        <v>6673</v>
       </c>
       <c r="G798" s="1" t="inlineStr">
         <is>
-          <t>ACJ COMERCIO DE EMBALAGENS LTDA</t>
+          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
         </is>
       </c>
       <c r="H798" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I798" s="1" t="inlineStr">
@@ -61486,10 +61509,10 @@
         </is>
       </c>
       <c r="J798" s="2" t="n">
-        <v>46282.47985864583</v>
+        <v>46225.61752997685</v>
       </c>
       <c r="K798" s="2" t="n">
-        <v>46286</v>
+        <v>46231</v>
       </c>
       <c r="L798" s="1" t="inlineStr">
         <is>
@@ -61498,24 +61521,22 @@
       </c>
       <c r="M798" s="1" t="inlineStr">
         <is>
-          <t>Sofia Souza</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="N798" s="1" t="n"/>
       <c r="O798" s="1" t="n"/>
       <c r="P798" s="2" t="n">
-        <v>46283.70308052083</v>
+        <v>46230.66237318287</v>
       </c>
       <c r="Q798" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="R798" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!
-Qual parcela que voce deseja que seja emitida?
-Simples Nacional ou PGFN Simples Nacional?</t>
+          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
         </is>
       </c>
       <c r="S798" s="1" t="inlineStr">
@@ -61528,7 +61549,7 @@
     </row>
     <row r="799">
       <c r="A799" s="1" t="n">
-        <v>81317</v>
+        <v>81316</v>
       </c>
       <c r="B799" s="1" t="inlineStr">
         <is>
@@ -61547,15 +61568,15 @@
       </c>
       <c r="E799" s="1" t="inlineStr">
         <is>
-          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
+          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
         </is>
       </c>
       <c r="F799" s="1" t="n">
-        <v>6673</v>
+        <v>6674</v>
       </c>
       <c r="G799" s="1" t="inlineStr">
         <is>
-          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
+          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
         </is>
       </c>
       <c r="H799" s="1" t="inlineStr">
@@ -61569,7 +61590,7 @@
         </is>
       </c>
       <c r="J799" s="2" t="n">
-        <v>46225.61752997685</v>
+        <v>46225.61705821759</v>
       </c>
       <c r="K799" s="2" t="n">
         <v>46231</v>
@@ -61587,7 +61608,7 @@
       <c r="N799" s="1" t="n"/>
       <c r="O799" s="1" t="n"/>
       <c r="P799" s="2" t="n">
-        <v>46230.66237318287</v>
+        <v>46230.66303518519</v>
       </c>
       <c r="Q799" s="1" t="inlineStr">
         <is>
@@ -61596,7 +61617,7 @@
       </c>
       <c r="R799" s="1" t="inlineStr">
         <is>
-          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
+          <t>Enviar a planilha devidamente preenchida e completa.</t>
         </is>
       </c>
       <c r="S799" s="1" t="inlineStr">
@@ -61609,39 +61630,39 @@
     </row>
     <row r="800">
       <c r="A800" s="1" t="n">
-        <v>81316</v>
+        <v>81987</v>
       </c>
       <c r="B800" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inclusão de Ata </t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D800" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E800" s="1" t="inlineStr">
         <is>
-          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
+          <t>6977 - PROTECTION SHIELD - MUDANÇAS NO CONTRATO SOCIALO Cliente precisa mudar o CNAI e incluir um sócio, poderia nos informar qual o honorário e quais documento você precisa?Desejo do cliente é fazer a transferência dos funcionário que estão hoje na 6976, para 6977, para isto é necessário haver a equiparação de atividades para não ter problemas Sindicais, então será necessita mudanças no CNAE, e para haver formação de grupo econômico a sócia deseja ter 1% de participação na 6977, hoje ela  da sociedade apenas como tutora do socio de menor, e como administradora.  Mais informações com o REYNALDO.Att.Vander</t>
         </is>
       </c>
       <c r="F800" s="1" t="n">
-        <v>6674</v>
+        <v>6977</v>
       </c>
       <c r="G800" s="1" t="inlineStr">
         <is>
-          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
+          <t>PROTECTION SHIELD LTDA</t>
         </is>
       </c>
       <c r="H800" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I800" s="1" t="inlineStr">
@@ -61650,39 +61671,35 @@
         </is>
       </c>
       <c r="J800" s="2" t="n">
-        <v>46225.61705821759</v>
+        <v>46240.55237392361</v>
       </c>
       <c r="K800" s="2" t="n">
-        <v>46231</v>
+        <v>46241</v>
       </c>
       <c r="L800" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M800" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
-        </is>
-      </c>
-      <c r="N800" s="1" t="n"/>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N800" s="2" t="n">
+        <v>46268.68733116899</v>
+      </c>
       <c r="O800" s="1" t="n"/>
-      <c r="P800" s="2" t="n">
-        <v>46230.66303518519</v>
-      </c>
-      <c r="Q800" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="P800" s="1" t="n"/>
+      <c r="Q800" s="1" t="inlineStr"/>
       <c r="R800" s="1" t="inlineStr">
         <is>
-          <t>Enviar a planilha devidamente preenchida e completa.</t>
+          <t>Favor, informar o que vai ser alterado de fato.</t>
         </is>
       </c>
       <c r="S800" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T800" s="1" t="n"/>
@@ -61690,7 +61707,7 @@
     </row>
     <row r="801">
       <c r="A801" s="1" t="n">
-        <v>81987</v>
+        <v>82091</v>
       </c>
       <c r="B801" s="1" t="inlineStr">
         <is>
@@ -61699,17 +61716,17 @@
       </c>
       <c r="C801" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D801" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E801" s="1" t="inlineStr">
         <is>
-          <t>6977 - PROTECTION SHIELD - MUDANÇAS NO CONTRATO SOCIALO Cliente precisa mudar o CNAI e incluir um sócio, poderia nos informar qual o honorário e quais documento você precisa?Desejo do cliente é fazer a transferência dos funcionário que estão hoje na 6976, para 6977, para isto é necessário haver a equiparação de atividades para não ter problemas Sindicais, então será necessita mudanças no CNAE, e para haver formação de grupo econômico a sócia deseja ter 1% de participação na 6977, hoje ela  da sociedade apenas como tutora do socio de menor, e como administradora.  Mais informações com o REYNALDO.Att.Vander</t>
+          <t>ALTERAÇÃO CONTRATUAL NA EMPRESA 6977-PROTECTION SHIELD LTDAGRUPO: FILM FACILALTERAÇÃO DE ATIVIDADE E QSAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$1.500,00EMPRESA DE ESTRATEGIA PARA FUNCIONARIOS, APÓS A TRANSFERRENCIA DOS FUNCIONÁRIOS, VOLTAR QUADRO SOCIETARIO ANTIGO</t>
         </is>
       </c>
       <c r="F801" s="1" t="n">
@@ -61731,10 +61748,10 @@
         </is>
       </c>
       <c r="J801" s="2" t="n">
-        <v>46240.55237392361</v>
+        <v>46241.64981377315</v>
       </c>
       <c r="K801" s="2" t="n">
-        <v>46241</v>
+        <v>46269</v>
       </c>
       <c r="L801" s="1" t="inlineStr">
         <is>
@@ -61743,18 +61760,18 @@
       </c>
       <c r="M801" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N801" s="2" t="n">
-        <v>46268.68733116899</v>
+        <v>46268.68579398148</v>
       </c>
       <c r="O801" s="1" t="n"/>
       <c r="P801" s="1" t="n"/>
       <c r="Q801" s="1" t="inlineStr"/>
       <c r="R801" s="1" t="inlineStr">
         <is>
-          <t>Favor, informar o que vai ser alterado de fato.</t>
+          <t>Raisa, a empresa  6977 já possui o quadro de sócios exatamente como consta na planilha, não tem o que ser alterado.</t>
         </is>
       </c>
       <c r="S801" s="1" t="inlineStr">
@@ -61767,26 +61784,26 @@
     </row>
     <row r="802">
       <c r="A802" s="1" t="n">
-        <v>82091</v>
+        <v>83899</v>
       </c>
       <c r="B802" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C802" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>Receita Federal</t>
         </is>
       </c>
       <c r="D802" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E802" s="1" t="inlineStr">
         <is>
-          <t>ALTERAÇÃO CONTRATUAL NA EMPRESA 6977-PROTECTION SHIELD LTDAGRUPO: FILM FACILALTERAÇÃO DE ATIVIDADE E QSAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$1.500,00EMPRESA DE ESTRATEGIA PARA FUNCIONARIOS, APÓS A TRANSFERRENCIA DOS FUNCIONÁRIOS, VOLTAR QUADRO SOCIETARIO ANTIGO</t>
+          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
         </is>
       </c>
       <c r="F802" s="1" t="n">
@@ -61799,7 +61816,7 @@
       </c>
       <c r="H802" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I802" s="1" t="inlineStr">
@@ -61808,32 +61825,26 @@
         </is>
       </c>
       <c r="J802" s="2" t="n">
-        <v>46241.64981377315</v>
+        <v>46279.39114621528</v>
       </c>
       <c r="K802" s="2" t="n">
-        <v>46269</v>
+        <v>46281</v>
       </c>
       <c r="L802" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M802" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N802" s="2" t="n">
-        <v>46268.68579398148</v>
-      </c>
+          <t>Ney Barbosa</t>
+        </is>
+      </c>
+      <c r="N802" s="1" t="n"/>
       <c r="O802" s="1" t="n"/>
       <c r="P802" s="1" t="n"/>
       <c r="Q802" s="1" t="inlineStr"/>
-      <c r="R802" s="1" t="inlineStr">
-        <is>
-          <t>Raisa, a empresa  6977 já possui o quadro de sócios exatamente como consta na planilha, não tem o que ser alterado.</t>
-        </is>
-      </c>
+      <c r="R802" s="1" t="inlineStr"/>
       <c r="S802" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -61844,39 +61855,39 @@
     </row>
     <row r="803">
       <c r="A803" s="1" t="n">
-        <v>83899</v>
+        <v>81753</v>
       </c>
       <c r="B803" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C803" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Sociedade - Comércio</t>
         </is>
       </c>
       <c r="D803" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E803" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t>ABERTURA DE EMPRESA - 6981-LUIZ GOMES DA SILVA - O GOIANOGRUPO: SUPERMERCADO AVENIDATRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIO FINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00EMPRESA DE ESTRATÉGIA, APÓS CONSTITUIDA MIGRAR OS FUNCIONARIOS. APÓS TERMINO DA MIGRAÇÃO ALTERAR ATIVIDADE E QUADRO SOCIETÁRIO.</t>
         </is>
       </c>
       <c r="F803" s="1" t="n">
-        <v>6977</v>
+        <v>6981</v>
       </c>
       <c r="G803" s="1" t="inlineStr">
         <is>
-          <t>PROTECTION SHIELD LTDA</t>
+          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
         </is>
       </c>
       <c r="H803" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I803" s="1" t="inlineStr">
@@ -61885,26 +61896,34 @@
         </is>
       </c>
       <c r="J803" s="2" t="n">
-        <v>46279.39114621528</v>
+        <v>46237.51070853009</v>
       </c>
       <c r="K803" s="2" t="n">
-        <v>46281</v>
+        <v>46265</v>
       </c>
       <c r="L803" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M803" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
-        </is>
-      </c>
-      <c r="N803" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N803" s="2" t="n">
+        <v>46246.66714818287</v>
+      </c>
       <c r="O803" s="1" t="n"/>
       <c r="P803" s="1" t="n"/>
       <c r="Q803" s="1" t="inlineStr"/>
-      <c r="R803" s="1" t="inlineStr"/>
+      <c r="R803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Processo de abertura em andamento. 
+Atenciosamente, </t>
+        </is>
+      </c>
       <c r="S803" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -61915,39 +61934,39 @@
     </row>
     <row r="804">
       <c r="A804" s="1" t="n">
-        <v>81753</v>
+        <v>83634</v>
       </c>
       <c r="B804" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C804" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D804" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E804" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA - 6981-LUIZ GOMES DA SILVA - O GOIANOGRUPO: SUPERMERCADO AVENIDATRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIO FINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00EMPRESA DE ESTRATÉGIA, APÓS CONSTITUIDA MIGRAR OS FUNCIONARIOS. APÓS TERMINO DA MIGRAÇÃO ALTERAR ATIVIDADE E QUADRO SOCIETÁRIO.</t>
+          <t>6984 – SUPERMERCADOS BANDEIRA LTDA - senha DA PREFEITURA DE ITAPECERICA DA SERRA - PARA DECLARAR ISS NA PREFEITURA</t>
         </is>
       </c>
       <c r="F804" s="1" t="n">
-        <v>6981</v>
+        <v>6984</v>
       </c>
       <c r="G804" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
         </is>
       </c>
       <c r="H804" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I804" s="1" t="inlineStr">
@@ -61956,10 +61975,10 @@
         </is>
       </c>
       <c r="J804" s="2" t="n">
-        <v>46237.51070853009</v>
+        <v>46273.39513472222</v>
       </c>
       <c r="K804" s="2" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="L804" s="1" t="inlineStr">
         <is>
@@ -61968,20 +61987,18 @@
       </c>
       <c r="M804" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Alaine Neres</t>
         </is>
       </c>
       <c r="N804" s="2" t="n">
-        <v>46246.66714818287</v>
+        <v>46274.49502619213</v>
       </c>
       <c r="O804" s="1" t="n"/>
       <c r="P804" s="1" t="n"/>
       <c r="Q804" s="1" t="inlineStr"/>
       <c r="R804" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Processo de abertura em andamento. 
-Atenciosamente, </t>
+          <t>Cobramos novamente o antigo contador</t>
         </is>
       </c>
       <c r="S804" s="1" t="inlineStr">
@@ -61994,39 +62011,39 @@
     </row>
     <row r="805">
       <c r="A805" s="1" t="n">
-        <v>83634</v>
+        <v>81933</v>
       </c>
       <c r="B805" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C805" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D805" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E805" s="1" t="inlineStr">
         <is>
-          <t>6984 – SUPERMERCADOS BANDEIRA LTDA - senha DA PREFEITURA DE ITAPECERICA DA SERRA - PARA DECLARAR ISS NA PREFEITURA</t>
+          <t>Por gentileza, providenciar:6990 - RC MATERIAIS ELETRICOS E HIDRAULICOS (MATRIZ) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL6991 - RC MATERIAIS ELETRICOS E HIDRAULICOS (FILIAL 1) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL</t>
         </is>
       </c>
       <c r="F805" s="1" t="n">
-        <v>6984</v>
+        <v>6990</v>
       </c>
       <c r="G805" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
+          <t>AMANCIO S ELETRICA, HIDRAULICA E CONSTRUCAO EM GERAL LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H805" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I805" s="1" t="inlineStr">
@@ -62035,35 +62052,39 @@
         </is>
       </c>
       <c r="J805" s="2" t="n">
-        <v>46273.39513472222</v>
+        <v>46239.72520292824</v>
       </c>
       <c r="K805" s="2" t="n">
-        <v>46275</v>
+        <v>46241</v>
       </c>
       <c r="L805" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M805" s="1" t="inlineStr">
         <is>
-          <t>Alaine Neres</t>
-        </is>
-      </c>
-      <c r="N805" s="2" t="n">
-        <v>46274.49502619213</v>
-      </c>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N805" s="1" t="n"/>
       <c r="O805" s="1" t="n"/>
-      <c r="P805" s="1" t="n"/>
-      <c r="Q805" s="1" t="inlineStr"/>
+      <c r="P805" s="2" t="n">
+        <v>46241.65195802083</v>
+      </c>
+      <c r="Q805" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="R805" s="1" t="inlineStr">
         <is>
-          <t>Cobramos novamente o antigo contador</t>
+          <t>Abrir um chamado por empresa, por gentileza.</t>
         </is>
       </c>
       <c r="S805" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T805" s="1" t="n"/>
@@ -62071,39 +62092,39 @@
     </row>
     <row r="806">
       <c r="A806" s="1" t="n">
-        <v>81933</v>
+        <v>81780</v>
       </c>
       <c r="B806" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C806" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Objeto Social</t>
         </is>
       </c>
       <c r="D806" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E806" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar:6990 - RC MATERIAIS ELETRICOS E HIDRAULICOS (MATRIZ) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL6991 - RC MATERIAIS ELETRICOS E HIDRAULICOS (FILIAL 1) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL</t>
+          <t>ALTERAÇÃO CONTRATUAL DA EMPRESA: 6993-GOMES SERVIÇOS - LTDAGRUPO: CRISTO REIALTERAÇÃO DE QSA E OBJETO SOCIALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00MESMA ATIVIDADE E SÓCIOS DO SUP. AVENIDA, APÓS ALTERAÇÃO MIGRAR FUNCIONÁRIOS PARA NOVA EMPRESA ALTERAR QSA E OBJETO SOCIAL.</t>
         </is>
       </c>
       <c r="F806" s="1" t="n">
-        <v>6990</v>
+        <v>6993</v>
       </c>
       <c r="G806" s="1" t="inlineStr">
         <is>
-          <t>AMANCIO S ELETRICA, HIDRAULICA E CONSTRUCAO EM GERAL LTDA (MATRIZ)</t>
+          <t>GOMES SERVIÇOS - LTDA</t>
         </is>
       </c>
       <c r="H806" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I806" s="1" t="inlineStr">
@@ -62112,39 +62133,37 @@
         </is>
       </c>
       <c r="J806" s="2" t="n">
-        <v>46239.72520292824</v>
+        <v>46237.62372283565</v>
       </c>
       <c r="K806" s="2" t="n">
-        <v>46241</v>
+        <v>46265</v>
       </c>
       <c r="L806" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M806" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N806" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N806" s="2" t="n">
+        <v>46246.66900671296</v>
+      </c>
       <c r="O806" s="1" t="n"/>
-      <c r="P806" s="2" t="n">
-        <v>46241.65195802083</v>
-      </c>
-      <c r="Q806" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+      <c r="P806" s="1" t="n"/>
+      <c r="Q806" s="1" t="inlineStr"/>
       <c r="R806" s="1" t="inlineStr">
         <is>
-          <t>Abrir um chamado por empresa, por gentileza.</t>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Alteração contratual em andamento. 
+Atenciosamente, </t>
         </is>
       </c>
       <c r="S806" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T806" s="1" t="n"/>
@@ -62152,34 +62171,34 @@
     </row>
     <row r="807">
       <c r="A807" s="1" t="n">
-        <v>81780</v>
+        <v>83921</v>
       </c>
       <c r="B807" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C807" s="1" t="inlineStr">
         <is>
-          <t>Objeto Social</t>
+          <t>Receita Federal</t>
         </is>
       </c>
       <c r="D807" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E807" s="1" t="inlineStr">
         <is>
-          <t>ALTERAÇÃO CONTRATUAL DA EMPRESA: 6993-GOMES SERVIÇOS - LTDAGRUPO: CRISTO REIALTERAÇÃO DE QSA E OBJETO SOCIALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00MESMA ATIVIDADE E SÓCIOS DO SUP. AVENIDA, APÓS ALTERAÇÃO MIGRAR FUNCIONÁRIOS PARA NOVA EMPRESA ALTERAR QSA E OBJETO SOCIAL.</t>
+          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
         </is>
       </c>
       <c r="F807" s="1" t="n">
-        <v>6993</v>
+        <v>6999</v>
       </c>
       <c r="G807" s="1" t="inlineStr">
         <is>
-          <t>GOMES SERVIÇOS - LTDA</t>
+          <t>VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="H807" s="1" t="inlineStr">
@@ -62193,34 +62212,26 @@
         </is>
       </c>
       <c r="J807" s="2" t="n">
-        <v>46237.62372283565</v>
+        <v>46279.39769957176</v>
       </c>
       <c r="K807" s="2" t="n">
-        <v>46265</v>
+        <v>46281</v>
       </c>
       <c r="L807" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M807" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N807" s="2" t="n">
-        <v>46246.66900671296</v>
-      </c>
+          <t>Ney Barbosa</t>
+        </is>
+      </c>
+      <c r="N807" s="1" t="n"/>
       <c r="O807" s="1" t="n"/>
       <c r="P807" s="1" t="n"/>
       <c r="Q807" s="1" t="inlineStr"/>
-      <c r="R807" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Alteração contratual em andamento. 
-Atenciosamente, </t>
-        </is>
-      </c>
+      <c r="R807" s="1" t="inlineStr"/>
       <c r="S807" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -62231,7 +62242,7 @@
     </row>
     <row r="808">
       <c r="A808" s="1" t="n">
-        <v>83921</v>
+        <v>83904</v>
       </c>
       <c r="B808" s="1" t="inlineStr">
         <is>
@@ -62254,16 +62265,16 @@
         </is>
       </c>
       <c r="F808" s="1" t="n">
-        <v>6999</v>
+        <v>7005</v>
       </c>
       <c r="G808" s="1" t="inlineStr">
         <is>
-          <t>VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H808" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I808" s="1" t="inlineStr">
@@ -62272,7 +62283,7 @@
         </is>
       </c>
       <c r="J808" s="2" t="n">
-        <v>46279.39769957176</v>
+        <v>46279.39261207176</v>
       </c>
       <c r="K808" s="2" t="n">
         <v>46281</v>
@@ -62302,7 +62313,7 @@
     </row>
     <row r="809">
       <c r="A809" s="1" t="n">
-        <v>83904</v>
+        <v>83905</v>
       </c>
       <c r="B809" s="1" t="inlineStr">
         <is>
@@ -62325,11 +62336,11 @@
         </is>
       </c>
       <c r="F809" s="1" t="n">
-        <v>7005</v>
+        <v>7006</v>
       </c>
       <c r="G809" s="1" t="inlineStr">
         <is>
-          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H809" s="1" t="inlineStr">
@@ -62343,7 +62354,7 @@
         </is>
       </c>
       <c r="J809" s="2" t="n">
-        <v>46279.39261207176</v>
+        <v>46279.39292399306</v>
       </c>
       <c r="K809" s="2" t="n">
         <v>46281</v>
@@ -62373,39 +62384,39 @@
     </row>
     <row r="810">
       <c r="A810" s="1" t="n">
-        <v>83905</v>
+        <v>83261</v>
       </c>
       <c r="B810" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C810" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D810" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E810" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t>Alteração contratual do QSA da empresa: 7046-RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDAGrupo: RamiroProposta já negociada no valor de R$1.800,00Retirar os dois sócios (João e Lucas) e deixar 100% do QSA com o Ramiro. Colocar atividade no Simples impeditiva, para que no mês de outubro essa empresa entre no Lucro Real</t>
         </is>
       </c>
       <c r="F810" s="1" t="n">
-        <v>7006</v>
+        <v>7046</v>
       </c>
       <c r="G810" s="1" t="inlineStr">
         <is>
-          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+          <t>RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDA</t>
         </is>
       </c>
       <c r="H810" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I810" s="1" t="inlineStr">
@@ -62414,26 +62425,34 @@
         </is>
       </c>
       <c r="J810" s="2" t="n">
-        <v>46279.39292399306</v>
+        <v>46265.45567503473</v>
       </c>
       <c r="K810" s="2" t="n">
-        <v>46281</v>
+        <v>46293</v>
       </c>
       <c r="L810" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M810" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
-        </is>
-      </c>
-      <c r="N810" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N810" s="2" t="n">
+        <v>46266.72388877315</v>
+      </c>
       <c r="O810" s="1" t="n"/>
       <c r="P810" s="1" t="n"/>
       <c r="Q810" s="1" t="inlineStr"/>
-      <c r="R810" s="1" t="inlineStr"/>
+      <c r="R810" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.
+Preparando a minuta.
+Atenciosamente,</t>
+        </is>
+      </c>
       <c r="S810" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -62444,34 +62463,34 @@
     </row>
     <row r="811">
       <c r="A811" s="1" t="n">
-        <v>83907</v>
+        <v>84107</v>
       </c>
       <c r="B811" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C811" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D811" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E811" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t xml:space="preserve">boa tarde!!Por gentileza, fazer ALVARÁ de funcionamento da loja. </t>
         </is>
       </c>
       <c r="F811" s="1" t="n">
-        <v>7041</v>
+        <v>7051</v>
       </c>
       <c r="G811" s="1" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN SERVICOS PROMOCIONAIS LTDA</t>
+          <t>TODOS ADMINISTRADORA DE CARTAO DE DESCONTOS BOTUCATU LTDA</t>
         </is>
       </c>
       <c r="H811" s="1" t="inlineStr">
@@ -62485,10 +62504,10 @@
         </is>
       </c>
       <c r="J811" s="2" t="n">
-        <v>46279.39348993055</v>
+        <v>46282.58430902778</v>
       </c>
       <c r="K811" s="2" t="n">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="L811" s="1" t="inlineStr">
         <is>
@@ -62497,7 +62516,7 @@
       </c>
       <c r="M811" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N811" s="1" t="n"/>
@@ -62515,39 +62534,39 @@
     </row>
     <row r="812">
       <c r="A812" s="1" t="n">
-        <v>83261</v>
+        <v>83908</v>
       </c>
       <c r="B812" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C812" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>Receita Federal</t>
         </is>
       </c>
       <c r="D812" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E812" s="1" t="inlineStr">
         <is>
-          <t>Alteração contratual do QSA da empresa: 7046-RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDAGrupo: RamiroProposta já negociada no valor de R$1.800,00Retirar os dois sócios (João e Lucas) e deixar 100% do QSA com o Ramiro. Colocar atividade no Simples impeditiva, para que no mês de outubro essa empresa entre no Lucro Real</t>
+          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
         </is>
       </c>
       <c r="F812" s="1" t="n">
-        <v>7046</v>
+        <v>7052</v>
       </c>
       <c r="G812" s="1" t="inlineStr">
         <is>
-          <t>RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDA</t>
+          <t>EMBRASIL COMERCIO DE AUTO PECAS LTDA</t>
         </is>
       </c>
       <c r="H812" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I812" s="1" t="inlineStr">
@@ -62556,34 +62575,26 @@
         </is>
       </c>
       <c r="J812" s="2" t="n">
-        <v>46265.45567503473</v>
+        <v>46279.3937971875</v>
       </c>
       <c r="K812" s="2" t="n">
-        <v>46293</v>
+        <v>46281</v>
       </c>
       <c r="L812" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M812" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N812" s="2" t="n">
-        <v>46266.72388877315</v>
-      </c>
+          <t>Ney Barbosa</t>
+        </is>
+      </c>
+      <c r="N812" s="1" t="n"/>
       <c r="O812" s="1" t="n"/>
       <c r="P812" s="1" t="n"/>
       <c r="Q812" s="1" t="inlineStr"/>
-      <c r="R812" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.
-Preparando a minuta.
-Atenciosamente,</t>
-        </is>
-      </c>
+      <c r="R812" s="1" t="inlineStr"/>
       <c r="S812" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -62594,39 +62605,39 @@
     </row>
     <row r="813">
       <c r="A813" s="1" t="n">
-        <v>84107</v>
+        <v>83909</v>
       </c>
       <c r="B813" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C813" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Receita Federal</t>
         </is>
       </c>
       <c r="D813" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E813" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">boa tarde!!Por gentileza, fazer ALVARÁ de funcionamento da loja. </t>
+          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
         </is>
       </c>
       <c r="F813" s="1" t="n">
-        <v>7051</v>
+        <v>7053</v>
       </c>
       <c r="G813" s="1" t="inlineStr">
         <is>
-          <t>TODOS ADMINISTRADORA DE CARTAO DE DESCONTOS BOTUCATU LTDA</t>
+          <t>BIANCA EMBREAGENS LTDA</t>
         </is>
       </c>
       <c r="H813" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I813" s="1" t="inlineStr">
@@ -62635,10 +62646,10 @@
         </is>
       </c>
       <c r="J813" s="2" t="n">
-        <v>46282.58430902778</v>
+        <v>46279.39412114584</v>
       </c>
       <c r="K813" s="2" t="n">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="L813" s="1" t="inlineStr">
         <is>
@@ -62647,7 +62658,7 @@
       </c>
       <c r="M813" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Ney Barbosa</t>
         </is>
       </c>
       <c r="N813" s="1" t="n"/>
@@ -62665,7 +62676,7 @@
     </row>
     <row r="814">
       <c r="A814" s="1" t="n">
-        <v>83908</v>
+        <v>83910</v>
       </c>
       <c r="B814" s="1" t="inlineStr">
         <is>
@@ -62688,11 +62699,11 @@
         </is>
       </c>
       <c r="F814" s="1" t="n">
-        <v>7052</v>
+        <v>7054</v>
       </c>
       <c r="G814" s="1" t="inlineStr">
         <is>
-          <t>EMBRASIL COMERCIO DE AUTO PECAS LTDA</t>
+          <t>KADOSH DISTRIBUIDOR COMERCIO E SERVICO DIGITAL LTDA</t>
         </is>
       </c>
       <c r="H814" s="1" t="inlineStr">
@@ -62706,7 +62717,7 @@
         </is>
       </c>
       <c r="J814" s="2" t="n">
-        <v>46279.3937971875</v>
+        <v>46279.39450123843</v>
       </c>
       <c r="K814" s="2" t="n">
         <v>46281</v>
@@ -62736,7 +62747,7 @@
     </row>
     <row r="815">
       <c r="A815" s="1" t="n">
-        <v>83909</v>
+        <v>83911</v>
       </c>
       <c r="B815" s="1" t="inlineStr">
         <is>
@@ -62759,11 +62770,11 @@
         </is>
       </c>
       <c r="F815" s="1" t="n">
-        <v>7053</v>
+        <v>7055</v>
       </c>
       <c r="G815" s="1" t="inlineStr">
         <is>
-          <t>BIANCA EMBREAGENS LTDA</t>
+          <t>YURI CESTARI DA SILVA EMBREAGENS OSASCO</t>
         </is>
       </c>
       <c r="H815" s="1" t="inlineStr">
@@ -62777,7 +62788,7 @@
         </is>
       </c>
       <c r="J815" s="2" t="n">
-        <v>46279.39412114584</v>
+        <v>46279.39479143519</v>
       </c>
       <c r="K815" s="2" t="n">
         <v>46281</v>
@@ -62807,7 +62818,7 @@
     </row>
     <row r="816">
       <c r="A816" s="1" t="n">
-        <v>83910</v>
+        <v>83912</v>
       </c>
       <c r="B816" s="1" t="inlineStr">
         <is>
@@ -62830,11 +62841,11 @@
         </is>
       </c>
       <c r="F816" s="1" t="n">
-        <v>7054</v>
+        <v>7056</v>
       </c>
       <c r="G816" s="1" t="inlineStr">
         <is>
-          <t>KADOSH DISTRIBUIDOR COMERCIO E SERVICO DIGITAL LTDA</t>
+          <t>AUTO CENTER EMBRASIL LTDA</t>
         </is>
       </c>
       <c r="H816" s="1" t="inlineStr">
@@ -62848,7 +62859,7 @@
         </is>
       </c>
       <c r="J816" s="2" t="n">
-        <v>46279.39450123843</v>
+        <v>46279.39518283565</v>
       </c>
       <c r="K816" s="2" t="n">
         <v>46281</v>
@@ -62878,7 +62889,7 @@
     </row>
     <row r="817">
       <c r="A817" s="1" t="n">
-        <v>83911</v>
+        <v>83913</v>
       </c>
       <c r="B817" s="1" t="inlineStr">
         <is>
@@ -62901,11 +62912,11 @@
         </is>
       </c>
       <c r="F817" s="1" t="n">
-        <v>7055</v>
+        <v>7057</v>
       </c>
       <c r="G817" s="1" t="inlineStr">
         <is>
-          <t>YURI CESTARI DA SILVA EMBREAGENS OSASCO</t>
+          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H817" s="1" t="inlineStr">
@@ -62919,7 +62930,7 @@
         </is>
       </c>
       <c r="J817" s="2" t="n">
-        <v>46279.39479143519</v>
+        <v>46279.39551385416</v>
       </c>
       <c r="K817" s="2" t="n">
         <v>46281</v>
@@ -62949,7 +62960,7 @@
     </row>
     <row r="818">
       <c r="A818" s="1" t="n">
-        <v>83912</v>
+        <v>83916</v>
       </c>
       <c r="B818" s="1" t="inlineStr">
         <is>
@@ -62972,11 +62983,11 @@
         </is>
       </c>
       <c r="F818" s="1" t="n">
-        <v>7056</v>
+        <v>7060</v>
       </c>
       <c r="G818" s="1" t="inlineStr">
         <is>
-          <t>AUTO CENTER EMBRASIL LTDA</t>
+          <t>GAPEMA LOCACAO DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="H818" s="1" t="inlineStr">
@@ -62990,7 +63001,7 @@
         </is>
       </c>
       <c r="J818" s="2" t="n">
-        <v>46279.39518283565</v>
+        <v>46279.39634756945</v>
       </c>
       <c r="K818" s="2" t="n">
         <v>46281</v>
@@ -63020,7 +63031,7 @@
     </row>
     <row r="819">
       <c r="A819" s="1" t="n">
-        <v>83913</v>
+        <v>83917</v>
       </c>
       <c r="B819" s="1" t="inlineStr">
         <is>
@@ -63043,11 +63054,11 @@
         </is>
       </c>
       <c r="F819" s="1" t="n">
-        <v>7057</v>
+        <v>7061</v>
       </c>
       <c r="G819" s="1" t="inlineStr">
         <is>
-          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (MATRIZ)</t>
+          <t>BF CORTES E FUROS TECNICOS E LOCACAO LTDA</t>
         </is>
       </c>
       <c r="H819" s="1" t="inlineStr">
@@ -63061,7 +63072,7 @@
         </is>
       </c>
       <c r="J819" s="2" t="n">
-        <v>46279.39551385416</v>
+        <v>46279.39663144676</v>
       </c>
       <c r="K819" s="2" t="n">
         <v>46281</v>
@@ -63091,7 +63102,7 @@
     </row>
     <row r="820">
       <c r="A820" s="1" t="n">
-        <v>83916</v>
+        <v>83918</v>
       </c>
       <c r="B820" s="1" t="inlineStr">
         <is>
@@ -63114,11 +63125,11 @@
         </is>
       </c>
       <c r="F820" s="1" t="n">
-        <v>7060</v>
+        <v>7062</v>
       </c>
       <c r="G820" s="1" t="inlineStr">
         <is>
-          <t>GAPEMA LOCACAO DE EQUIPAMENTOS LTDA</t>
+          <t>ALFA MAQUINAS LOCACAO E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="H820" s="1" t="inlineStr">
@@ -63132,7 +63143,7 @@
         </is>
       </c>
       <c r="J820" s="2" t="n">
-        <v>46279.39634756945</v>
+        <v>46279.39692175926</v>
       </c>
       <c r="K820" s="2" t="n">
         <v>46281</v>
@@ -63162,7 +63173,7 @@
     </row>
     <row r="821">
       <c r="A821" s="1" t="n">
-        <v>83917</v>
+        <v>83919</v>
       </c>
       <c r="B821" s="1" t="inlineStr">
         <is>
@@ -63185,11 +63196,11 @@
         </is>
       </c>
       <c r="F821" s="1" t="n">
-        <v>7061</v>
+        <v>7063</v>
       </c>
       <c r="G821" s="1" t="inlineStr">
         <is>
-          <t>BF CORTES E FUROS TECNICOS E LOCACAO LTDA</t>
+          <t>CR LOCACAO E VENDAS DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="H821" s="1" t="inlineStr">
@@ -63203,7 +63214,7 @@
         </is>
       </c>
       <c r="J821" s="2" t="n">
-        <v>46279.39663144676</v>
+        <v>46279.39713047454</v>
       </c>
       <c r="K821" s="2" t="n">
         <v>46281</v>
@@ -63233,39 +63244,39 @@
     </row>
     <row r="822">
       <c r="A822" s="1" t="n">
-        <v>83918</v>
+        <v>83982</v>
       </c>
       <c r="B822" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C822" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Sociedade - Comércio</t>
         </is>
       </c>
       <c r="D822" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E822" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t>Abertura de nova empresa do grupo: 7064-BC SUPERMERCADOTributação: Simples NacionalTipo de Atividade: ComércioFinalidade: OperacionalForma Juridica: LtdaProposta: já negociada no valor de R$1.800,00</t>
         </is>
       </c>
       <c r="F822" s="1" t="n">
-        <v>7062</v>
+        <v>7064</v>
       </c>
       <c r="G822" s="1" t="inlineStr">
         <is>
-          <t>ALFA MAQUINAS LOCACAO E SERVICOS LTDA</t>
+          <t>BISPO E CARVALHO SUPERMERCADO LTDA</t>
         </is>
       </c>
       <c r="H822" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I822" s="1" t="inlineStr">
@@ -63274,10 +63285,10 @@
         </is>
       </c>
       <c r="J822" s="2" t="n">
-        <v>46279.39692175926</v>
+        <v>46280.39557824074</v>
       </c>
       <c r="K822" s="2" t="n">
-        <v>46281</v>
+        <v>46308</v>
       </c>
       <c r="L822" s="1" t="inlineStr">
         <is>
@@ -63286,7 +63297,7 @@
       </c>
       <c r="M822" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N822" s="1" t="n"/>
@@ -63304,7 +63315,7 @@
     </row>
     <row r="823">
       <c r="A823" s="1" t="n">
-        <v>83919</v>
+        <v>83922</v>
       </c>
       <c r="B823" s="1" t="inlineStr">
         <is>
@@ -63327,16 +63338,16 @@
         </is>
       </c>
       <c r="F823" s="1" t="n">
-        <v>7063</v>
+        <v>7065</v>
       </c>
       <c r="G823" s="1" t="inlineStr">
         <is>
-          <t>CR LOCACAO E VENDAS DE EQUIPAMENTOS LTDA</t>
+          <t>GRANUA AGROINDUSTRIA E COMERCIO DE ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H823" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I823" s="1" t="inlineStr">
@@ -63345,7 +63356,7 @@
         </is>
       </c>
       <c r="J823" s="2" t="n">
-        <v>46279.39713047454</v>
+        <v>46279.39797662037</v>
       </c>
       <c r="K823" s="2" t="n">
         <v>46281</v>
@@ -63375,67 +63386,75 @@
     </row>
     <row r="824">
       <c r="A824" s="1" t="n">
-        <v>83982</v>
+        <v>83218</v>
       </c>
       <c r="B824" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C824" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Comércio</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D824" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E824" s="1" t="inlineStr">
         <is>
-          <t>Abertura de nova empresa do grupo: 7064-BC SUPERMERCADOTributação: Simples NacionalTipo de Atividade: ComércioFinalidade: OperacionalForma Juridica: LtdaProposta: já negociada no valor de R$1.800,00</t>
+          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa;Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F824" s="1" t="n">
-        <v>7064</v>
+        <v>7063</v>
       </c>
       <c r="G824" s="1" t="inlineStr">
         <is>
-          <t>BISPO E CARVALHO SUPERMERCADO LTDA</t>
+          <t>CR LOCACAO E VENDAS DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="H824" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I824" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J824" s="2" t="n">
-        <v>46280.39557824074</v>
+        <v>46262.49630575231</v>
       </c>
       <c r="K824" s="2" t="n">
-        <v>46308</v>
+        <v>46265</v>
       </c>
       <c r="L824" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M824" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N824" s="1" t="n"/>
-      <c r="O824" s="1" t="n"/>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N824" s="2" t="n">
+        <v>46267.54627245371</v>
+      </c>
+      <c r="O824" s="2" t="n">
+        <v>46283</v>
+      </c>
       <c r="P824" s="1" t="n"/>
       <c r="Q824" s="1" t="inlineStr"/>
-      <c r="R824" s="1" t="inlineStr"/>
+      <c r="R824" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando o SAC liberar para cobrar os documentos .</t>
+        </is>
+      </c>
       <c r="S824" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -63446,67 +63465,75 @@
     </row>
     <row r="825">
       <c r="A825" s="1" t="n">
-        <v>83922</v>
+        <v>83216</v>
       </c>
       <c r="B825" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C825" s="1" t="inlineStr">
         <is>
-          <t>Receita Federal</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D825" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E825" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderia providenciar o código de acesso do portal do Simples Nacional no MG controle.Desde já, agradeço.Atenciosamente.</t>
+          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa;Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F825" s="1" t="n">
-        <v>7065</v>
+        <v>7061</v>
       </c>
       <c r="G825" s="1" t="inlineStr">
         <is>
-          <t>GRANUA AGROINDUSTRIA E COMERCIO DE ALIMENTOS LTDA</t>
+          <t>BF CORTES E FUROS TECNICOS E LOCACAO LTDA</t>
         </is>
       </c>
       <c r="H825" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I825" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J825" s="2" t="n">
-        <v>46279.39797662037</v>
+        <v>46262.49574116898</v>
       </c>
       <c r="K825" s="2" t="n">
-        <v>46281</v>
+        <v>46265</v>
       </c>
       <c r="L825" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M825" s="1" t="inlineStr">
         <is>
-          <t>Ney Barbosa</t>
-        </is>
-      </c>
-      <c r="N825" s="1" t="n"/>
-      <c r="O825" s="1" t="n"/>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N825" s="2" t="n">
+        <v>46267.54612248843</v>
+      </c>
+      <c r="O825" s="2" t="n">
+        <v>46283</v>
+      </c>
       <c r="P825" s="1" t="n"/>
       <c r="Q825" s="1" t="inlineStr"/>
-      <c r="R825" s="1" t="inlineStr"/>
+      <c r="R825" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando o SAC liberar para cobrar os documentos .</t>
+        </is>
+      </c>
       <c r="S825" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -63517,7 +63544,7 @@
     </row>
     <row r="826">
       <c r="A826" s="1" t="n">
-        <v>83218</v>
+        <v>83217</v>
       </c>
       <c r="B826" s="1" t="inlineStr">
         <is>
@@ -63540,11 +63567,11 @@
         </is>
       </c>
       <c r="F826" s="1" t="n">
-        <v>7063</v>
+        <v>7062</v>
       </c>
       <c r="G826" s="1" t="inlineStr">
         <is>
-          <t>CR LOCACAO E VENDAS DE EQUIPAMENTOS LTDA</t>
+          <t>ALFA MAQUINAS LOCACAO E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="H826" s="1" t="inlineStr">
@@ -63554,18 +63581,18 @@
       </c>
       <c r="I826" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J826" s="2" t="n">
-        <v>46262.49630575231</v>
+        <v>46262.49604351852</v>
       </c>
       <c r="K826" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="L826" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M826" s="1" t="inlineStr">
@@ -63573,9 +63600,7 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N826" s="2" t="n">
-        <v>46267.54627245371</v>
-      </c>
+      <c r="N826" s="1" t="n"/>
       <c r="O826" s="2" t="n">
         <v>46283</v>
       </c>
@@ -63591,12 +63616,16 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T826" s="1" t="n"/>
+      <c r="T826" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
       <c r="U826" s="1" t="inlineStr"/>
     </row>
     <row r="827">
       <c r="A827" s="1" t="n">
-        <v>83216</v>
+        <v>83213</v>
       </c>
       <c r="B827" s="1" t="inlineStr">
         <is>
@@ -63619,11 +63648,11 @@
         </is>
       </c>
       <c r="F827" s="1" t="n">
-        <v>7061</v>
+        <v>7058</v>
       </c>
       <c r="G827" s="1" t="inlineStr">
         <is>
-          <t>BF CORTES E FUROS TECNICOS E LOCACAO LTDA</t>
+          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H827" s="1" t="inlineStr">
@@ -63633,18 +63662,18 @@
       </c>
       <c r="I827" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J827" s="2" t="n">
-        <v>46262.49574116898</v>
+        <v>46262.49500332176</v>
       </c>
       <c r="K827" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="L827" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M827" s="1" t="inlineStr">
@@ -63652,9 +63681,7 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N827" s="2" t="n">
-        <v>46267.54612248843</v>
-      </c>
+      <c r="N827" s="1" t="n"/>
       <c r="O827" s="2" t="n">
         <v>46283</v>
       </c>
@@ -63670,12 +63697,16 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T827" s="1" t="n"/>
+      <c r="T827" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
       <c r="U827" s="1" t="inlineStr"/>
     </row>
     <row r="828">
       <c r="A828" s="1" t="n">
-        <v>83217</v>
+        <v>83214</v>
       </c>
       <c r="B828" s="1" t="inlineStr">
         <is>
@@ -63698,11 +63729,11 @@
         </is>
       </c>
       <c r="F828" s="1" t="n">
-        <v>7062</v>
+        <v>7059</v>
       </c>
       <c r="G828" s="1" t="inlineStr">
         <is>
-          <t>ALFA MAQUINAS LOCACAO E SERVICOS LTDA</t>
+          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (FILIAL 2)</t>
         </is>
       </c>
       <c r="H828" s="1" t="inlineStr">
@@ -63716,7 +63747,7 @@
         </is>
       </c>
       <c r="J828" s="2" t="n">
-        <v>46262.49604351852</v>
+        <v>46262.49526809028</v>
       </c>
       <c r="K828" s="2" t="n">
         <v>46265</v>
@@ -63756,7 +63787,7 @@
     </row>
     <row r="829">
       <c r="A829" s="1" t="n">
-        <v>83213</v>
+        <v>83215</v>
       </c>
       <c r="B829" s="1" t="inlineStr">
         <is>
@@ -63779,11 +63810,11 @@
         </is>
       </c>
       <c r="F829" s="1" t="n">
-        <v>7058</v>
+        <v>7060</v>
       </c>
       <c r="G829" s="1" t="inlineStr">
         <is>
-          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (FILIAL 1)</t>
+          <t>GAPEMA LOCACAO DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="H829" s="1" t="inlineStr">
@@ -63793,18 +63824,18 @@
       </c>
       <c r="I829" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J829" s="2" t="n">
-        <v>46262.49500332176</v>
+        <v>46262.49551331018</v>
       </c>
       <c r="K829" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="L829" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M829" s="1" t="inlineStr">
@@ -63812,7 +63843,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N829" s="1" t="n"/>
+      <c r="N829" s="2" t="n">
+        <v>46267.54604818287</v>
+      </c>
       <c r="O829" s="2" t="n">
         <v>46283</v>
       </c>
@@ -63828,16 +63861,12 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T829" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
+      <c r="T829" s="1" t="n"/>
       <c r="U829" s="1" t="inlineStr"/>
     </row>
     <row r="830">
       <c r="A830" s="1" t="n">
-        <v>83214</v>
+        <v>83117</v>
       </c>
       <c r="B830" s="1" t="inlineStr">
         <is>
@@ -63856,15 +63885,15 @@
       </c>
       <c r="E830" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa;Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa.</t>
         </is>
       </c>
       <c r="F830" s="1" t="n">
-        <v>7059</v>
+        <v>7056</v>
       </c>
       <c r="G830" s="1" t="inlineStr">
         <is>
-          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (FILIAL 2)</t>
+          <t>AUTO CENTER EMBRASIL LTDA</t>
         </is>
       </c>
       <c r="H830" s="1" t="inlineStr">
@@ -63874,18 +63903,18 @@
       </c>
       <c r="I830" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J830" s="2" t="n">
-        <v>46262.49526809028</v>
+        <v>46261.47502040509</v>
       </c>
       <c r="K830" s="2" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="L830" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M830" s="1" t="inlineStr">
@@ -63893,7 +63922,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N830" s="1" t="n"/>
+      <c r="N830" s="2" t="n">
+        <v>46261.69782774305</v>
+      </c>
       <c r="O830" s="2" t="n">
         <v>46283</v>
       </c>
@@ -63901,7 +63932,7 @@
       <c r="Q830" s="1" t="inlineStr"/>
       <c r="R830" s="1" t="inlineStr">
         <is>
-          <t>Aguardando o SAC liberar para cobrar os documentos .</t>
+          <t>Cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S830" s="1" t="inlineStr">
@@ -63909,16 +63940,12 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T830" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
+      <c r="T830" s="1" t="n"/>
       <c r="U830" s="1" t="inlineStr"/>
     </row>
     <row r="831">
       <c r="A831" s="1" t="n">
-        <v>83215</v>
+        <v>83212</v>
       </c>
       <c r="B831" s="1" t="inlineStr">
         <is>
@@ -63941,11 +63968,11 @@
         </is>
       </c>
       <c r="F831" s="1" t="n">
-        <v>7060</v>
+        <v>7057</v>
       </c>
       <c r="G831" s="1" t="inlineStr">
         <is>
-          <t>GAPEMA LOCACAO DE EQUIPAMENTOS LTDA</t>
+          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H831" s="1" t="inlineStr">
@@ -63955,18 +63982,18 @@
       </c>
       <c r="I831" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J831" s="2" t="n">
-        <v>46262.49551331018</v>
+        <v>46262.49474181713</v>
       </c>
       <c r="K831" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="L831" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M831" s="1" t="inlineStr">
@@ -63974,9 +64001,7 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N831" s="2" t="n">
-        <v>46267.54604818287</v>
-      </c>
+      <c r="N831" s="1" t="n"/>
       <c r="O831" s="2" t="n">
         <v>46283</v>
       </c>
@@ -63992,12 +64017,16 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T831" s="1" t="n"/>
+      <c r="T831" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
       <c r="U831" s="1" t="inlineStr"/>
     </row>
     <row r="832">
       <c r="A832" s="1" t="n">
-        <v>83117</v>
+        <v>83115</v>
       </c>
       <c r="B832" s="1" t="inlineStr">
         <is>
@@ -64020,11 +64049,11 @@
         </is>
       </c>
       <c r="F832" s="1" t="n">
-        <v>7056</v>
+        <v>7054</v>
       </c>
       <c r="G832" s="1" t="inlineStr">
         <is>
-          <t>AUTO CENTER EMBRASIL LTDA</t>
+          <t>KADOSH DISTRIBUIDOR COMERCIO E SERVICO DIGITAL LTDA</t>
         </is>
       </c>
       <c r="H832" s="1" t="inlineStr">
@@ -64038,7 +64067,7 @@
         </is>
       </c>
       <c r="J832" s="2" t="n">
-        <v>46261.47502040509</v>
+        <v>46261.47454267361</v>
       </c>
       <c r="K832" s="2" t="n">
         <v>46262</v>
@@ -64054,7 +64083,7 @@
         </is>
       </c>
       <c r="N832" s="2" t="n">
-        <v>46261.69782774305</v>
+        <v>46261.6975778125</v>
       </c>
       <c r="O832" s="2" t="n">
         <v>46283</v>
@@ -64076,7 +64105,7 @@
     </row>
     <row r="833">
       <c r="A833" s="1" t="n">
-        <v>83212</v>
+        <v>83116</v>
       </c>
       <c r="B833" s="1" t="inlineStr">
         <is>
@@ -64095,15 +64124,15 @@
       </c>
       <c r="E833" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa;Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa.</t>
         </is>
       </c>
       <c r="F833" s="1" t="n">
-        <v>7057</v>
+        <v>7055</v>
       </c>
       <c r="G833" s="1" t="inlineStr">
         <is>
-          <t>JP LOCACAO COMERCIO DE EQUIPAMENTOS LTDA (MATRIZ)</t>
+          <t>YURI CESTARI DA SILVA EMBREAGENS OSASCO</t>
         </is>
       </c>
       <c r="H833" s="1" t="inlineStr">
@@ -64113,18 +64142,18 @@
       </c>
       <c r="I833" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J833" s="2" t="n">
-        <v>46262.49474181713</v>
+        <v>46261.47479783565</v>
       </c>
       <c r="K833" s="2" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="L833" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M833" s="1" t="inlineStr">
@@ -64132,7 +64161,9 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N833" s="1" t="n"/>
+      <c r="N833" s="2" t="n">
+        <v>46261.69765454861</v>
+      </c>
       <c r="O833" s="2" t="n">
         <v>46283</v>
       </c>
@@ -64140,7 +64171,7 @@
       <c r="Q833" s="1" t="inlineStr"/>
       <c r="R833" s="1" t="inlineStr">
         <is>
-          <t>Aguardando o SAC liberar para cobrar os documentos .</t>
+          <t>Cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S833" s="1" t="inlineStr">
@@ -64148,16 +64179,12 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T833" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
+      <c r="T833" s="1" t="n"/>
       <c r="U833" s="1" t="inlineStr"/>
     </row>
     <row r="834">
       <c r="A834" s="1" t="n">
-        <v>83115</v>
+        <v>83112</v>
       </c>
       <c r="B834" s="1" t="inlineStr">
         <is>
@@ -64180,11 +64207,11 @@
         </is>
       </c>
       <c r="F834" s="1" t="n">
-        <v>7054</v>
+        <v>7052</v>
       </c>
       <c r="G834" s="1" t="inlineStr">
         <is>
-          <t>KADOSH DISTRIBUIDOR COMERCIO E SERVICO DIGITAL LTDA</t>
+          <t>EMBRASIL COMERCIO DE AUTO PECAS LTDA</t>
         </is>
       </c>
       <c r="H834" s="1" t="inlineStr">
@@ -64198,7 +64225,7 @@
         </is>
       </c>
       <c r="J834" s="2" t="n">
-        <v>46261.47454267361</v>
+        <v>46261.47219082176</v>
       </c>
       <c r="K834" s="2" t="n">
         <v>46262</v>
@@ -64214,7 +64241,7 @@
         </is>
       </c>
       <c r="N834" s="2" t="n">
-        <v>46261.6975778125</v>
+        <v>46261.69723422454</v>
       </c>
       <c r="O834" s="2" t="n">
         <v>46283</v>
@@ -64236,7 +64263,7 @@
     </row>
     <row r="835">
       <c r="A835" s="1" t="n">
-        <v>83116</v>
+        <v>82905</v>
       </c>
       <c r="B835" s="1" t="inlineStr">
         <is>
@@ -64255,15 +64282,15 @@
       </c>
       <c r="E835" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa.</t>
+          <t xml:space="preserve">Boa tarde, por gentileza, solicitar os documentos para a implantação da empresa. </t>
         </is>
       </c>
       <c r="F835" s="1" t="n">
-        <v>7055</v>
+        <v>7046</v>
       </c>
       <c r="G835" s="1" t="inlineStr">
         <is>
-          <t>YURI CESTARI DA SILVA EMBREAGENS OSASCO</t>
+          <t>RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDA</t>
         </is>
       </c>
       <c r="H835" s="1" t="inlineStr">
@@ -64277,10 +64304,10 @@
         </is>
       </c>
       <c r="J835" s="2" t="n">
-        <v>46261.47479783565</v>
+        <v>46258.65608700232</v>
       </c>
       <c r="K835" s="2" t="n">
-        <v>46262</v>
+        <v>46259</v>
       </c>
       <c r="L835" s="1" t="inlineStr">
         <is>
@@ -64293,7 +64320,7 @@
         </is>
       </c>
       <c r="N835" s="2" t="n">
-        <v>46261.69765454861</v>
+        <v>46259.7507258449</v>
       </c>
       <c r="O835" s="2" t="n">
         <v>46283</v>
@@ -64302,7 +64329,7 @@
       <c r="Q835" s="1" t="inlineStr"/>
       <c r="R835" s="1" t="inlineStr">
         <is>
-          <t>Cobramos os documentos do antigo contador.</t>
+          <t xml:space="preserve">Cobramos os documentos </t>
         </is>
       </c>
       <c r="S835" s="1" t="inlineStr">
@@ -64315,7 +64342,7 @@
     </row>
     <row r="836">
       <c r="A836" s="1" t="n">
-        <v>83112</v>
+        <v>82755</v>
       </c>
       <c r="B836" s="1" t="inlineStr">
         <is>
@@ -64334,15 +64361,15 @@
       </c>
       <c r="E836" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza, providenciar os documentos para implantação da empresa.</t>
+          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
         </is>
       </c>
       <c r="F836" s="1" t="n">
-        <v>7052</v>
+        <v>7005</v>
       </c>
       <c r="G836" s="1" t="inlineStr">
         <is>
-          <t>EMBRASIL COMERCIO DE AUTO PECAS LTDA</t>
+          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H836" s="1" t="inlineStr">
@@ -64356,10 +64383,10 @@
         </is>
       </c>
       <c r="J836" s="2" t="n">
-        <v>46261.47219082176</v>
+        <v>46254.65957604167</v>
       </c>
       <c r="K836" s="2" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="L836" s="1" t="inlineStr">
         <is>
@@ -64372,7 +64399,7 @@
         </is>
       </c>
       <c r="N836" s="2" t="n">
-        <v>46261.69723422454</v>
+        <v>46255.48691519676</v>
       </c>
       <c r="O836" s="2" t="n">
         <v>46283</v>
@@ -64381,7 +64408,7 @@
       <c r="Q836" s="1" t="inlineStr"/>
       <c r="R836" s="1" t="inlineStr">
         <is>
-          <t>Cobramos os documentos do antigo contador.</t>
+          <t>cobramos novamente o retorno dos documentos</t>
         </is>
       </c>
       <c r="S836" s="1" t="inlineStr">
@@ -64394,7 +64421,7 @@
     </row>
     <row r="837">
       <c r="A837" s="1" t="n">
-        <v>82905</v>
+        <v>82756</v>
       </c>
       <c r="B837" s="1" t="inlineStr">
         <is>
@@ -64413,15 +64440,15 @@
       </c>
       <c r="E837" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, solicitar os documentos para a implantação da empresa. </t>
+          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
         </is>
       </c>
       <c r="F837" s="1" t="n">
-        <v>7046</v>
+        <v>7006</v>
       </c>
       <c r="G837" s="1" t="inlineStr">
         <is>
-          <t>RAMIRO EQUIPAMENTOS GASTRONOMICOS LTDA</t>
+          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H837" s="1" t="inlineStr">
@@ -64435,10 +64462,10 @@
         </is>
       </c>
       <c r="J837" s="2" t="n">
-        <v>46258.65608700232</v>
+        <v>46254.65986380787</v>
       </c>
       <c r="K837" s="2" t="n">
-        <v>46259</v>
+        <v>46255</v>
       </c>
       <c r="L837" s="1" t="inlineStr">
         <is>
@@ -64451,7 +64478,7 @@
         </is>
       </c>
       <c r="N837" s="2" t="n">
-        <v>46259.7507258449</v>
+        <v>46255.48792758102</v>
       </c>
       <c r="O837" s="2" t="n">
         <v>46283</v>
@@ -64460,7 +64487,7 @@
       <c r="Q837" s="1" t="inlineStr"/>
       <c r="R837" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobramos os documentos </t>
+          <t>cobramos novamente os documentos</t>
         </is>
       </c>
       <c r="S837" s="1" t="inlineStr">
@@ -64473,7 +64500,7 @@
     </row>
     <row r="838">
       <c r="A838" s="1" t="n">
-        <v>82755</v>
+        <v>79867</v>
       </c>
       <c r="B838" s="1" t="inlineStr">
         <is>
@@ -64482,30 +64509,30 @@
       </c>
       <c r="C838" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D838" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E838" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F838" s="1" t="n">
-        <v>7005</v>
+        <v>6704</v>
       </c>
       <c r="G838" s="1" t="inlineStr">
         <is>
-          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H838" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I838" s="1" t="inlineStr">
@@ -64514,10 +64541,10 @@
         </is>
       </c>
       <c r="J838" s="2" t="n">
-        <v>46254.65957604167</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K838" s="2" t="n">
-        <v>46255</v>
+        <v>46185</v>
       </c>
       <c r="L838" s="1" t="inlineStr">
         <is>
@@ -64526,20 +64553,19 @@
       </c>
       <c r="M838" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N838" s="2" t="n">
-        <v>46255.48691519676</v>
-      </c>
-      <c r="O838" s="2" t="n">
-        <v>46283</v>
-      </c>
+        <v>46237.4174340625</v>
+      </c>
+      <c r="O838" s="1" t="n"/>
       <c r="P838" s="1" t="n"/>
       <c r="Q838" s="1" t="inlineStr"/>
       <c r="R838" s="1" t="inlineStr">
         <is>
-          <t>cobramos novamente o retorno dos documentos</t>
+          <t>Bom dia!
+Cobramos a antiga contabilidade.</t>
         </is>
       </c>
       <c r="S838" s="1" t="inlineStr">
@@ -64552,7 +64578,7 @@
     </row>
     <row r="839">
       <c r="A839" s="1" t="n">
-        <v>82756</v>
+        <v>82310</v>
       </c>
       <c r="B839" s="1" t="inlineStr">
         <is>
@@ -64561,25 +64587,25 @@
       </c>
       <c r="C839" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D839" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E839" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
+          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
         </is>
       </c>
       <c r="F839" s="1" t="n">
-        <v>7006</v>
+        <v>6974</v>
       </c>
       <c r="G839" s="1" t="inlineStr">
         <is>
-          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
         </is>
       </c>
       <c r="H839" s="1" t="inlineStr">
@@ -64593,10 +64619,10 @@
         </is>
       </c>
       <c r="J839" s="2" t="n">
-        <v>46254.65986380787</v>
+        <v>46247.3783179051</v>
       </c>
       <c r="K839" s="2" t="n">
-        <v>46255</v>
+        <v>46248</v>
       </c>
       <c r="L839" s="1" t="inlineStr">
         <is>
@@ -64605,20 +64631,20 @@
       </c>
       <c r="M839" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N839" s="2" t="n">
-        <v>46255.48792758102</v>
+        <v>46253.39089305556</v>
       </c>
       <c r="O839" s="2" t="n">
-        <v>46283</v>
+        <v>46297</v>
       </c>
       <c r="P839" s="1" t="n"/>
       <c r="Q839" s="1" t="inlineStr"/>
       <c r="R839" s="1" t="inlineStr">
         <is>
-          <t>cobramos novamente os documentos</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S839" s="1" t="inlineStr">
@@ -64631,16 +64657,16 @@
     </row>
     <row r="840">
       <c r="A840" s="1" t="n">
-        <v>79867</v>
+        <v>79865</v>
       </c>
       <c r="B840" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C840" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D840" s="1" t="inlineStr">
@@ -64650,20 +64676,20 @@
       </c>
       <c r="E840" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F840" s="1" t="n">
-        <v>6704</v>
+        <v>6278</v>
       </c>
       <c r="G840" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H840" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I840" s="1" t="inlineStr">
@@ -64672,7 +64698,7 @@
         </is>
       </c>
       <c r="J840" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K840" s="2" t="n">
         <v>46185</v>
@@ -64688,7 +64714,7 @@
         </is>
       </c>
       <c r="N840" s="2" t="n">
-        <v>46237.4174340625</v>
+        <v>46246.6616841088</v>
       </c>
       <c r="O840" s="1" t="n"/>
       <c r="P840" s="1" t="n"/>
@@ -64696,7 +64722,7 @@
       <c r="R840" s="1" t="inlineStr">
         <is>
           <t>Bom dia!
-Cobramos a antiga contabilidade.</t>
+Já foi atendido?</t>
         </is>
       </c>
       <c r="S840" s="1" t="inlineStr">
@@ -64709,7 +64735,7 @@
     </row>
     <row r="841">
       <c r="A841" s="1" t="n">
-        <v>82310</v>
+        <v>82701</v>
       </c>
       <c r="B841" s="1" t="inlineStr">
         <is>
@@ -64718,27 +64744,23 @@
       </c>
       <c r="C841" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D841" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E841" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
+          <t>Boa tarde, por gentileza, providencias documentos de implantação da empresa: 7037 - EXPANDItens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F841" s="1" t="n">
-        <v>6974</v>
-      </c>
-      <c r="G841" s="1" t="inlineStr">
-        <is>
-          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G841" s="1" t="n"/>
       <c r="H841" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -64750,10 +64772,10 @@
         </is>
       </c>
       <c r="J841" s="2" t="n">
-        <v>46247.3783179051</v>
+        <v>46253.71124814815</v>
       </c>
       <c r="K841" s="2" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="L841" s="1" t="inlineStr">
         <is>
@@ -64762,20 +64784,20 @@
       </c>
       <c r="M841" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N841" s="2" t="n">
-        <v>46253.39089305556</v>
+        <v>46255.46909065972</v>
       </c>
       <c r="O841" s="2" t="n">
-        <v>46297</v>
+        <v>46283</v>
       </c>
       <c r="P841" s="1" t="n"/>
       <c r="Q841" s="1" t="inlineStr"/>
       <c r="R841" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t xml:space="preserve">CObramos os documentos </t>
         </is>
       </c>
       <c r="S841" s="1" t="inlineStr">
@@ -64788,36 +64810,32 @@
     </row>
     <row r="842">
       <c r="A842" s="1" t="n">
-        <v>79865</v>
+        <v>82706</v>
       </c>
       <c r="B842" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C842" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D842" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E842" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 6978 - HEPA FILTROS.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F842" s="1" t="n">
-        <v>6278</v>
-      </c>
-      <c r="G842" s="1" t="inlineStr">
-        <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G842" s="1" t="n"/>
       <c r="H842" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -64829,10 +64847,10 @@
         </is>
       </c>
       <c r="J842" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46253.72086076389</v>
       </c>
       <c r="K842" s="2" t="n">
-        <v>46185</v>
+        <v>46255</v>
       </c>
       <c r="L842" s="1" t="inlineStr">
         <is>
@@ -64841,19 +64859,18 @@
       </c>
       <c r="M842" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N842" s="2" t="n">
-        <v>46246.6616841088</v>
+        <v>46255.48540517361</v>
       </c>
       <c r="O842" s="1" t="n"/>
       <c r="P842" s="1" t="n"/>
       <c r="Q842" s="1" t="inlineStr"/>
       <c r="R842" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!
-Já foi atendido?</t>
+          <t>cobramos os documentos.</t>
         </is>
       </c>
       <c r="S842" s="1" t="inlineStr">
@@ -64863,227 +64880,6 @@
       </c>
       <c r="T842" s="1" t="n"/>
       <c r="U842" s="1" t="inlineStr"/>
-    </row>
-    <row r="843">
-      <c r="A843" s="1" t="n">
-        <v>82701</v>
-      </c>
-      <c r="B843" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C843" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D843" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E843" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde, por gentileza, providencias documentos de implantação da empresa: 7037 - EXPANDItens dispensáveis, por gentileza, sinalizar.</t>
-        </is>
-      </c>
-      <c r="F843" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G843" s="1" t="n"/>
-      <c r="H843" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I843" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J843" s="2" t="n">
-        <v>46253.71124814815</v>
-      </c>
-      <c r="K843" s="2" t="n">
-        <v>46255</v>
-      </c>
-      <c r="L843" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M843" s="1" t="inlineStr">
-        <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N843" s="2" t="n">
-        <v>46255.46909065972</v>
-      </c>
-      <c r="O843" s="2" t="n">
-        <v>46283</v>
-      </c>
-      <c r="P843" s="1" t="n"/>
-      <c r="Q843" s="1" t="inlineStr"/>
-      <c r="R843" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CObramos os documentos </t>
-        </is>
-      </c>
-      <c r="S843" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T843" s="1" t="n"/>
-      <c r="U843" s="1" t="inlineStr"/>
-    </row>
-    <row r="844">
-      <c r="A844" s="1" t="n">
-        <v>82706</v>
-      </c>
-      <c r="B844" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C844" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D844" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E844" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 6978 - HEPA FILTROS.Itens dispensáveis, por gentileza, sinalizar.</t>
-        </is>
-      </c>
-      <c r="F844" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G844" s="1" t="n"/>
-      <c r="H844" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I844" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J844" s="2" t="n">
-        <v>46253.72086076389</v>
-      </c>
-      <c r="K844" s="2" t="n">
-        <v>46255</v>
-      </c>
-      <c r="L844" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M844" s="1" t="inlineStr">
-        <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N844" s="2" t="n">
-        <v>46255.48540517361</v>
-      </c>
-      <c r="O844" s="1" t="n"/>
-      <c r="P844" s="1" t="n"/>
-      <c r="Q844" s="1" t="inlineStr"/>
-      <c r="R844" s="1" t="inlineStr">
-        <is>
-          <t>cobramos os documentos.</t>
-        </is>
-      </c>
-      <c r="S844" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T844" s="1" t="n"/>
-      <c r="U844" s="1" t="inlineStr"/>
-    </row>
-    <row r="845">
-      <c r="A845" s="1" t="n">
-        <v>81055</v>
-      </c>
-      <c r="B845" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C845" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D845" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E845" s="1" t="inlineStr">
-        <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
-        </is>
-      </c>
-      <c r="F845" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G845" s="1" t="n"/>
-      <c r="H845" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I845" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J845" s="2" t="n">
-        <v>46218.40379614583</v>
-      </c>
-      <c r="K845" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="L845" s="1" t="inlineStr">
-        <is>
-          <t>Devolvido</t>
-        </is>
-      </c>
-      <c r="M845" s="1" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N845" s="1" t="n"/>
-      <c r="O845" s="2" t="n">
-        <v>46295</v>
-      </c>
-      <c r="P845" s="1" t="n"/>
-      <c r="Q845" s="1" t="inlineStr"/>
-      <c r="R845" s="1" t="inlineStr">
-        <is>
-          <t>Aguardando retorno dos dados do contador</t>
-        </is>
-      </c>
-      <c r="S845" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T845" s="1" t="n"/>
-      <c r="U845" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-23 15:42
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1097,7 +1097,7 @@
       <c r="G8" s="1" t="n"/>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Edivaldo Veiga</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="L8" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M8" s="1" t="inlineStr">
@@ -1121,28 +1121,18 @@
           <t>Mauricio Lermen</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
-        <v>46288.63074707176</v>
-      </c>
+      <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="n"/>
       <c r="Q8" s="1" t="inlineStr"/>
-      <c r="R8" s="1" t="inlineStr">
-        <is>
-          <t>Cadastros revisados e atualizações realizadas, nas empresas de prola-bore, pendente as empresas de domésticas. Em andamento.</t>
-        </is>
-      </c>
+      <c r="R8" s="1" t="inlineStr"/>
       <c r="S8" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T8" s="1" t="n"/>
-      <c r="U8" s="1" t="inlineStr">
-        <is>
-          <t>Edivaldo Veiga</t>
-        </is>
-      </c>
+      <c r="U8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -15662,7 +15652,11 @@
           <t>NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H183" s="1" t="n"/>
+      <c r="H183" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I183" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -15676,7 +15670,7 @@
       </c>
       <c r="L183" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M183" s="1" t="inlineStr">
@@ -15688,14 +15682,18 @@
       <c r="O183" s="1" t="n"/>
       <c r="P183" s="1" t="n"/>
       <c r="Q183" s="1" t="inlineStr"/>
-      <c r="R183" s="1" t="n"/>
+      <c r="R183" s="1" t="inlineStr"/>
       <c r="S183" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T183" s="1" t="n"/>
-      <c r="U183" s="1" t="inlineStr"/>
+      <c r="U183" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -16164,7 +16162,11 @@
           <t>POWER FINANCIAL DO BRASIL S.A. (FILIAL 1)</t>
         </is>
       </c>
-      <c r="H189" s="1" t="n"/>
+      <c r="H189" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I189" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -16178,7 +16180,7 @@
       </c>
       <c r="L189" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M189" s="1" t="inlineStr">
@@ -16190,14 +16192,18 @@
       <c r="O189" s="1" t="n"/>
       <c r="P189" s="1" t="n"/>
       <c r="Q189" s="1" t="inlineStr"/>
-      <c r="R189" s="1" t="n"/>
+      <c r="R189" s="1" t="inlineStr"/>
       <c r="S189" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T189" s="1" t="n"/>
-      <c r="U189" s="1" t="inlineStr"/>
+      <c r="U189" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -51859,7 +51865,7 @@
       </c>
       <c r="L677" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M677" s="1" t="inlineStr">
@@ -51867,7 +51873,9 @@
           <t>Ricardo Fischer</t>
         </is>
       </c>
-      <c r="N677" s="1" t="n"/>
+      <c r="N677" s="2" t="n">
+        <v>46288.64739603009</v>
+      </c>
       <c r="O677" s="1" t="n"/>
       <c r="P677" s="1" t="n"/>
       <c r="Q677" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 08:46
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -10135,16 +10135,16 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>84337</v>
+        <v>83101</v>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza verificar resultado de 2025, DRE do período com resultado de R$ 58.181,84 e Balanço R$58.163,88</t>
+          <t xml:space="preserve">Bom dia, por gentileza verificar a pendência e encaminhar ao cliente. </t>
         </is>
       </c>
       <c r="F117" s="1" t="n">
@@ -10167,23 +10167,23 @@
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I117" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J117" s="2" t="n">
-        <v>46287.7431491088</v>
+        <v>46261.41588966435</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>46288</v>
+        <v>46265</v>
       </c>
       <c r="L117" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M117" s="1" t="inlineStr">
@@ -10191,35 +10191,45 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N117" s="1" t="n"/>
-      <c r="O117" s="1" t="n"/>
-      <c r="P117" s="1" t="n"/>
-      <c r="Q117" s="1" t="inlineStr"/>
-      <c r="R117" s="1" t="inlineStr"/>
+      <c r="N117" s="2" t="n">
+        <v>46261.6168647801</v>
+      </c>
+      <c r="O117" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="P117" s="2" t="n">
+        <v>46266.68528174768</v>
+      </c>
+      <c r="Q117" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R117" s="1" t="inlineStr">
+        <is>
+          <t>em analise</t>
+        </is>
+      </c>
       <c r="S117" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T117" s="1" t="n"/>
-      <c r="U117" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
+      <c r="U117" s="1" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>83101</v>
+        <v>83532</v>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
@@ -10229,7 +10239,7 @@
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, por gentileza verificar a pendência e encaminhar ao cliente. </t>
+          <t>Bom dia, por gentileza anexar balanço e dre 2025 e 2026 separados. das empresas 5053 RJR 5054 DINIZ5873 FRRD 6450 RDF</t>
         </is>
       </c>
       <c r="F118" s="1" t="n">
@@ -10242,19 +10252,19 @@
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="I118" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J118" s="2" t="n">
-        <v>46261.41588966435</v>
+        <v>46268.36181149306</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="L118" s="1" t="inlineStr">
         <is>
@@ -10266,23 +10276,21 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N118" s="2" t="n">
-        <v>46261.6168647801</v>
-      </c>
+      <c r="N118" s="1" t="n"/>
       <c r="O118" s="2" t="n">
-        <v>46266</v>
+        <v>46290</v>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46266.68528174768</v>
+        <v>46287.75748996528</v>
       </c>
       <c r="Q118" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="R118" s="1" t="inlineStr">
         <is>
-          <t>em analise</t>
+          <t>em anexo</t>
         </is>
       </c>
       <c r="S118" s="1" t="inlineStr">
@@ -10291,20 +10299,24 @@
         </is>
       </c>
       <c r="T118" s="1" t="n"/>
-      <c r="U118" s="1" t="inlineStr"/>
+      <c r="U118" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>83532</v>
+        <v>81712</v>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
@@ -10314,32 +10326,32 @@
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza anexar balanço e dre 2025 e 2026 separados. das empresas 5053 RJR 5054 DINIZ5873 FRRD 6450 RDF</t>
+          <t>Prezados,Por gentileza, providenciar regularização do transporte de saldo credor incorreto ICMS período 08, 11 e 12/2025.Grato,Bruno.</t>
         </is>
       </c>
       <c r="F119" s="1" t="n">
-        <v>5053</v>
+        <v>5100</v>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>RJR INDUSTRIA DE ALIMENTOS LTDA</t>
+          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I119" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J119" s="2" t="n">
-        <v>46268.36181149306</v>
+        <v>46234.60319799768</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>46269</v>
+        <v>46241</v>
       </c>
       <c r="L119" s="1" t="inlineStr">
         <is>
@@ -10348,115 +10360,115 @@
       </c>
       <c r="M119" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N119" s="1" t="n"/>
       <c r="O119" s="2" t="n">
-        <v>46290</v>
+        <v>46241</v>
       </c>
       <c r="P119" s="2" t="n">
-        <v>46287.75748996528</v>
+        <v>46241.67638564815</v>
       </c>
       <c r="Q119" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="R119" s="1" t="inlineStr">
-        <is>
-          <t>em anexo</t>
-        </is>
-      </c>
-      <c r="S119" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T119" s="1" t="n"/>
-      <c r="U119" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="1" t="n">
-        <v>81712</v>
-      </c>
-      <c r="B120" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Credor Incorreto</t>
-        </is>
-      </c>
-      <c r="C120" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Credor Incorreto</t>
-        </is>
-      </c>
-      <c r="D120" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E120" s="1" t="inlineStr">
-        <is>
-          <t>Prezados,Por gentileza, providenciar regularização do transporte de saldo credor incorreto ICMS período 08, 11 e 12/2025.Grato,Bruno.</t>
-        </is>
-      </c>
-      <c r="F120" s="1" t="n">
-        <v>5100</v>
-      </c>
-      <c r="G120" s="1" t="inlineStr">
-        <is>
-          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
-        </is>
-      </c>
-      <c r="H120" s="1" t="inlineStr">
-        <is>
-          <t>Thaiza Oliveira</t>
-        </is>
-      </c>
-      <c r="I120" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J120" s="2" t="n">
-        <v>46234.60319799768</v>
-      </c>
-      <c r="K120" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="L120" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M120" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N120" s="1" t="n"/>
-      <c r="O120" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="P120" s="2" t="n">
-        <v>46241.67638564815</v>
-      </c>
-      <c r="Q120" s="1" t="inlineStr">
-        <is>
-          <t>Thaiza Oliveira</t>
-        </is>
-      </c>
-      <c r="R120" s="1" t="inlineStr">
         <is>
           <t>Boa tarde,
 O saldo credor deste período refere-se aos meses de 01 a 07/2025, nos quais o cliente não enviou os arquivos SPED ou os encaminhou com inconsistências.Não recebemos o retorno e a montagem não estava autorizada.
 Para regularizar essa pendência, solicitamos, por gentileza, que sejam solicitados ao cliente os arquivos SPED corrigidos referentes ao período de 01 a 07/2025.</t>
         </is>
       </c>
+      <c r="S119" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T119" s="1" t="n"/>
+      <c r="U119" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>79665</v>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>Autorregularização</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>Autorregularização</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E120" s="1" t="inlineStr">
+        <is>
+          <t>Autoregularização - Simples Nacional - Janeiro a Dezembro 2024Cliente recebeu notificação de autoregularização do Simples Nacional referente período 2024. Por gentileza, providenciar retificação dentro do prazo estipulado pela Receita.</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="n">
+        <v>5100</v>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
+        </is>
+      </c>
+      <c r="H120" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
+      <c r="I120" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>46176.49184155092</v>
+      </c>
+      <c r="K120" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="L120" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M120" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>46183.62114679398</v>
+      </c>
+      <c r="O120" s="1" t="n"/>
+      <c r="P120" s="2" t="n">
+        <v>46211.66080744213</v>
+      </c>
+      <c r="Q120" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
+      <c r="R120" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando definição gerencia departamento e gerencia operacional</t>
+        </is>
+      </c>
       <c r="S120" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -10471,51 +10483,51 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>79665</v>
+        <v>79930</v>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>Autoregularização - Simples Nacional - Janeiro a Dezembro 2024Cliente recebeu notificação de autoregularização do Simples Nacional referente período 2024. Por gentileza, providenciar retificação dentro do prazo estipulado pela Receita.</t>
+          <t>Por gentileza, poderiam providenciar Última declaração do IRPJ entregue do cliente CEREALISTA</t>
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>5100</v>
+        <v>5101</v>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
+          <t>CEREALISTA IDEAL DE SÃO CAETANO LTDA</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="I121" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J121" s="2" t="n">
-        <v>46176.49184155092</v>
+        <v>46184.70223510417</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>46199</v>
+        <v>46185</v>
       </c>
       <c r="L121" s="1" t="inlineStr">
         <is>
@@ -10524,24 +10536,22 @@
       </c>
       <c r="M121" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N121" s="2" t="n">
-        <v>46183.62114679398</v>
-      </c>
+          <t>Leticia Queiroz</t>
+        </is>
+      </c>
+      <c r="N121" s="1" t="n"/>
       <c r="O121" s="1" t="n"/>
       <c r="P121" s="2" t="n">
-        <v>46211.66080744213</v>
+        <v>46192.46905616898</v>
       </c>
       <c r="Q121" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="R121" s="1" t="inlineStr">
         <is>
-          <t>Aguardando definição gerencia departamento e gerencia operacional</t>
+          <t xml:space="preserve">Bom dia, não entendi, favor ser mais e especifica, seria memoria de cálculo ou alguma obrigação acessória como Sped????? </t>
         </is>
       </c>
       <c r="S121" s="1" t="inlineStr">
@@ -10552,57 +10562,57 @@
       <c r="T121" s="1" t="n"/>
       <c r="U121" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>79930</v>
+        <v>81857</v>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderiam providenciar Última declaração do IRPJ entregue do cliente CEREALISTA</t>
+          <t xml:space="preserve">Por gentileza, emitir a guia do DIFAL referente a  Notificação de Pendência Fiscal - ICMS DIFCON - Sefaz MS - CNPJ: 02.905.133/0001-32 -CABEXPRESS e enviar para cliente pagar copiando toda equipe da CABEX e o Sr. Reginaldo 'Reginaldo J Chagas' &lt;reginaldo@adviserempresarial.com.br&gt; </t>
         </is>
       </c>
       <c r="F122" s="1" t="n">
-        <v>5101</v>
+        <v>5132</v>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>CEREALISTA IDEAL DE SÃO CAETANO LTDA</t>
+          <t>CABEXPRESS INDUSTRIA E COMÉRCIO DE CABOS ELÉTRICOS LTDA</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I122" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J122" s="2" t="n">
-        <v>46184.70223510417</v>
+        <v>46238.64146678241</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>46185</v>
+        <v>46240</v>
       </c>
       <c r="L122" s="1" t="inlineStr">
         <is>
@@ -10611,22 +10621,24 @@
       </c>
       <c r="M122" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Simone Marques</t>
         </is>
       </c>
       <c r="N122" s="1" t="n"/>
-      <c r="O122" s="1" t="n"/>
+      <c r="O122" s="2" t="n">
+        <v>46241</v>
+      </c>
       <c r="P122" s="2" t="n">
-        <v>46192.46905616898</v>
+        <v>46238.74667160879</v>
       </c>
       <c r="Q122" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="R122" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, não entendi, favor ser mais e especifica, seria memoria de cálculo ou alguma obrigação acessória como Sped????? </t>
+          <t>Recalculo DIFAL enviado ao cliente no e-mail na data de hoje</t>
         </is>
       </c>
       <c r="S122" s="1" t="inlineStr">
@@ -10637,100 +10649,96 @@
       <c r="T122" s="1" t="n"/>
       <c r="U122" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>81857</v>
+        <v>82046</v>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, emitir a guia do DIFAL referente a  Notificação de Pendência Fiscal - ICMS DIFCON - Sefaz MS - CNPJ: 02.905.133/0001-32 -CABEXPRESS e enviar para cliente pagar copiando toda equipe da CABEX e o Sr. Reginaldo 'Reginaldo J Chagas' &lt;reginaldo@adviserempresarial.com.br&gt; </t>
+          <t>Por favor verificar - Transporte de saldo credor incorreto EFD 05, 09, 10, 11 e 12/2024. Não veio no material de reunião, por favor verificar esta pendência!</t>
         </is>
       </c>
       <c r="F123" s="1" t="n">
-        <v>5132</v>
+        <v>5142</v>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>CABEXPRESS INDUSTRIA E COMÉRCIO DE CABOS ELÉTRICOS LTDA</t>
+          <t>MERCADO, PADARIA ACOUGUE E RESTAURANTE OLIMPIA LTDA</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I123" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J123" s="2" t="n">
-        <v>46238.64146678241</v>
+        <v>46241.44565771991</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>46240</v>
+        <v>46248</v>
       </c>
       <c r="L123" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M123" s="1" t="inlineStr">
         <is>
-          <t>Simone Marques</t>
-        </is>
-      </c>
-      <c r="N123" s="1" t="n"/>
+          <t>Rodrigo Rego</t>
+        </is>
+      </c>
+      <c r="N123" s="2" t="n">
+        <v>46245.74680853009</v>
+      </c>
       <c r="O123" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="P123" s="2" t="n">
-        <v>46238.74667160879</v>
-      </c>
-      <c r="Q123" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+        <v>46288</v>
+      </c>
+      <c r="P123" s="1" t="n"/>
+      <c r="Q123" s="1" t="inlineStr"/>
       <c r="R123" s="1" t="inlineStr">
         <is>
-          <t>Recalculo DIFAL enviado ao cliente no e-mail na data de hoje</t>
+          <t xml:space="preserve">VERIFICANDO </t>
         </is>
       </c>
       <c r="S123" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T123" s="1" t="n"/>
       <c r="U123" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>82046</v>
+        <v>82044</v>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
@@ -10749,36 +10757,36 @@
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>Por favor verificar - Transporte de saldo credor incorreto EFD 05, 09, 10, 11 e 12/2024. Não veio no material de reunião, por favor verificar esta pendência!</t>
+          <t>"Empresa iniciou recebimentos de aluguel no mês 02/2026.Por gentileza, verificar nos extratos da empresa os recebimentos para fins de fechamento fiscal mensal (PIS/ COFINS) e fechamentos trimestrais (IRPJ/ CSLL).Por gentileza revisar os extratos da empresa para confirmação de não movimentação, visto que a empresa está realizando locações, como acima apontado. Por favor me retornar com a conclusão."</t>
         </is>
       </c>
       <c r="F124" s="1" t="n">
-        <v>5142</v>
+        <v>5145</v>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>MERCADO, PADARIA ACOUGUE E RESTAURANTE OLIMPIA LTDA</t>
+          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
       <c r="I124" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J124" s="2" t="n">
-        <v>46241.44565771991</v>
+        <v>46241.43949221065</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="L124" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M124" s="1" t="inlineStr">
@@ -10786,43 +10794,48 @@
           <t>Rodrigo Rego</t>
         </is>
       </c>
-      <c r="N124" s="2" t="n">
-        <v>46245.74680853009</v>
-      </c>
+      <c r="N124" s="1" t="n"/>
       <c r="O124" s="2" t="n">
-        <v>46288</v>
-      </c>
-      <c r="P124" s="1" t="n"/>
-      <c r="Q124" s="1" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="P124" s="2" t="n">
+        <v>46244.5917212963</v>
+      </c>
+      <c r="Q124" s="1" t="inlineStr">
+        <is>
+          <t>Lucas Fischer</t>
+        </is>
+      </c>
       <c r="R124" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFICANDO </t>
+          <t>Não identificamos recebimentos de aluguel nessa empresa.
+Precisamos de mais informações para procurar. Qual o nome do favorecido? quais são os valores? Foi recebido em qual banco?</t>
         </is>
       </c>
       <c r="S124" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T124" s="1" t="n"/>
       <c r="U124" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>82044</v>
+        <v>81298</v>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
@@ -10832,7 +10845,7 @@
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>"Empresa iniciou recebimentos de aluguel no mês 02/2026.Por gentileza, verificar nos extratos da empresa os recebimentos para fins de fechamento fiscal mensal (PIS/ COFINS) e fechamentos trimestrais (IRPJ/ CSLL).Por gentileza revisar os extratos da empresa para confirmação de não movimentação, visto que a empresa está realizando locações, como acima apontado. Por favor me retornar com a conclusão."</t>
+          <t>Por favor verificar com urgencia se na epoca foi enviado o debito que a receita esta notificando conforme anexo e enviar o DAS com o valor atualizado</t>
         </is>
       </c>
       <c r="F125" s="1" t="n">
@@ -10845,19 +10858,19 @@
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>Lucas Fischer</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I125" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J125" s="2" t="n">
-        <v>46241.43949221065</v>
+        <v>46225.48881790509</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>46248</v>
+        <v>46227</v>
       </c>
       <c r="L125" s="1" t="inlineStr">
         <is>
@@ -10869,22 +10882,23 @@
           <t>Rodrigo Rego</t>
         </is>
       </c>
-      <c r="N125" s="1" t="n"/>
+      <c r="N125" s="2" t="n">
+        <v>46230.71356496528</v>
+      </c>
       <c r="O125" s="2" t="n">
-        <v>46245</v>
+        <v>46285</v>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46244.5917212963</v>
+        <v>46287.75830049768</v>
       </c>
       <c r="Q125" s="1" t="inlineStr">
         <is>
-          <t>Lucas Fischer</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="R125" s="1" t="inlineStr">
         <is>
-          <t>Não identificamos recebimentos de aluguel nessa empresa.
-Precisamos de mais informações para procurar. Qual o nome do favorecido? quais são os valores? Foi recebido em qual banco?</t>
+          <t>verificando</t>
         </is>
       </c>
       <c r="S125" s="1" t="inlineStr">
@@ -10895,57 +10909,57 @@
       <c r="T125" s="1" t="n"/>
       <c r="U125" s="1" t="inlineStr">
         <is>
-          <t>Lucas Fischer</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>81298</v>
+        <v>79896</v>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>Por favor verificar com urgencia se na epoca foi enviado o debito que a receita esta notificando conforme anexo e enviar o DAS com o valor atualizado</t>
+          <t>Não estamos conseguindo dar continuidade ao assunto em cima do chamado 79551 -Favor emitir os DARFs de IRPJ e CSLL para atendimento ao Auto de Regularização da COXA -PRAZO PARA ATENDIMENTO 11.06.2026 (anexo). No e-mail (anexo) constam os valores originais dos débitos. O cliente está aguardando o os DARFs para efetuar o pagamento. Por gentileza, após a emissão, encaminhar os DARFs por e-mail  para gerencia de contas para que possamos enviá-los à Isadora, da COXA, visto que se trata de um ex-cliente e não será possível disponibilizar a documentação pelo SCI.  Solicitamos também que a ECF seja retificada ainda hoje,(11/06/2026), para que a Receita Federal tenha ciência de que o autorregularização foi atendido dentro do prazo estabelecido,(12/06/2026.)</t>
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>5145</v>
+        <v>5178</v>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA</t>
+          <t>COXA PARTICIPACOES S A</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="I126" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J126" s="2" t="n">
-        <v>46225.48881790509</v>
+        <v>46184.47763410879</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>46227</v>
+        <v>46188</v>
       </c>
       <c r="L126" s="1" t="inlineStr">
         <is>
@@ -10954,26 +10968,22 @@
       </c>
       <c r="M126" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
-        </is>
-      </c>
-      <c r="N126" s="2" t="n">
-        <v>46230.71356496528</v>
-      </c>
-      <c r="O126" s="2" t="n">
-        <v>46285</v>
-      </c>
+          <t>Simone Marques</t>
+        </is>
+      </c>
+      <c r="N126" s="1" t="n"/>
+      <c r="O126" s="1" t="n"/>
       <c r="P126" s="2" t="n">
-        <v>46287.75830049768</v>
+        <v>46240.68738668982</v>
       </c>
       <c r="Q126" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="R126" s="1" t="inlineStr">
         <is>
-          <t>verificando</t>
+          <t>DARFS e PERDCOMP CONCLUIDOS EM 15/06/2026 - ENVIADO POR E-MAIL</t>
         </is>
       </c>
       <c r="S126" s="1" t="inlineStr">
@@ -10984,22 +10994,22 @@
       <c r="T126" s="1" t="n"/>
       <c r="U126" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>79896</v>
+        <v>80417</v>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Reembolso</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Reembolso</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
@@ -11009,7 +11019,7 @@
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>Não estamos conseguindo dar continuidade ao assunto em cima do chamado 79551 -Favor emitir os DARFs de IRPJ e CSLL para atendimento ao Auto de Regularização da COXA -PRAZO PARA ATENDIMENTO 11.06.2026 (anexo). No e-mail (anexo) constam os valores originais dos débitos. O cliente está aguardando o os DARFs para efetuar o pagamento. Por gentileza, após a emissão, encaminhar os DARFs por e-mail  para gerencia de contas para que possamos enviá-los à Isadora, da COXA, visto que se trata de um ex-cliente e não será possível disponibilizar a documentação pelo SCI.  Solicitamos também que a ECF seja retificada ainda hoje,(11/06/2026), para que a Receita Federal tenha ciência de que o autorregularização foi atendido dentro do prazo estabelecido,(12/06/2026.)</t>
+          <t>O cliente está cobrando o reembolso no valor de R$ 15.748,98, referente aos juros e à multa dos DARFs pagos para atendimento da malha de débitos do 4º trimestre de 2023. Anexo comprovante de pagamento Dados bancários:Banco Itau (341)Ag: 8729CC: 99892-5CNPJ: 42.169.691/0001-00COXA PARTICIPAÇÕES S/A</t>
         </is>
       </c>
       <c r="F127" s="1" t="n">
@@ -11022,7 +11032,7 @@
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I127" s="1" t="inlineStr">
@@ -11031,10 +11041,10 @@
         </is>
       </c>
       <c r="J127" s="2" t="n">
-        <v>46184.47763410879</v>
+        <v>46195.6876917824</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>46188</v>
+        <v>46197</v>
       </c>
       <c r="L127" s="1" t="inlineStr">
         <is>
@@ -11049,16 +11059,17 @@
       <c r="N127" s="1" t="n"/>
       <c r="O127" s="1" t="n"/>
       <c r="P127" s="2" t="n">
-        <v>46240.68738668982</v>
+        <v>46204.40209097222</v>
       </c>
       <c r="Q127" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="R127" s="1" t="inlineStr">
         <is>
-          <t>DARFS e PERDCOMP CONCLUIDOS EM 15/06/2026 - ENVIADO POR E-MAIL</t>
+          <t>bom Dia, 
+Processo de reembolso realizado a entregue ao Andre Coelho no dia 01-07-2026</t>
         </is>
       </c>
       <c r="S127" s="1" t="inlineStr">
@@ -11067,24 +11078,20 @@
         </is>
       </c>
       <c r="T127" s="1" t="n"/>
-      <c r="U127" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+      <c r="U127" s="1" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>80417</v>
+        <v>81016</v>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Reembolso</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>Reembolso</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
@@ -11094,32 +11101,32 @@
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>O cliente está cobrando o reembolso no valor de R$ 15.748,98, referente aos juros e à multa dos DARFs pagos para atendimento da malha de débitos do 4º trimestre de 2023. Anexo comprovante de pagamento Dados bancários:Banco Itau (341)Ag: 8729CC: 99892-5CNPJ: 42.169.691/0001-00COXA PARTICIPAÇÕES S/A</t>
+          <t>Prezados, O cliente Marajoara disponibilizou novos arquivos no FTP correspondentes aos meses de abril, maio e junho 2026 para reapuração das entradas/ saídas do período.De acordo com o cliente, os arquivos speds enviados na época não estavam considerando todas as notas fiscais do período.</t>
         </is>
       </c>
       <c r="F128" s="1" t="n">
-        <v>5178</v>
+        <v>5253</v>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>COXA PARTICIPACOES S A</t>
+          <t>MARAJOARA II COMÉRCIO VAREJISTA DE CARNES, LANCHES E BEBIDAS LTDA</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I128" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J128" s="2" t="n">
-        <v>46195.6876917824</v>
+        <v>46217.42263804398</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>46197</v>
+        <v>46224</v>
       </c>
       <c r="L128" s="1" t="inlineStr">
         <is>
@@ -11128,23 +11135,24 @@
       </c>
       <c r="M128" s="1" t="inlineStr">
         <is>
-          <t>Simone Marques</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N128" s="1" t="n"/>
-      <c r="O128" s="1" t="n"/>
+      <c r="O128" s="2" t="n">
+        <v>46233</v>
+      </c>
       <c r="P128" s="2" t="n">
-        <v>46204.40209097222</v>
+        <v>46234.38291929398</v>
       </c>
       <c r="Q128" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="R128" s="1" t="inlineStr">
         <is>
-          <t>bom Dia, 
-Processo de reembolso realizado a entregue ao Andre Coelho no dia 01-07-2026</t>
+          <t>Conforme conversamos precisamos de um novo SPED contendo as notas faltantes ou somente os XMLs faltantes.</t>
         </is>
       </c>
       <c r="S128" s="1" t="inlineStr">
@@ -11153,20 +11161,24 @@
         </is>
       </c>
       <c r="T128" s="1" t="n"/>
-      <c r="U128" s="1" t="inlineStr"/>
+      <c r="U128" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>81016</v>
+        <v>79674</v>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
@@ -11176,32 +11188,32 @@
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>Prezados, O cliente Marajoara disponibilizou novos arquivos no FTP correspondentes aos meses de abril, maio e junho 2026 para reapuração das entradas/ saídas do período.De acordo com o cliente, os arquivos speds enviados na época não estavam considerando todas as notas fiscais do período.</t>
+          <t>Favor retificar DCTF do período de MAIO/2025. Os valores de PIS e COFINS estão divergentes da apuração que consta no sistema de análise.</t>
         </is>
       </c>
       <c r="F129" s="1" t="n">
-        <v>5253</v>
+        <v>5331</v>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>MARAJOARA II COMÉRCIO VAREJISTA DE CARNES, LANCHES E BEBIDAS LTDA</t>
+          <t>PIRANA - AUTO SERVIÇO LTDA</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Danielle Silva</t>
         </is>
       </c>
       <c r="I129" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J129" s="2" t="n">
-        <v>46217.42263804398</v>
+        <v>46176.62133761574</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>46224</v>
+        <v>46191</v>
       </c>
       <c r="L129" s="1" t="inlineStr">
         <is>
@@ -11214,20 +11226,18 @@
         </is>
       </c>
       <c r="N129" s="1" t="n"/>
-      <c r="O129" s="2" t="n">
-        <v>46233</v>
-      </c>
+      <c r="O129" s="1" t="n"/>
       <c r="P129" s="2" t="n">
-        <v>46234.38291929398</v>
+        <v>46181.60648179398</v>
       </c>
       <c r="Q129" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Danielle Silva</t>
         </is>
       </c>
       <c r="R129" s="1" t="inlineStr">
         <is>
-          <t>Conforme conversamos precisamos de um novo SPED contendo as notas faltantes ou somente os XMLs faltantes.</t>
+          <t>Valores retificados na DCTFWEB em 08/06/2026.</t>
         </is>
       </c>
       <c r="S129" s="1" t="inlineStr">
@@ -11238,22 +11248,22 @@
       <c r="T129" s="1" t="n"/>
       <c r="U129" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Karina Fonseca</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>79674</v>
+        <v>79877</v>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
@@ -11263,7 +11273,7 @@
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>Favor retificar DCTF do período de MAIO/2025. Os valores de PIS e COFINS estão divergentes da apuração que consta no sistema de análise.</t>
+          <t>Por gentileza, providenciar regularização de transporte de saldo credor incorreto, conforme ocorrência no posto fiscal.</t>
         </is>
       </c>
       <c r="F130" s="1" t="n">
@@ -11276,23 +11286,23 @@
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>Danielle Silva</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I130" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J130" s="2" t="n">
-        <v>46176.62133761574</v>
+        <v>46183.73675975695</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>46191</v>
+        <v>46199</v>
       </c>
       <c r="L130" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M130" s="1" t="inlineStr">
@@ -11300,45 +11310,43 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N130" s="1" t="n"/>
-      <c r="O130" s="1" t="n"/>
-      <c r="P130" s="2" t="n">
-        <v>46181.60648179398</v>
-      </c>
-      <c r="Q130" s="1" t="inlineStr">
-        <is>
-          <t>Danielle Silva</t>
-        </is>
-      </c>
+      <c r="N130" s="2" t="n">
+        <v>46189.6799341088</v>
+      </c>
+      <c r="O130" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="P130" s="1" t="n"/>
+      <c r="Q130" s="1" t="inlineStr"/>
       <c r="R130" s="1" t="inlineStr">
         <is>
-          <t>Valores retificados na DCTFWEB em 08/06/2026.</t>
+          <t>Verificando.</t>
         </is>
       </c>
       <c r="S130" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T130" s="1" t="n"/>
       <c r="U130" s="1" t="inlineStr">
         <is>
-          <t>Karina Fonseca</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>79877</v>
+        <v>82725</v>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>SPED</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>SPED</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
@@ -11348,7 +11356,7 @@
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar regularização de transporte de saldo credor incorreto, conforme ocorrência no posto fiscal.</t>
+          <t>Conforme autorização da diretoria, por gentileza, incluir crédito no valor de R$50.132,65 na apuração de julho 2026.Documento de aprovação anexo.</t>
         </is>
       </c>
       <c r="F131" s="1" t="n">
@@ -11370,14 +11378,14 @@
         </is>
       </c>
       <c r="J131" s="2" t="n">
-        <v>46183.73675975695</v>
+        <v>46254.44089421296</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>46199</v>
+        <v>46255</v>
       </c>
       <c r="L131" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M131" s="1" t="inlineStr">
@@ -11385,22 +11393,24 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N131" s="2" t="n">
-        <v>46189.6799341088</v>
-      </c>
-      <c r="O131" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="P131" s="1" t="n"/>
-      <c r="Q131" s="1" t="inlineStr"/>
+      <c r="N131" s="1" t="n"/>
+      <c r="O131" s="1" t="n"/>
+      <c r="P131" s="2" t="n">
+        <v>46254.68301747685</v>
+      </c>
+      <c r="Q131" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
       <c r="R131" s="1" t="inlineStr">
         <is>
-          <t>Verificando.</t>
+          <t>Credito lançado,  novo imposto publicado!</t>
         </is>
       </c>
       <c r="S131" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T131" s="1" t="n"/>
@@ -11412,16 +11422,16 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>82725</v>
+        <v>80737</v>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>SPED</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>SPED</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
@@ -11431,20 +11441,20 @@
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>Conforme autorização da diretoria, por gentileza, incluir crédito no valor de R$50.132,65 na apuração de julho 2026.Documento de aprovação anexo.</t>
+          <t>Prezados,Cliente 5350-Akafer Materiais Elétricos recebeu Auto de regularização referente GIA/EFD dos períodos 07/2024 a 12/2024 totalizando R$126.900,69.Por gentileza, providenciar regularização dentro do prazo estipulado que encerra-se em 31/07/2026.</t>
         </is>
       </c>
       <c r="F132" s="1" t="n">
-        <v>5331</v>
+        <v>5350</v>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>PIRANA - AUTO SERVIÇO LTDA</t>
+          <t>AKAFER MATERIAIS ELETRICOS LTDA</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="I132" s="1" t="inlineStr">
@@ -11453,10 +11463,10 @@
         </is>
       </c>
       <c r="J132" s="2" t="n">
-        <v>46254.44089421296</v>
+        <v>46206.7217474537</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>46255</v>
+        <v>46213</v>
       </c>
       <c r="L132" s="1" t="inlineStr">
         <is>
@@ -11471,16 +11481,17 @@
       <c r="N132" s="1" t="n"/>
       <c r="O132" s="1" t="n"/>
       <c r="P132" s="2" t="n">
-        <v>46254.68301747685</v>
+        <v>46209.50008553241</v>
       </c>
       <c r="Q132" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="R132" s="1" t="inlineStr">
         <is>
-          <t>Credito lançado,  novo imposto publicado!</t>
+          <t>Bom dia,
+Empresa pertence ao MG express, por gentileza direcionar ao Romero/ Helmer.</t>
         </is>
       </c>
       <c r="S132" s="1" t="inlineStr">
@@ -11489,24 +11500,20 @@
         </is>
       </c>
       <c r="T132" s="1" t="n"/>
-      <c r="U132" s="1" t="inlineStr">
-        <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
+      <c r="U132" s="1" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>80737</v>
+        <v>81703</v>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
@@ -11516,32 +11523,32 @@
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>Prezados,Cliente 5350-Akafer Materiais Elétricos recebeu Auto de regularização referente GIA/EFD dos períodos 07/2024 a 12/2024 totalizando R$126.900,69.Por gentileza, providenciar regularização dentro do prazo estipulado que encerra-se em 31/07/2026.</t>
+          <t>Bom dia, Por gentileza verificar mensagem recebida em nossa caixa referente a omissão, inconsistência ou omissão na Escritura fiscal Digital (EFD) ou em uma Dapi de período anterior.</t>
         </is>
       </c>
       <c r="F133" s="1" t="n">
-        <v>5350</v>
+        <v>5442</v>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>AKAFER MATERIAIS ELETRICOS LTDA</t>
+          <t>G13 IMPORTACAO E EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>Idna Sousa</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I133" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J133" s="2" t="n">
-        <v>46206.7217474537</v>
+        <v>46234.47681732639</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>46213</v>
+        <v>46237</v>
       </c>
       <c r="L133" s="1" t="inlineStr">
         <is>
@@ -11550,23 +11557,26 @@
       </c>
       <c r="M133" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N133" s="1" t="n"/>
-      <c r="O133" s="1" t="n"/>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N133" s="2" t="n">
+        <v>46238.74622743056</v>
+      </c>
+      <c r="O133" s="2" t="n">
+        <v>46255</v>
+      </c>
       <c r="P133" s="2" t="n">
-        <v>46209.50008553241</v>
+        <v>46286.59377850695</v>
       </c>
       <c r="Q133" s="1" t="inlineStr">
         <is>
-          <t>Idna Sousa</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="R133" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,
-Empresa pertence ao MG express, por gentileza direcionar ao Romero/ Helmer.</t>
+          <t>Analisando</t>
         </is>
       </c>
       <c r="S133" s="1" t="inlineStr">
@@ -11575,20 +11585,24 @@
         </is>
       </c>
       <c r="T133" s="1" t="n"/>
-      <c r="U133" s="1" t="inlineStr"/>
+      <c r="U133" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>81703</v>
+        <v>82955</v>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
@@ -11598,7 +11612,7 @@
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, Por gentileza verificar mensagem recebida em nossa caixa referente a omissão, inconsistência ou omissão na Escritura fiscal Digital (EFD) ou em uma Dapi de período anterior.</t>
+          <t>Bom dia, por gentileza verificar omissão de DAPI</t>
         </is>
       </c>
       <c r="F134" s="1" t="n">
@@ -11611,7 +11625,7 @@
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I134" s="1" t="inlineStr">
@@ -11620,10 +11634,10 @@
         </is>
       </c>
       <c r="J134" s="2" t="n">
-        <v>46234.47681732639</v>
+        <v>46259.46279479167</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>46237</v>
+        <v>46261</v>
       </c>
       <c r="L134" s="1" t="inlineStr">
         <is>
@@ -11636,22 +11650,22 @@
         </is>
       </c>
       <c r="N134" s="2" t="n">
-        <v>46238.74622743056</v>
+        <v>46260.75763707176</v>
       </c>
       <c r="O134" s="2" t="n">
-        <v>46255</v>
+        <v>46269</v>
       </c>
       <c r="P134" s="2" t="n">
-        <v>46286.59377850695</v>
+        <v>46269.47718869213</v>
       </c>
       <c r="Q134" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="R134" s="1" t="inlineStr">
         <is>
-          <t>Analisando</t>
+          <t>operação realizando atendimento</t>
         </is>
       </c>
       <c r="S134" s="1" t="inlineStr">
@@ -11660,24 +11674,20 @@
         </is>
       </c>
       <c r="T134" s="1" t="n"/>
-      <c r="U134" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+      <c r="U134" s="1" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>82955</v>
+        <v>84145</v>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
@@ -11687,32 +11697,32 @@
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza verificar omissão de DAPI</t>
+          <t>Bom dia, por gentileza encaminhar a documentação abaixo:  1. Balancetes mensais do ano corrente (janeiro até o último mês fechado);2. Relatório de receitas e despesas (DRE ou planilha equivalente) dos últimos 12</t>
         </is>
       </c>
       <c r="F135" s="1" t="n">
-        <v>5442</v>
+        <v>5472</v>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>G13 IMPORTACAO E EXPORTACAO LTDA</t>
+          <t>T C DE CASTRO EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="I135" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J135" s="2" t="n">
-        <v>46259.46279479167</v>
+        <v>46283.40513741898</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>46261</v>
+        <v>46286</v>
       </c>
       <c r="L135" s="1" t="inlineStr">
         <is>
@@ -11725,22 +11735,22 @@
         </is>
       </c>
       <c r="N135" s="2" t="n">
-        <v>46260.75763707176</v>
+        <v>46286.65661658565</v>
       </c>
       <c r="O135" s="2" t="n">
-        <v>46269</v>
+        <v>46287</v>
       </c>
       <c r="P135" s="2" t="n">
-        <v>46269.47718869213</v>
+        <v>46287.75436478009</v>
       </c>
       <c r="Q135" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="R135" s="1" t="inlineStr">
         <is>
-          <t>operação realizando atendimento</t>
+          <t>Boa tarde, Segue documentação solicitada.</t>
         </is>
       </c>
       <c r="S135" s="1" t="inlineStr">
@@ -11749,20 +11759,24 @@
         </is>
       </c>
       <c r="T135" s="1" t="n"/>
-      <c r="U135" s="1" t="inlineStr"/>
+      <c r="U135" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>84145</v>
+        <v>80685</v>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
@@ -11772,36 +11786,36 @@
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza encaminhar a documentação abaixo:  1. Balancetes mensais do ano corrente (janeiro até o último mês fechado);2. Relatório de receitas e despesas (DRE ou planilha equivalente) dos últimos 12</t>
+          <t>Boa tarde, por gentileza verificar mensagem recebida em nossa caixa referente o Sistema de conformidade. ATENÇÃO: A autorregularização deve ser feita até 14/08/2026. Após essa data, o contribuinte está sujeito à abertura de operação fiscal para apuração e constituição de eventuais créditos tributários relacionados.</t>
         </is>
       </c>
       <c r="F136" s="1" t="n">
-        <v>5472</v>
+        <v>5587</v>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>T C DE CASTRO EMPREENDIMENTOS LTDA</t>
+          <t>DALMEC SISTEMAS DE PONTO E ACESSO LTDA</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I136" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J136" s="2" t="n">
-        <v>46283.40513741898</v>
+        <v>46204.62099849537</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>46286</v>
+        <v>46206</v>
       </c>
       <c r="L136" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M136" s="1" t="inlineStr">
@@ -11809,40 +11823,33 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N136" s="2" t="n">
-        <v>46286.65661658565</v>
-      </c>
+      <c r="N136" s="1" t="n"/>
       <c r="O136" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="P136" s="2" t="n">
-        <v>46287.75436478009</v>
-      </c>
-      <c r="Q136" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
+        <v>46233</v>
+      </c>
+      <c r="P136" s="1" t="n"/>
+      <c r="Q136" s="1" t="inlineStr"/>
       <c r="R136" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Segue documentação solicitada.</t>
+          <t>TAREFA SENDO EXECUTADA PELA OPERAÇÃO, 
+PRAZO 31/07</t>
         </is>
       </c>
       <c r="S136" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T136" s="1" t="n"/>
-      <c r="U136" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T136" s="1" t="inlineStr">
+        <is>
+          <t>EF - INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="U136" s="1" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>80685</v>
+        <v>79664</v>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
@@ -11861,79 +11868,84 @@
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza verificar mensagem recebida em nossa caixa referente o Sistema de conformidade. ATENÇÃO: A autorregularização deve ser feita até 14/08/2026. Após essa data, o contribuinte está sujeito à abertura de operação fiscal para apuração e constituição de eventuais créditos tributários relacionados.</t>
+          <t>Autoregularização  Simples Nacional - Janeiro a Dezembro 2024.Cliente recebeu notificação de auto regularização referente período mencionado acima. Por gentileza, providenciar dentro do prazo estipulado pela Receita.</t>
         </is>
       </c>
       <c r="F137" s="1" t="n">
-        <v>5587</v>
+        <v>5595</v>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>DALMEC SISTEMAS DE PONTO E ACESSO LTDA</t>
+          <t>SUPERMERCADO QUEIROZ LTDA</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I137" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J137" s="2" t="n">
-        <v>46204.62099849537</v>
+        <v>46176.46938182871</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>46206</v>
+        <v>46199</v>
       </c>
       <c r="L137" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M137" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
-        </is>
-      </c>
-      <c r="N137" s="1" t="n"/>
-      <c r="O137" s="2" t="n">
-        <v>46233</v>
-      </c>
-      <c r="P137" s="1" t="n"/>
-      <c r="Q137" s="1" t="inlineStr"/>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N137" s="2" t="n">
+        <v>46183.62132037037</v>
+      </c>
+      <c r="O137" s="1" t="n"/>
+      <c r="P137" s="2" t="n">
+        <v>46210.54752037037</v>
+      </c>
+      <c r="Q137" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
       <c r="R137" s="1" t="inlineStr">
         <is>
-          <t>TAREFA SENDO EXECUTADA PELA OPERAÇÃO, 
-PRAZO 31/07</t>
+          <t>Aguardando definição gerencia departamento e gerencia operacional</t>
         </is>
       </c>
       <c r="S137" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T137" s="1" t="inlineStr">
-        <is>
-          <t>EF - INDUSTRIA</t>
-        </is>
-      </c>
-      <c r="U137" s="1" t="inlineStr"/>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T137" s="1" t="n"/>
+      <c r="U137" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>79664</v>
+        <v>79916</v>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
@@ -11943,7 +11955,7 @@
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>Autoregularização  Simples Nacional - Janeiro a Dezembro 2024.Cliente recebeu notificação de auto regularização referente período mencionado acima. Por gentileza, providenciar dentro do prazo estipulado pela Receita.</t>
+          <t>Verificar Omissão de DCTF (Período de Apuração) 2024 - OUT NOV DEZ</t>
         </is>
       </c>
       <c r="F138" s="1" t="n">
@@ -11956,7 +11968,7 @@
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I138" s="1" t="inlineStr">
@@ -11965,10 +11977,10 @@
         </is>
       </c>
       <c r="J138" s="2" t="n">
-        <v>46176.46938182871</v>
+        <v>46184.59114753472</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>46199</v>
+        <v>46192</v>
       </c>
       <c r="L138" s="1" t="inlineStr">
         <is>
@@ -11980,21 +11992,19 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N138" s="2" t="n">
-        <v>46183.62132037037</v>
-      </c>
+      <c r="N138" s="1" t="n"/>
       <c r="O138" s="1" t="n"/>
       <c r="P138" s="2" t="n">
-        <v>46210.54752037037</v>
+        <v>46191.43697144676</v>
       </c>
       <c r="Q138" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="R138" s="1" t="inlineStr">
         <is>
-          <t>Aguardando definição gerencia departamento e gerencia operacional</t>
+          <t>Por favor, verificar com o contabil.</t>
         </is>
       </c>
       <c r="S138" s="1" t="inlineStr">
@@ -12005,22 +12015,22 @@
       <c r="T138" s="1" t="n"/>
       <c r="U138" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>79916</v>
+        <v>83300</v>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
@@ -12030,7 +12040,7 @@
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>Verificar Omissão de DCTF (Período de Apuração) 2024 - OUT NOV DEZ</t>
+          <t>Por gentileza, providenciar regularização de transporte de saldo credor incorreto 08 e 09/2025 conforme situação do contribuinte anexo.</t>
         </is>
       </c>
       <c r="F139" s="1" t="n">
@@ -12043,7 +12053,7 @@
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="I139" s="1" t="inlineStr">
@@ -12052,10 +12062,10 @@
         </is>
       </c>
       <c r="J139" s="2" t="n">
-        <v>46184.59114753472</v>
+        <v>46265.73964244213</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>46192</v>
+        <v>46276</v>
       </c>
       <c r="L139" s="1" t="inlineStr">
         <is>
@@ -12070,99 +12080,14 @@
       <c r="N139" s="1" t="n"/>
       <c r="O139" s="1" t="n"/>
       <c r="P139" s="2" t="n">
-        <v>46191.43697144676</v>
+        <v>46280.4460440625</v>
       </c>
       <c r="Q139" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="R139" s="1" t="inlineStr">
-        <is>
-          <t>Por favor, verificar com o contabil.</t>
-        </is>
-      </c>
-      <c r="S139" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T139" s="1" t="n"/>
-      <c r="U139" s="1" t="inlineStr">
-        <is>
-          <t>Thaiza Oliveira</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="1" t="n">
-        <v>83300</v>
-      </c>
-      <c r="B140" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Credor Incorreto</t>
-        </is>
-      </c>
-      <c r="C140" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Credor Incorreto</t>
-        </is>
-      </c>
-      <c r="D140" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E140" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, providenciar regularização de transporte de saldo credor incorreto 08 e 09/2025 conforme situação do contribuinte anexo.</t>
-        </is>
-      </c>
-      <c r="F140" s="1" t="n">
-        <v>5595</v>
-      </c>
-      <c r="G140" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO QUEIROZ LTDA</t>
-        </is>
-      </c>
-      <c r="H140" s="1" t="inlineStr">
-        <is>
-          <t>Idna Sousa</t>
-        </is>
-      </c>
-      <c r="I140" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J140" s="2" t="n">
-        <v>46265.73964244213</v>
-      </c>
-      <c r="K140" s="2" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L140" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M140" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N140" s="1" t="n"/>
-      <c r="O140" s="1" t="n"/>
-      <c r="P140" s="2" t="n">
-        <v>46280.4460440625</v>
-      </c>
-      <c r="Q140" s="1" t="inlineStr">
-        <is>
-          <t>Idna Sousa</t>
-        </is>
-      </c>
-      <c r="R140" s="1" t="inlineStr">
         <is>
           <t>Bom dia,
 Mes 07/2025 não recebemos o sped icms para validação.
@@ -12170,26 +12095,111 @@
 Por gentileza providenciar os arquivos para que o EFV possa validar e fazer as devidas retificações.</t>
         </is>
       </c>
+      <c r="S139" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T139" s="1" t="n"/>
+      <c r="U139" s="1" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>79914</v>
+      </c>
+      <c r="B140" s="1" t="inlineStr">
+        <is>
+          <t>Omissão de Obrigações Acessórias</t>
+        </is>
+      </c>
+      <c r="C140" s="1" t="inlineStr">
+        <is>
+          <t>Omissão de Obrigações Acessórias</t>
+        </is>
+      </c>
+      <c r="D140" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E140" s="1" t="inlineStr">
+        <is>
+          <t>Verificar Omissão de Omissão de DIRF (Ano de Retenção) 2023</t>
+        </is>
+      </c>
+      <c r="F140" s="1" t="n">
+        <v>5596</v>
+      </c>
+      <c r="G140" s="1" t="inlineStr">
+        <is>
+          <t>SILVESTRE MERCADO E PADARIA LTDA</t>
+        </is>
+      </c>
+      <c r="H140" s="1" t="inlineStr">
+        <is>
+          <t>Larice Souza</t>
+        </is>
+      </c>
+      <c r="I140" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="n">
+        <v>46184.58962711805</v>
+      </c>
+      <c r="K140" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="L140" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M140" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N140" s="1" t="n"/>
+      <c r="O140" s="1" t="n"/>
+      <c r="P140" s="2" t="n">
+        <v>46188.70596524305</v>
+      </c>
+      <c r="Q140" s="1" t="inlineStr">
+        <is>
+          <t>Larice Souza</t>
+        </is>
+      </c>
+      <c r="R140" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde. Por favor direcionar o chamado ao departamento contábil qual é o  responsavel pela entrega da DIRF, </t>
+        </is>
+      </c>
       <c r="S140" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
       <c r="T140" s="1" t="n"/>
-      <c r="U140" s="1" t="inlineStr"/>
+      <c r="U140" s="1" t="inlineStr">
+        <is>
+          <t>Larice Souza</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>79914</v>
+        <v>79915</v>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
@@ -12199,7 +12209,7 @@
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>Verificar Omissão de Omissão de DIRF (Ano de Retenção) 2023</t>
+          <t>Verificar EFD Transporte de Saldo Credor Incorreto ref. 08/2025 e 09/2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="n">
@@ -12221,10 +12231,10 @@
         </is>
       </c>
       <c r="J141" s="2" t="n">
-        <v>46184.58962711805</v>
+        <v>46184.59060590278</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="L141" s="1" t="inlineStr">
         <is>
@@ -12239,7 +12249,7 @@
       <c r="N141" s="1" t="n"/>
       <c r="O141" s="1" t="n"/>
       <c r="P141" s="2" t="n">
-        <v>46188.70596524305</v>
+        <v>46188.71399788195</v>
       </c>
       <c r="Q141" s="1" t="inlineStr">
         <is>
@@ -12248,7 +12258,7 @@
       </c>
       <c r="R141" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde. Por favor direcionar o chamado ao departamento contábil qual é o  responsavel pela entrega da DIRF, </t>
+          <t>Por gentileza, verificar solicitação. Loja 5596 optante pelo simples nacional.</t>
         </is>
       </c>
       <c r="S141" s="1" t="inlineStr">
@@ -12265,92 +12275,90 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>79915</v>
+        <v>83696</v>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Levantamento Divergências</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t xml:space="preserve">Levantar Divergencias </t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>Verificar EFD Transporte de Saldo Credor Incorreto ref. 08/2025 e 09/2025</t>
+          <t>Bom dia,  A empresa 5598 - Distribuidor de Morangos tem o pró-labore registrado em nome de Thais Kazi de Menezes, porém o sócio é Fabio Pereira da CostaPor favor, verificar.Agradeço</t>
         </is>
       </c>
       <c r="F142" s="1" t="n">
-        <v>5596</v>
+        <v>5598</v>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>SILVESTRE MERCADO E PADARIA LTDA</t>
+          <t>DISTRIBUIDOR DE MORANGOS LTDA</t>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
         <is>
-          <t>Larice Souza</t>
+          <t>Vitor Guedes</t>
         </is>
       </c>
       <c r="I142" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J142" s="2" t="n">
-        <v>46184.59060590278</v>
+        <v>46274.38345836806</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>46192</v>
+        <v>46276</v>
       </c>
       <c r="L142" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M142" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N142" s="1" t="n"/>
-      <c r="O142" s="1" t="n"/>
-      <c r="P142" s="2" t="n">
-        <v>46188.71399788195</v>
-      </c>
-      <c r="Q142" s="1" t="inlineStr">
-        <is>
-          <t>Larice Souza</t>
-        </is>
-      </c>
+          <t>Fatima Rocha</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="n">
+        <v>46275.46922966436</v>
+      </c>
+      <c r="O142" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="P142" s="1" t="n"/>
+      <c r="Q142" s="1" t="inlineStr"/>
       <c r="R142" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, verificar solicitação. Loja 5596 optante pelo simples nacional.</t>
+          <t>Realizando os ajustes.</t>
         </is>
       </c>
       <c r="S142" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T142" s="1" t="n"/>
       <c r="U142" s="1" t="inlineStr">
         <is>
-          <t>Larice Souza</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>83696</v>
+        <v>83697</v>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
@@ -12369,15 +12377,15 @@
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,  A empresa 5598 - Distribuidor de Morangos tem o pró-labore registrado em nome de Thais Kazi de Menezes, porém o sócio é Fabio Pereira da CostaPor favor, verificar.Agradeço</t>
+          <t>Bom dia,  A empresa 5599 - Sweet Berry tem o pró-labore registrado em nome de Fábio Pereira da Costa, porém a sócia é Thais Kazi de Menezes. Por favor, verificar.Agradeço</t>
         </is>
       </c>
       <c r="F143" s="1" t="n">
-        <v>5598</v>
+        <v>5599</v>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDOR DE MORANGOS LTDA</t>
+          <t>SWEET BERRY COMERCIO DE FRUTAS LTDA</t>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
@@ -12391,7 +12399,7 @@
         </is>
       </c>
       <c r="J143" s="2" t="n">
-        <v>46274.38345836806</v>
+        <v>46274.38682858797</v>
       </c>
       <c r="K143" s="2" t="n">
         <v>46276</v>
@@ -12407,7 +12415,7 @@
         </is>
       </c>
       <c r="N143" s="2" t="n">
-        <v>46275.46922966436</v>
+        <v>46275.46928533565</v>
       </c>
       <c r="O143" s="2" t="n">
         <v>46286</v>
@@ -12433,99 +12441,103 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>83697</v>
+        <v>83983</v>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>Levantamento Divergências</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Levantar Divergencias </t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,  A empresa 5599 - Sweet Berry tem o pró-labore registrado em nome de Fábio Pereira da Costa, porém a sócia é Thais Kazi de Menezes. Por favor, verificar.Agradeço</t>
+          <t xml:space="preserve">Prezados, boa tarde!Tudo bem?O cliente solicitou o Balanço Patrimonial, balancete e a DRE referentes ao exercício de 2026 até o mês 06/2026Fico no aguardo do envio dos documentos para que possamos encaminhá-los ao cliente.Desde já, agradeço pela atenção </t>
         </is>
       </c>
       <c r="F144" s="1" t="n">
-        <v>5599</v>
+        <v>5617</v>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>SWEET BERRY COMERCIO DE FRUTAS LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
         <is>
-          <t>Vitor Guedes</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="I144" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J144" s="2" t="n">
-        <v>46274.38682858797</v>
+        <v>46280.40219806713</v>
       </c>
       <c r="K144" s="2" t="n">
-        <v>46276</v>
+        <v>46281</v>
       </c>
       <c r="L144" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M144" s="1" t="inlineStr">
         <is>
-          <t>Fatima Rocha</t>
-        </is>
-      </c>
-      <c r="N144" s="2" t="n">
-        <v>46275.46928533565</v>
-      </c>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N144" s="1" t="n"/>
       <c r="O144" s="2" t="n">
-        <v>46286</v>
-      </c>
-      <c r="P144" s="1" t="n"/>
-      <c r="Q144" s="1" t="inlineStr"/>
+        <v>46283</v>
+      </c>
+      <c r="P144" s="2" t="n">
+        <v>46283.45726087963</v>
+      </c>
+      <c r="Q144" s="1" t="inlineStr">
+        <is>
+          <t>Jackson Silva</t>
+        </is>
+      </c>
       <c r="R144" s="1" t="inlineStr">
         <is>
-          <t>Realizando os ajustes.</t>
+          <t>Segue relatórios como solicitados.</t>
         </is>
       </c>
       <c r="S144" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T144" s="1" t="n"/>
       <c r="U144" s="1" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>83983</v>
+        <v>83861</v>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
@@ -12535,32 +12547,32 @@
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, boa tarde!Tudo bem?O cliente solicitou o Balanço Patrimonial, balancete e a DRE referentes ao exercício de 2026 até o mês 06/2026Fico no aguardo do envio dos documentos para que possamos encaminhá-los ao cliente.Desde já, agradeço pela atenção </t>
+          <t>Boa tarde!!Por gentileza, verificar o saldo credor incorreto.</t>
         </is>
       </c>
       <c r="F145" s="1" t="n">
-        <v>5617</v>
+        <v>5650</v>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>RICHETTI COMERCIO DE BEBIDAS E ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I145" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J145" s="2" t="n">
-        <v>46280.40219806713</v>
+        <v>46276.62149768518</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="L145" s="1" t="inlineStr">
         <is>
@@ -12569,24 +12581,23 @@
       </c>
       <c r="M145" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N145" s="1" t="n"/>
-      <c r="O145" s="2" t="n">
-        <v>46283</v>
-      </c>
+      <c r="O145" s="1" t="n"/>
       <c r="P145" s="2" t="n">
-        <v>46283.45726087963</v>
+        <v>46280.51998788195</v>
       </c>
       <c r="Q145" s="1" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="R145" s="1" t="inlineStr">
         <is>
-          <t>Segue relatórios como solicitados.</t>
+          <t>Boa tarde,
+Para regularizar, precisamos retificar os períodos, entretanto, o cliente não paga taxa eletrônica. Por favor, verificar com o cliente sobre o pagamento da taxa.</t>
         </is>
       </c>
       <c r="S145" s="1" t="inlineStr">
@@ -12597,32 +12608,32 @@
       <c r="T145" s="1" t="n"/>
       <c r="U145" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>83861</v>
+        <v>83989</v>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!!Por gentileza, verificar o saldo credor incorreto.</t>
+          <t>Encaminho autorregularização da loja com prazo para conclusão 18/09/2026</t>
         </is>
       </c>
       <c r="F146" s="1" t="n">
@@ -12644,40 +12655,31 @@
         </is>
       </c>
       <c r="J146" s="2" t="n">
-        <v>46276.62149768518</v>
+        <v>46280.4334184375</v>
       </c>
       <c r="K146" s="2" t="n">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="L146" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M146" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N146" s="1" t="n"/>
-      <c r="O146" s="1" t="n"/>
-      <c r="P146" s="2" t="n">
-        <v>46280.51998788195</v>
-      </c>
-      <c r="Q146" s="1" t="inlineStr">
-        <is>
-          <t>Thaiza Oliveira</t>
-        </is>
-      </c>
-      <c r="R146" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde,
-Para regularizar, precisamos retificar os períodos, entretanto, o cliente não paga taxa eletrônica. Por favor, verificar com o cliente sobre o pagamento da taxa.</t>
-        </is>
-      </c>
+      <c r="O146" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="P146" s="1" t="n"/>
+      <c r="Q146" s="1" t="inlineStr"/>
+      <c r="R146" s="1" t="inlineStr"/>
       <c r="S146" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T146" s="1" t="n"/>
@@ -12689,16 +12691,16 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>83989</v>
+        <v>80617</v>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
@@ -12708,74 +12710,84 @@
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>Encaminho autorregularização da loja com prazo para conclusão 18/09/2026</t>
+          <t>Consta saldo residual IRRF nos períodos de 05/2025 e 01/2026.Por gentileza, verificar se os débitos são devidos ou se a DCTF do período deve ser retificada.</t>
         </is>
       </c>
       <c r="F147" s="1" t="n">
-        <v>5650</v>
+        <v>5666</v>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>RICHETTI COMERCIO DE BEBIDAS E ALIMENTOS LTDA</t>
+          <t>S.K. UEHARA CIA LTDA</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Diogo Calazans</t>
         </is>
       </c>
       <c r="I147" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J147" s="2" t="n">
-        <v>46280.4334184375</v>
+        <v>46203.44491331019</v>
       </c>
       <c r="K147" s="2" t="n">
-        <v>46283</v>
+        <v>46206</v>
       </c>
       <c r="L147" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M147" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N147" s="1" t="n"/>
       <c r="O147" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="P147" s="1" t="n"/>
-      <c r="Q147" s="1" t="inlineStr"/>
-      <c r="R147" s="1" t="inlineStr"/>
+        <v>46269</v>
+      </c>
+      <c r="P147" s="2" t="n">
+        <v>46269.68145385417</v>
+      </c>
+      <c r="Q147" s="1" t="inlineStr">
+        <is>
+          <t>Diogo Calazans</t>
+        </is>
+      </c>
+      <c r="R147" s="1" t="inlineStr">
+        <is>
+          <t>Não é devido, enviamos e-mail ao fiscal pedindo a retificação da Reinf para corrigir o valor.</t>
+        </is>
+      </c>
       <c r="S147" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T147" s="1" t="n"/>
       <c r="U147" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Karina Fonseca</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>80617</v>
+        <v>79827</v>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Alteração de Regime Tributário</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Alteração de Regime Tributário</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
@@ -12785,32 +12797,32 @@
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>Consta saldo residual IRRF nos períodos de 05/2025 e 01/2026.Por gentileza, verificar se os débitos são devidos ou se a DCTF do período deve ser retificada.</t>
+          <t xml:space="preserve">caros, O referido cliente deveria ter migrado para o lucro real no início de 2026.Em conversa com o Ronaldo, devemos retificar as obrigações acessórias e as guias de PIS e COFINS que outrora foram recolhidas como lucro presumido, quando concluido devemos comunicá-lo para que faça o pedido de alteração. </t>
         </is>
       </c>
       <c r="F148" s="1" t="n">
-        <v>5666</v>
+        <v>5726</v>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>S.K. UEHARA CIA LTDA</t>
+          <t>VIANA &amp; CIA LTDA</t>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
         <is>
-          <t>Diogo Calazans</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I148" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J148" s="2" t="n">
-        <v>46203.44491331019</v>
+        <v>46183.43924510416</v>
       </c>
       <c r="K148" s="2" t="n">
-        <v>46206</v>
+        <v>46185</v>
       </c>
       <c r="L148" s="1" t="inlineStr">
         <is>
@@ -12819,24 +12831,24 @@
       </c>
       <c r="M148" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N148" s="1" t="n"/>
-      <c r="O148" s="2" t="n">
-        <v>46269</v>
-      </c>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="n">
+        <v>46197.48391481482</v>
+      </c>
+      <c r="O148" s="1" t="n"/>
       <c r="P148" s="2" t="n">
-        <v>46269.68145385417</v>
+        <v>46204.7453832176</v>
       </c>
       <c r="Q148" s="1" t="inlineStr">
         <is>
-          <t>Diogo Calazans</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="R148" s="1" t="inlineStr">
         <is>
-          <t>Não é devido, enviamos e-mail ao fiscal pedindo a retificação da Reinf para corrigir o valor.</t>
+          <t xml:space="preserve">operação realizando o re-processo </t>
         </is>
       </c>
       <c r="S148" s="1" t="inlineStr">
@@ -12847,22 +12859,22 @@
       <c r="T148" s="1" t="n"/>
       <c r="U148" s="1" t="inlineStr">
         <is>
-          <t>Karina Fonseca</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>79827</v>
+        <v>82879</v>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Regime Tributário</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Regime Tributário</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
@@ -12872,84 +12884,80 @@
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">caros, O referido cliente deveria ter migrado para o lucro real no início de 2026.Em conversa com o Ronaldo, devemos retificar as obrigações acessórias e as guias de PIS e COFINS que outrora foram recolhidas como lucro presumido, quando concluido devemos comunicá-lo para que faça o pedido de alteração. </t>
+          <t>Conforme informado no chamado 78447 encerrado indevidamente, consta pendência de saldo credor incorreto do cliente 5740-Queiroz de Cotia no período de Abril 2026 e pendência de entrega de EFD/GIA do mês de Janeiro 2026.Por gentileza, providenciar correção.</t>
         </is>
       </c>
       <c r="F149" s="1" t="n">
-        <v>5726</v>
+        <v>5740</v>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VIANA &amp; CIA LTDA</t>
+          <t>QUEIROZ SUPERMERCADOS MJRR LTDA</t>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Larice Souza</t>
         </is>
       </c>
       <c r="I149" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J149" s="2" t="n">
-        <v>46183.43924510416</v>
+        <v>46258.42635717593</v>
       </c>
       <c r="K149" s="2" t="n">
-        <v>46185</v>
+        <v>46265</v>
       </c>
       <c r="L149" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M149" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N149" s="2" t="n">
-        <v>46197.48391481482</v>
-      </c>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N149" s="1" t="n"/>
       <c r="O149" s="1" t="n"/>
-      <c r="P149" s="2" t="n">
-        <v>46204.7453832176</v>
-      </c>
-      <c r="Q149" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+      <c r="P149" s="1" t="n"/>
+      <c r="Q149" s="1" t="inlineStr"/>
       <c r="R149" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">operação realizando o re-processo </t>
+          <t>Situação em analise, o cliente foi desnquadrado do SN e não temos arquivo do periodo</t>
         </is>
       </c>
       <c r="S149" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T149" s="1" t="n"/>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T149" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
       <c r="U149" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Larice Souza</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>82879</v>
+        <v>83251</v>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
@@ -12959,71 +12967,71 @@
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>Conforme informado no chamado 78447 encerrado indevidamente, consta pendência de saldo credor incorreto do cliente 5740-Queiroz de Cotia no período de Abril 2026 e pendência de entrega de EFD/GIA do mês de Janeiro 2026.Por gentileza, providenciar correção.</t>
+          <t xml:space="preserve">Bom dia, por gentileza emitir as guias em aberto da prefeitura de Caieiras. </t>
         </is>
       </c>
       <c r="F150" s="1" t="n">
-        <v>5740</v>
+        <v>5801</v>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>QUEIROZ SUPERMERCADOS MJRR LTDA</t>
+          <t xml:space="preserve">Nilcap Renovadora de Pneus LTDA </t>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
         <is>
-          <t>Larice Souza</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I150" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J150" s="2" t="n">
-        <v>46258.42635717593</v>
+        <v>46265.39660358796</v>
       </c>
       <c r="K150" s="2" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="L150" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M150" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N150" s="1" t="n"/>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="n">
+        <v>46266.64227881945</v>
+      </c>
       <c r="O150" s="1" t="n"/>
-      <c r="P150" s="1" t="n"/>
-      <c r="Q150" s="1" t="inlineStr"/>
+      <c r="P150" s="2" t="n">
+        <v>46266.68481299769</v>
+      </c>
+      <c r="Q150" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R150" s="1" t="inlineStr">
         <is>
-          <t>Situação em analise, o cliente foi desnquadrado do SN e não temos arquivo do periodo</t>
+          <t xml:space="preserve">operação realizando a demanda </t>
         </is>
       </c>
       <c r="S150" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T150" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="U150" s="1" t="inlineStr">
-        <is>
-          <t>Larice Souza</t>
-        </is>
-      </c>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T150" s="1" t="n"/>
+      <c r="U150" s="1" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>83251</v>
+        <v>84144</v>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
@@ -13042,7 +13050,7 @@
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, por gentileza emitir as guias em aberto da prefeitura de Caieiras. </t>
+          <t xml:space="preserve">Bom dia, por gentileza verificar a guia de ISS em aberto e encaminhar  recalculada </t>
         </is>
       </c>
       <c r="F151" s="1" t="n">
@@ -13055,7 +13063,7 @@
       </c>
       <c r="H151" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I151" s="1" t="inlineStr">
@@ -13064,10 +13072,10 @@
         </is>
       </c>
       <c r="J151" s="2" t="n">
-        <v>46265.39660358796</v>
+        <v>46283.40019563658</v>
       </c>
       <c r="K151" s="2" t="n">
-        <v>46266</v>
+        <v>46286</v>
       </c>
       <c r="L151" s="1" t="inlineStr">
         <is>
@@ -13079,21 +13087,20 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N151" s="2" t="n">
-        <v>46266.64227881945</v>
-      </c>
+      <c r="N151" s="1" t="n"/>
       <c r="O151" s="1" t="n"/>
       <c r="P151" s="2" t="n">
-        <v>46266.68481299769</v>
+        <v>46286.61436994213</v>
       </c>
       <c r="Q151" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="R151" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">operação realizando a demanda </t>
+          <t xml:space="preserve">Enviado por e-mail dia 18/09/2026
+</t>
         </is>
       </c>
       <c r="S151" s="1" t="inlineStr">
@@ -13102,162 +13109,157 @@
         </is>
       </c>
       <c r="T151" s="1" t="n"/>
-      <c r="U151" s="1" t="inlineStr"/>
+      <c r="U151" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>84144</v>
+        <v>83676</v>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Documentação</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Solicitação de Documentação</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, por gentileza verificar a guia de ISS em aberto e encaminhar  recalculada </t>
+          <t>Boa tarde!Por gentileza, disponibilizar a documentação para envio a nova contabilidade.</t>
         </is>
       </c>
       <c r="F152" s="1" t="n">
-        <v>5801</v>
+        <v>5822</v>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nilcap Renovadora de Pneus LTDA </t>
+          <t>RODRIGUES SERVICE SOLUTIONS LTDA</t>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Grasiele Santos</t>
         </is>
       </c>
       <c r="I152" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J152" s="2" t="n">
-        <v>46283.40019563658</v>
+        <v>46273.6644775463</v>
       </c>
       <c r="K152" s="2" t="n">
-        <v>46286</v>
+        <v>46274</v>
       </c>
       <c r="L152" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M152" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="N152" s="1" t="n"/>
       <c r="O152" s="1" t="n"/>
-      <c r="P152" s="2" t="n">
-        <v>46286.61436994213</v>
-      </c>
-      <c r="Q152" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+      <c r="P152" s="1" t="n"/>
+      <c r="Q152" s="1" t="inlineStr"/>
       <c r="R152" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enviado por e-mail dia 18/09/2026
-</t>
+          <t>Boa tarde, Karina!
+Poderia me informar qual a relação de documentos que devo enviar?</t>
         </is>
       </c>
       <c r="S152" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T152" s="1" t="n"/>
       <c r="U152" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Edivaldo Veiga</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>83676</v>
+        <v>84252</v>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentação</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, disponibilizar a documentação para envio a nova contabilidade.</t>
+          <t>bom dia!!verificar balanço e dre 2025, porque o valor do resultado está divergente.verificar balanço e dre 01-06 2026, porque o valor do resultado está divergente.</t>
         </is>
       </c>
       <c r="F153" s="1" t="n">
-        <v>5822</v>
+        <v>5834</v>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>RODRIGUES SERVICE SOLUTIONS LTDA</t>
+          <t>Caete Comunicacao Visual LTDA</t>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>Grasiele Santos</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="I153" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J153" s="2" t="n">
-        <v>46273.6644775463</v>
+        <v>46287.44208723379</v>
       </c>
       <c r="K153" s="2" t="n">
-        <v>46274</v>
+        <v>46288</v>
       </c>
       <c r="L153" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M153" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N153" s="1" t="n"/>
-      <c r="O153" s="1" t="n"/>
+      <c r="O153" s="2" t="n">
+        <v>46289</v>
+      </c>
       <c r="P153" s="1" t="n"/>
       <c r="Q153" s="1" t="inlineStr"/>
-      <c r="R153" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde, Karina!
-Poderia me informar qual a relação de documentos que devo enviar?</t>
-        </is>
-      </c>
+      <c r="R153" s="1" t="inlineStr"/>
       <c r="S153" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -13266,22 +13268,22 @@
       <c r="T153" s="1" t="n"/>
       <c r="U153" s="1" t="inlineStr">
         <is>
-          <t>Edivaldo Veiga</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>84252</v>
+        <v>81709</v>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
@@ -13291,15 +13293,15 @@
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>bom dia!!verificar balanço e dre 2025, porque o valor do resultado está divergente.verificar balanço e dre 01-06 2026, porque o valor do resultado está divergente.</t>
+          <t>5885 - segue comunicado ecac referente a dctf omisso abril 2026</t>
         </is>
       </c>
       <c r="F154" s="1" t="n">
-        <v>5834</v>
+        <v>5885</v>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>Caete Comunicacao Visual LTDA</t>
+          <t>INSTITUTO DE TECNOLOGIA ASSISTIVA LTDA</t>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
@@ -13309,35 +13311,45 @@
       </c>
       <c r="I154" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J154" s="2" t="n">
-        <v>46287.44208723379</v>
+        <v>46234.50876994213</v>
       </c>
       <c r="K154" s="2" t="n">
-        <v>46288</v>
+        <v>46237</v>
       </c>
       <c r="L154" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M154" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N154" s="1" t="n"/>
       <c r="O154" s="2" t="n">
-        <v>46289</v>
-      </c>
-      <c r="P154" s="1" t="n"/>
-      <c r="Q154" s="1" t="inlineStr"/>
-      <c r="R154" s="1" t="inlineStr"/>
+        <v>46237</v>
+      </c>
+      <c r="P154" s="2" t="n">
+        <v>46237.49066496528</v>
+      </c>
+      <c r="Q154" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R154" s="1" t="inlineStr">
+        <is>
+          <t>RESOLVIDO</t>
+        </is>
+      </c>
       <c r="S154" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T154" s="1" t="n"/>
@@ -13349,16 +13361,16 @@
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>81709</v>
+        <v>83938</v>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Fiscalização Municipal</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
@@ -13368,102 +13380,92 @@
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>5885 - segue comunicado ecac referente a dctf omisso abril 2026</t>
+          <t>Bom dia!Segue mensagem recebida no DEC Municipal, por gentileza, verificar.Prazo: 09/10/2026</t>
         </is>
       </c>
       <c r="F155" s="1" t="n">
-        <v>5885</v>
+        <v>5901</v>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>INSTITUTO DE TECNOLOGIA ASSISTIVA LTDA</t>
+          <t>Local Serviços Especializados LTDA</t>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I155" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J155" s="2" t="n">
-        <v>46234.50876994213</v>
+        <v>46279.44351177083</v>
       </c>
       <c r="K155" s="2" t="n">
-        <v>46237</v>
+        <v>46286</v>
       </c>
       <c r="L155" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M155" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Ana Santana</t>
         </is>
       </c>
       <c r="N155" s="1" t="n"/>
       <c r="O155" s="2" t="n">
-        <v>46237</v>
-      </c>
-      <c r="P155" s="2" t="n">
-        <v>46237.49066496528</v>
-      </c>
-      <c r="Q155" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
+        <v>46290</v>
+      </c>
+      <c r="P155" s="1" t="n"/>
+      <c r="Q155" s="1" t="inlineStr"/>
       <c r="R155" s="1" t="inlineStr">
         <is>
-          <t>RESOLVIDO</t>
+          <t>e-mail sobre a fiscalização respondido. GC irá dar continuidade no processo</t>
         </is>
       </c>
       <c r="S155" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T155" s="1" t="n"/>
-      <c r="U155" s="1" t="inlineStr">
-        <is>
-          <t>Isabella Nascimento</t>
-        </is>
-      </c>
+      <c r="U155" s="1" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>83938</v>
+        <v>83137</v>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>Fiscalização Municipal</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Segue mensagem recebida no DEC Municipal, por gentileza, verificar.Prazo: 09/10/2026</t>
+          <t>Cliente está solicitando a certidão negativa de débitos da PIZZA CREK, estadual. Ao tentar gerar aparecendo a pendencia anexa. Por favor solucionar o mais breve possivel.</t>
         </is>
       </c>
       <c r="F156" s="1" t="n">
-        <v>5901</v>
+        <v>5902</v>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>Local Serviços Especializados LTDA</t>
+          <t>PIZZA CREK FAST FOOD LTDA (FILIAL 7)</t>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
@@ -13477,35 +13479,41 @@
         </is>
       </c>
       <c r="J156" s="2" t="n">
-        <v>46279.44351177083</v>
+        <v>46261.54069120371</v>
       </c>
       <c r="K156" s="2" t="n">
-        <v>46286</v>
+        <v>46265</v>
       </c>
       <c r="L156" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M156" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N156" s="1" t="n"/>
       <c r="O156" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="P156" s="1" t="n"/>
-      <c r="Q156" s="1" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="P156" s="2" t="n">
+        <v>46279.49325150463</v>
+      </c>
+      <c r="Q156" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R156" s="1" t="inlineStr">
         <is>
-          <t>e-mail sobre a fiscalização respondido. GC irá dar continuidade no processo</t>
+          <t xml:space="preserve">sped já entregue </t>
         </is>
       </c>
       <c r="S156" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T156" s="1" t="n"/>
@@ -13513,16 +13521,16 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>83137</v>
+        <v>80527</v>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Documentação</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Ajuste de Documentação</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
@@ -13532,32 +13540,32 @@
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>Cliente está solicitando a certidão negativa de débitos da PIZZA CREK, estadual. Ao tentar gerar aparecendo a pendencia anexa. Por favor solucionar o mais breve possivel.</t>
+          <t>Prezados,Conforme solicitação do cliente favor providenciar o prólabore abaixo a partir do mês de julho 2026Merch Link LTDA: 49.797.761/0001-05- Ana Ligia Ribeiro Terensi Silva (proprietária)- ?Pró-labore: R$3.000,00</t>
         </is>
       </c>
       <c r="F157" s="1" t="n">
-        <v>5902</v>
+        <v>5908</v>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>PIZZA CREK FAST FOOD LTDA (FILIAL 7)</t>
+          <t>MERCH LINK LTDA</t>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Sara Cavalheiro</t>
         </is>
       </c>
       <c r="I157" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J157" s="2" t="n">
-        <v>46261.54069120371</v>
+        <v>46197.47626122685</v>
       </c>
       <c r="K157" s="2" t="n">
-        <v>46265</v>
+        <v>46203</v>
       </c>
       <c r="L157" s="1" t="inlineStr">
         <is>
@@ -13566,24 +13574,24 @@
       </c>
       <c r="M157" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
-        </is>
-      </c>
-      <c r="N157" s="1" t="n"/>
-      <c r="O157" s="2" t="n">
-        <v>46280</v>
-      </c>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N157" s="2" t="n">
+        <v>46197.57248116898</v>
+      </c>
+      <c r="O157" s="1" t="n"/>
       <c r="P157" s="2" t="n">
-        <v>46279.49325150463</v>
+        <v>46203.72243090278</v>
       </c>
       <c r="Q157" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Sara Cavalheiro</t>
         </is>
       </c>
       <c r="R157" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sped já entregue </t>
+          <t>Realizando cadastro para a folha de pro-labore.</t>
         </is>
       </c>
       <c r="S157" s="1" t="inlineStr">
@@ -13592,20 +13600,24 @@
         </is>
       </c>
       <c r="T157" s="1" t="n"/>
-      <c r="U157" s="1" t="inlineStr"/>
+      <c r="U157" s="1" t="inlineStr">
+        <is>
+          <t>Sara Cavalheiro</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>80527</v>
+        <v>80203</v>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>Ajuste de Documentação</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
@@ -13615,7 +13627,7 @@
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>Prezados,Conforme solicitação do cliente favor providenciar o prólabore abaixo a partir do mês de julho 2026Merch Link LTDA: 49.797.761/0001-05- Ana Ligia Ribeiro Terensi Silva (proprietária)- ?Pró-labore: R$3.000,00</t>
+          <t>Prezados, Boa tarde!Clienrte notificado ref autoregularização ref divergências na comparação por referência entre os valores do PGDAS e da Declaração de Informações de Meios de Pagamentos (DIMP).Prazo para regularização até 12/07/26Documentos disponiveis na pasta abaixo:J:\Importação\AUTO REGULARIZAÇÃO - PGDAS\5908</t>
         </is>
       </c>
       <c r="F158" s="1" t="n">
@@ -13628,16 +13640,16 @@
       </c>
       <c r="H158" s="1" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I158" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J158" s="2" t="n">
-        <v>46197.47626122685</v>
+        <v>46191.57591585648</v>
       </c>
       <c r="K158" s="2" t="n">
         <v>46203</v>
@@ -13653,20 +13665,20 @@
         </is>
       </c>
       <c r="N158" s="2" t="n">
-        <v>46197.57248116898</v>
+        <v>46192.52378078704</v>
       </c>
       <c r="O158" s="1" t="n"/>
       <c r="P158" s="2" t="n">
-        <v>46203.72243090278</v>
+        <v>46238.45672908565</v>
       </c>
       <c r="Q158" s="1" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="R158" s="1" t="inlineStr">
         <is>
-          <t>Realizando cadastro para a folha de pro-labore.</t>
+          <t xml:space="preserve">verificando </t>
         </is>
       </c>
       <c r="S158" s="1" t="inlineStr">
@@ -13677,22 +13689,22 @@
       <c r="T158" s="1" t="n"/>
       <c r="U158" s="1" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
-        <v>80203</v>
+        <v>79868</v>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
@@ -13702,7 +13714,7 @@
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>Prezados, Boa tarde!Clienrte notificado ref autoregularização ref divergências na comparação por referência entre os valores do PGDAS e da Declaração de Informações de Meios de Pagamentos (DIMP).Prazo para regularização até 12/07/26Documentos disponiveis na pasta abaixo:J:\Importação\AUTO REGULARIZAÇÃO - PGDAS\5908</t>
+          <t>Prezados, boa tarde!Cliente comunicou que o valor apurado no período de março 2026 está incompleto. Segundo cliente os valores de NFCe não foram considerados.Por gentileza, avaliar se os arquivos disponibilizados na época, via FTP foram escriturados.</t>
         </is>
       </c>
       <c r="F159" s="1" t="n">
@@ -13720,48 +13732,45 @@
       </c>
       <c r="I159" s="1" t="inlineStr">
         <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="n">
+        <v>46183.63777893518</v>
+      </c>
+      <c r="K159" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="L159" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido para Solicitante</t>
+        </is>
+      </c>
+      <c r="M159" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N159" s="1" t="n"/>
+      <c r="O159" s="1" t="n"/>
+      <c r="P159" s="1" t="n"/>
+      <c r="Q159" s="1" t="inlineStr"/>
+      <c r="R159" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irei verificar. 
+foi enviado ao cliente a confirmação de faturamento, porém não tivemos retorno na época. </t>
+        </is>
+      </c>
+      <c r="S159" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T159" s="1" t="inlineStr">
+        <is>
           <t>EF - VAREJO</t>
         </is>
       </c>
-      <c r="J159" s="2" t="n">
-        <v>46191.57591585648</v>
-      </c>
-      <c r="K159" s="2" t="n">
-        <v>46203</v>
-      </c>
-      <c r="L159" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M159" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N159" s="2" t="n">
-        <v>46192.52378078704</v>
-      </c>
-      <c r="O159" s="1" t="n"/>
-      <c r="P159" s="2" t="n">
-        <v>46238.45672908565</v>
-      </c>
-      <c r="Q159" s="1" t="inlineStr">
-        <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
-      <c r="R159" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verificando </t>
-        </is>
-      </c>
-      <c r="S159" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T159" s="1" t="n"/>
       <c r="U159" s="1" t="inlineStr">
         <is>
           <t>Lorrane Santos</t>
@@ -13770,16 +13779,16 @@
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
-        <v>79868</v>
+        <v>79820</v>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Pendência de Débito</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
@@ -13789,7 +13798,7 @@
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!Cliente comunicou que o valor apurado no período de março 2026 está incompleto. Segundo cliente os valores de NFCe não foram considerados.Por gentileza, avaliar se os arquivos disponibilizados na época, via FTP foram escriturados.</t>
+          <t>Consta pendência parcial de INSS referente mês 03/2026. Favor verificar se a pendência é indevida para retificação da DCTF.</t>
         </is>
       </c>
       <c r="F160" s="1" t="n">
@@ -13802,23 +13811,23 @@
       </c>
       <c r="H160" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Mauricio Lermen</t>
         </is>
       </c>
       <c r="I160" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J160" s="2" t="n">
-        <v>46183.63777893518</v>
+        <v>46182.79089837963</v>
       </c>
       <c r="K160" s="2" t="n">
-        <v>46184</v>
+        <v>46189</v>
       </c>
       <c r="L160" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M160" s="1" t="inlineStr">
@@ -13828,99 +13837,15 @@
       </c>
       <c r="N160" s="1" t="n"/>
       <c r="O160" s="1" t="n"/>
-      <c r="P160" s="1" t="n"/>
-      <c r="Q160" s="1" t="inlineStr"/>
+      <c r="P160" s="2" t="n">
+        <v>46189.41413730324</v>
+      </c>
+      <c r="Q160" s="1" t="inlineStr">
+        <is>
+          <t>Mauricio Lermen</t>
+        </is>
+      </c>
       <c r="R160" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Irei verificar. 
-foi enviado ao cliente a confirmação de faturamento, porém não tivemos retorno na época. </t>
-        </is>
-      </c>
-      <c r="S160" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T160" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="U160" s="1" t="inlineStr">
-        <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="1" t="n">
-        <v>79820</v>
-      </c>
-      <c r="B161" s="1" t="inlineStr">
-        <is>
-          <t>Pendência de Débito</t>
-        </is>
-      </c>
-      <c r="C161" s="1" t="inlineStr">
-        <is>
-          <t>Pendência de Débito</t>
-        </is>
-      </c>
-      <c r="D161" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E161" s="1" t="inlineStr">
-        <is>
-          <t>Consta pendência parcial de INSS referente mês 03/2026. Favor verificar se a pendência é indevida para retificação da DCTF.</t>
-        </is>
-      </c>
-      <c r="F161" s="1" t="n">
-        <v>5908</v>
-      </c>
-      <c r="G161" s="1" t="inlineStr">
-        <is>
-          <t>MERCH LINK LTDA</t>
-        </is>
-      </c>
-      <c r="H161" s="1" t="inlineStr">
-        <is>
-          <t>Mauricio Lermen</t>
-        </is>
-      </c>
-      <c r="I161" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="J161" s="2" t="n">
-        <v>46182.79089837963</v>
-      </c>
-      <c r="K161" s="2" t="n">
-        <v>46189</v>
-      </c>
-      <c r="L161" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M161" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N161" s="1" t="n"/>
-      <c r="O161" s="1" t="n"/>
-      <c r="P161" s="2" t="n">
-        <v>46189.41413730324</v>
-      </c>
-      <c r="Q161" s="1" t="inlineStr">
-        <is>
-          <t>Mauricio Lermen</t>
-        </is>
-      </c>
-      <c r="R161" s="1" t="inlineStr">
         <is>
           <t>Bom dia!
 Os valores são devidos conforme resumo, estou levantando se houve alteração após liberação.
@@ -13928,26 +13853,103 @@
 devolve este chamado para continuidade.</t>
         </is>
       </c>
+      <c r="S160" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T160" s="1" t="n"/>
+      <c r="U160" s="1" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>84257</v>
+      </c>
+      <c r="B161" s="1" t="inlineStr">
+        <is>
+          <t>Pendência de Débito</t>
+        </is>
+      </c>
+      <c r="C161" s="1" t="inlineStr">
+        <is>
+          <t>Pendência de Débito</t>
+        </is>
+      </c>
+      <c r="D161" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E161" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia!Por gentileza, verificar se é devido. Não localizamos a guia no SCI.</t>
+        </is>
+      </c>
+      <c r="F161" s="1" t="n">
+        <v>5920</v>
+      </c>
+      <c r="G161" s="1" t="inlineStr">
+        <is>
+          <t>G13 IMPORTAÇÃO E EXPORTAÇÃO LTDA (FILIAL 3)</t>
+        </is>
+      </c>
+      <c r="H161" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
+      <c r="I161" s="1" t="inlineStr">
+        <is>
+          <t>EF - INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="n">
+        <v>46287.4576400463</v>
+      </c>
+      <c r="K161" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="L161" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M161" s="1" t="inlineStr">
+        <is>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N161" s="1" t="n"/>
+      <c r="O161" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="P161" s="1" t="n"/>
+      <c r="Q161" s="1" t="inlineStr"/>
+      <c r="R161" s="1" t="inlineStr"/>
       <c r="S161" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T161" s="1" t="n"/>
-      <c r="U161" s="1" t="inlineStr"/>
+      <c r="U161" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>84257</v>
+        <v>83738</v>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
@@ -13957,133 +13959,56 @@
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Por gentileza, verificar se é devido. Não localizamos a guia no SCI.</t>
+          <t>por gentileza, providenciar regularização conforme anexo.Prazo para atendimento até 20/09/206periodo fora da gestão MG, cliente ciente que haverá custo para a realização do serviço.</t>
         </is>
       </c>
       <c r="F162" s="1" t="n">
-        <v>5920</v>
+        <v>5929</v>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>G13 IMPORTAÇÃO E EXPORTAÇÃO LTDA (FILIAL 3)</t>
+          <t>BAR E RESTAURANTE 1566 LTDA</t>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
       <c r="I162" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J162" s="2" t="n">
-        <v>46287.4576400463</v>
+        <v>46274.63414938658</v>
       </c>
       <c r="K162" s="2" t="n">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="L162" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M162" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N162" s="1" t="n"/>
       <c r="O162" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="P162" s="1" t="n"/>
-      <c r="Q162" s="1" t="inlineStr"/>
-      <c r="R162" s="1" t="inlineStr"/>
-      <c r="S162" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T162" s="1" t="n"/>
-      <c r="U162" s="1" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="1" t="n">
-        <v>83738</v>
-      </c>
-      <c r="B163" s="1" t="inlineStr">
-        <is>
-          <t>Autorregularização</t>
-        </is>
-      </c>
-      <c r="C163" s="1" t="inlineStr">
-        <is>
-          <t>Autorregularização</t>
-        </is>
-      </c>
-      <c r="D163" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E163" s="1" t="inlineStr">
-        <is>
-          <t>por gentileza, providenciar regularização conforme anexo.Prazo para atendimento até 20/09/206periodo fora da gestão MG, cliente ciente que haverá custo para a realização do serviço.</t>
-        </is>
-      </c>
-      <c r="F163" s="1" t="n">
-        <v>5929</v>
-      </c>
-      <c r="G163" s="1" t="inlineStr">
-        <is>
-          <t>BAR E RESTAURANTE 1566 LTDA</t>
-        </is>
-      </c>
-      <c r="H163" s="1" t="inlineStr">
+        <v>46276</v>
+      </c>
+      <c r="P162" s="2" t="n">
+        <v>46280.45140825232</v>
+      </c>
+      <c r="Q162" s="1" t="inlineStr">
         <is>
           <t>Lucas Fischer</t>
         </is>
       </c>
-      <c r="I163" s="1" t="inlineStr">
-        <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
-        </is>
-      </c>
-      <c r="J163" s="2" t="n">
-        <v>46274.63414938658</v>
-      </c>
-      <c r="K163" s="2" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L163" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M163" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N163" s="1" t="n"/>
-      <c r="O163" s="2" t="n">
-        <v>46276</v>
-      </c>
-      <c r="P163" s="2" t="n">
-        <v>46280.45140825232</v>
-      </c>
-      <c r="Q163" s="1" t="inlineStr">
-        <is>
-          <t>Lucas Fischer</t>
-        </is>
-      </c>
-      <c r="R163" s="1" t="inlineStr">
+      <c r="R162" s="1" t="inlineStr">
         <is>
           <t>Bom dia, 
 Precisamos que voces providenciem as informações para realizarmos a regularização:
@@ -14092,17 +14017,84 @@
 Não temos essa informação e não conseguimos se o cliente ou ex contador não informar.</t>
         </is>
       </c>
+      <c r="S162" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T162" s="1" t="n"/>
+      <c r="U162" s="1" t="inlineStr">
+        <is>
+          <t>Lucas Fischer</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>84398</v>
+      </c>
+      <c r="B163" s="1" t="inlineStr">
+        <is>
+          <t>Saldo Credor Incorreto</t>
+        </is>
+      </c>
+      <c r="C163" s="1" t="inlineStr">
+        <is>
+          <t>Saldo Credor Incorreto</t>
+        </is>
+      </c>
+      <c r="D163" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E163" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providencia regularização saldo credor incorreto, conforme situação do contribuinte anexa.</t>
+        </is>
+      </c>
+      <c r="F163" s="1" t="n">
+        <v>5930</v>
+      </c>
+      <c r="G163" s="1" t="inlineStr">
+        <is>
+          <t>ESPETINHO VILA MARIANA LTDA</t>
+        </is>
+      </c>
+      <c r="H163" s="1" t="n"/>
+      <c r="I163" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="n">
+        <v>46288.79362025463</v>
+      </c>
+      <c r="K163" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="L163" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M163" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N163" s="1" t="n"/>
+      <c r="O163" s="1" t="n"/>
+      <c r="P163" s="1" t="n"/>
+      <c r="Q163" s="1" t="inlineStr"/>
+      <c r="R163" s="1" t="n"/>
       <c r="S163" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T163" s="1" t="n"/>
-      <c r="U163" s="1" t="inlineStr">
-        <is>
-          <t>Lucas Fischer</t>
-        </is>
-      </c>
+      <c r="U163" s="1" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -54271,7 +54263,7 @@
       </c>
       <c r="H709" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I709" s="1" t="inlineStr">
@@ -54287,7 +54279,7 @@
       </c>
       <c r="L709" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M709" s="1" t="inlineStr">
@@ -54297,12 +54289,23 @@
       </c>
       <c r="N709" s="1" t="n"/>
       <c r="O709" s="1" t="n"/>
-      <c r="P709" s="1" t="n"/>
-      <c r="Q709" s="1" t="inlineStr"/>
-      <c r="R709" s="1" t="inlineStr"/>
+      <c r="P709" s="2" t="n">
+        <v>46288.7633241088</v>
+      </c>
+      <c r="Q709" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R709" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+As declarações foram retificadas? Precisamos das copias das declarações originais e retificadoras.</t>
+        </is>
+      </c>
       <c r="S709" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T709" s="1" t="n"/>
@@ -58811,7 +58814,7 @@
       </c>
       <c r="H767" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I767" s="1" t="inlineStr">
@@ -58827,7 +58830,7 @@
       </c>
       <c r="L767" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M767" s="1" t="inlineStr">
@@ -58837,12 +58840,23 @@
       </c>
       <c r="N767" s="1" t="n"/>
       <c r="O767" s="1" t="n"/>
-      <c r="P767" s="1" t="n"/>
-      <c r="Q767" s="1" t="inlineStr"/>
-      <c r="R767" s="1" t="inlineStr"/>
+      <c r="P767" s="2" t="n">
+        <v>46288.76317905093</v>
+      </c>
+      <c r="Q767" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R767" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+As declarações foram retificadas? Precisamos das copias das declarações originais e retificadoras.</t>
+        </is>
+      </c>
       <c r="S767" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T767" s="1" t="n"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 09:37
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -51006,69 +51006,59 @@
     </row>
     <row r="666">
       <c r="A666" s="1" t="n">
-        <v>81777</v>
+        <v>84403</v>
       </c>
       <c r="B666" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C666" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D666" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - EF</t>
         </is>
       </c>
       <c r="E666" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, poderia fazer o processo administrativo da empresa 3616 - CCV do ISS mes 04/2026, a guia foi cancelada para realizar emissão de notas da MG Negócios , que tinha nota emitidas contra a CCV, pós o financeiro realizou o pagamento da guia de ISS de serviços prestados </t>
+          <t>Bom dia,Solicito, por gentileza, a baixa das tarefas referentes à entrega da DIPAM das empresas 5945, 5986, 6114 e 6115.Ao realizar a transmissão dos arquivos, o sistema informa que o arquivo já se encontra na base de dados, indicando que a entrega foi realizada. Porém, ao tentar acessar a transmissão para consultar e obter o recibo, o sistema informa que não foi encontrado nenhum arquivo.Dessa forma, não estamos conseguindo acessar os recibos para anexá-los às respectivas tarefas.Informo também que já estou tomando as providências necessárias para obter os arquivos/recibos das transmissões.Empresas: 5945 – 5986 – 6114 – 6115</t>
         </is>
       </c>
       <c r="F666" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G666" s="1" t="n"/>
-      <c r="H666" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+      <c r="H666" s="1" t="n"/>
       <c r="I666" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J666" s="2" t="n">
-        <v>46237.59220239583</v>
+        <v>46289.39711704861</v>
       </c>
       <c r="K666" s="2" t="n">
-        <v>46239</v>
+        <v>46290</v>
       </c>
       <c r="L666" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M666" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
-        </is>
-      </c>
-      <c r="N666" s="2" t="n">
-        <v>46241.63536697916</v>
-      </c>
+          <t>Jasmina Melo</t>
+        </is>
+      </c>
+      <c r="N666" s="1" t="n"/>
       <c r="O666" s="1" t="n"/>
       <c r="P666" s="1" t="n"/>
       <c r="Q666" s="1" t="inlineStr"/>
-      <c r="R666" s="1" t="inlineStr">
-        <is>
-          <t>Solicitei orientações à Prefeitura em como proceder para regularização, aguardando retorno.</t>
-        </is>
-      </c>
+      <c r="R666" s="1" t="n"/>
       <c r="S666" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -51079,26 +51069,26 @@
     </row>
     <row r="667">
       <c r="A667" s="1" t="n">
-        <v>82094</v>
+        <v>81777</v>
       </c>
       <c r="B667" s="1" t="inlineStr">
         <is>
-          <t>Processo de VISA</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C667" s="1" t="inlineStr">
         <is>
-          <t>Renovação</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D667" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E667" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar a renovação da vigilância sanitária das empresas do grupo Atalaia - código - 1685/2616/4881/6175 - com urgência. Muito Obrigada!</t>
+          <t xml:space="preserve">Boa tarde, poderia fazer o processo administrativo da empresa 3616 - CCV do ISS mes 04/2026, a guia foi cancelada para realizar emissão de notas da MG Negócios , que tinha nota emitidas contra a CCV, pós o financeiro realizou o pagamento da guia de ISS de serviços prestados </t>
         </is>
       </c>
       <c r="F667" s="1" t="n">
@@ -51107,43 +51097,116 @@
       <c r="G667" s="1" t="n"/>
       <c r="H667" s="1" t="inlineStr">
         <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="I667" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J667" s="2" t="n">
+        <v>46237.59220239583</v>
+      </c>
+      <c r="K667" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="L667" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M667" s="1" t="inlineStr">
+        <is>
+          <t>Romario Silva</t>
+        </is>
+      </c>
+      <c r="N667" s="2" t="n">
+        <v>46241.63536697916</v>
+      </c>
+      <c r="O667" s="1" t="n"/>
+      <c r="P667" s="1" t="n"/>
+      <c r="Q667" s="1" t="inlineStr"/>
+      <c r="R667" s="1" t="inlineStr">
+        <is>
+          <t>Solicitei orientações à Prefeitura em como proceder para regularização, aguardando retorno.</t>
+        </is>
+      </c>
+      <c r="S667" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T667" s="1" t="n"/>
+      <c r="U667" s="1" t="inlineStr"/>
+    </row>
+    <row r="668">
+      <c r="A668" s="1" t="n">
+        <v>82094</v>
+      </c>
+      <c r="B668" s="1" t="inlineStr">
+        <is>
+          <t>Processo de VISA</t>
+        </is>
+      </c>
+      <c r="C668" s="1" t="inlineStr">
+        <is>
+          <t>Renovação</t>
+        </is>
+      </c>
+      <c r="D668" s="1" t="inlineStr">
+        <is>
+          <t>SANTOS - GC</t>
+        </is>
+      </c>
+      <c r="E668" s="1" t="inlineStr">
+        <is>
+          <t>Favor providenciar a renovação da vigilância sanitária das empresas do grupo Atalaia - código - 1685/2616/4881/6175 - com urgência. Muito Obrigada!</t>
+        </is>
+      </c>
+      <c r="F668" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G668" s="1" t="n"/>
+      <c r="H668" s="1" t="inlineStr">
+        <is>
           <t>Talita Silva</t>
         </is>
       </c>
-      <c r="I667" s="1" t="inlineStr">
+      <c r="I668" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J667" s="2" t="n">
+      <c r="J668" s="2" t="n">
         <v>46241.66958043981</v>
       </c>
-      <c r="K667" s="2" t="n">
+      <c r="K668" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="L667" s="1" t="inlineStr">
+      <c r="L668" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M667" s="1" t="inlineStr">
+      <c r="M668" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N667" s="2" t="n">
+      <c r="N668" s="2" t="n">
         <v>46252.70058159722</v>
       </c>
-      <c r="O667" s="1" t="n"/>
-      <c r="P667" s="2" t="n">
+      <c r="O668" s="1" t="n"/>
+      <c r="P668" s="2" t="n">
         <v>46280.42831450231</v>
       </c>
-      <c r="Q667" s="1" t="inlineStr">
+      <c r="Q668" s="1" t="inlineStr">
         <is>
           <t>Talita Silva</t>
         </is>
       </c>
-      <c r="R667" s="1" t="inlineStr">
+      <c r="R668" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Olá, boa tarde!
 Enviei por e-mail o Anexo III das empresas para assinatura.
@@ -51151,85 +51214,6 @@
 </t>
         </is>
       </c>
-      <c r="S667" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T667" s="1" t="n"/>
-      <c r="U667" s="1" t="inlineStr"/>
-    </row>
-    <row r="668">
-      <c r="A668" s="1" t="n">
-        <v>82296</v>
-      </c>
-      <c r="B668" s="1" t="inlineStr">
-        <is>
-          <t>Parcelamento Estadual</t>
-        </is>
-      </c>
-      <c r="C668" s="1" t="inlineStr">
-        <is>
-          <t>Divida Ativa</t>
-        </is>
-      </c>
-      <c r="D668" s="1" t="inlineStr">
-        <is>
-          <t>SANTOS - ADM</t>
-        </is>
-      </c>
-      <c r="E668" s="1" t="inlineStr">
-        <is>
-          <t>Cliente 5219 e 5551 solicitou parcelamento do ICMS , pode fazer a simulação</t>
-        </is>
-      </c>
-      <c r="F668" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G668" s="1" t="n"/>
-      <c r="H668" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="I668" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J668" s="2" t="n">
-        <v>46246.6211778588</v>
-      </c>
-      <c r="K668" s="2" t="n">
-        <v>46248</v>
-      </c>
-      <c r="L668" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M668" s="1" t="inlineStr">
-        <is>
-          <t>Lidia Tavares</t>
-        </is>
-      </c>
-      <c r="N668" s="2" t="n">
-        <v>46268.68634155093</v>
-      </c>
-      <c r="O668" s="1" t="n"/>
-      <c r="P668" s="2" t="n">
-        <v>46276.37282434028</v>
-      </c>
-      <c r="Q668" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="R668" s="1" t="inlineStr">
-        <is>
-          <t>Deve ser aberto um chamado para cada solicitação/cliente.</t>
-        </is>
-      </c>
       <c r="S668" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -51240,16 +51224,16 @@
     </row>
     <row r="669">
       <c r="A669" s="1" t="n">
-        <v>81227</v>
+        <v>82296</v>
       </c>
       <c r="B669" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Parcelamento Estadual</t>
         </is>
       </c>
       <c r="C669" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D669" s="1" t="inlineStr">
@@ -51259,7 +51243,7 @@
       </c>
       <c r="E669" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>Cliente 5219 e 5551 solicitou parcelamento do ICMS , pode fazer a simulação</t>
         </is>
       </c>
       <c r="F669" s="1" t="n">
@@ -51277,14 +51261,14 @@
         </is>
       </c>
       <c r="J669" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46246.6211778588</v>
       </c>
       <c r="K669" s="2" t="n">
-        <v>46224</v>
+        <v>46248</v>
       </c>
       <c r="L669" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M669" s="1" t="inlineStr">
@@ -51293,19 +51277,25 @@
         </is>
       </c>
       <c r="N669" s="2" t="n">
-        <v>46232.73233688658</v>
+        <v>46268.68634155093</v>
       </c>
       <c r="O669" s="1" t="n"/>
-      <c r="P669" s="1" t="n"/>
-      <c r="Q669" s="1" t="inlineStr"/>
+      <c r="P669" s="2" t="n">
+        <v>46276.37282434028</v>
+      </c>
+      <c r="Q669" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="R669" s="1" t="inlineStr">
         <is>
-          <t>Verificando via chat.</t>
+          <t>Deve ser aberto um chamado para cada solicitação/cliente.</t>
         </is>
       </c>
       <c r="S669" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T669" s="1" t="n"/>
@@ -51313,26 +51303,26 @@
     </row>
     <row r="670">
       <c r="A670" s="1" t="n">
-        <v>83249</v>
+        <v>81227</v>
       </c>
       <c r="B670" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C670" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D670" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E670" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">6533 - OFICIALMED BOM JESUS PRODUTOS FARMACÊUTICOS E APOIO ADMINISTRATIVO LTDA - Renovação do Alvará </t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F670" s="1" t="n">
@@ -51341,122 +51331,195 @@
       <c r="G670" s="1" t="n"/>
       <c r="H670" s="1" t="inlineStr">
         <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="I670" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J670" s="2" t="n">
+        <v>46223.69836307871</v>
+      </c>
+      <c r="K670" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="L670" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M670" s="1" t="inlineStr">
+        <is>
+          <t>Lidia Tavares</t>
+        </is>
+      </c>
+      <c r="N670" s="2" t="n">
+        <v>46232.73233688658</v>
+      </c>
+      <c r="O670" s="1" t="n"/>
+      <c r="P670" s="1" t="n"/>
+      <c r="Q670" s="1" t="inlineStr"/>
+      <c r="R670" s="1" t="inlineStr">
+        <is>
+          <t>Verificando via chat.</t>
+        </is>
+      </c>
+      <c r="S670" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T670" s="1" t="n"/>
+      <c r="U670" s="1" t="inlineStr"/>
+    </row>
+    <row r="671">
+      <c r="A671" s="1" t="n">
+        <v>83249</v>
+      </c>
+      <c r="B671" s="1" t="inlineStr">
+        <is>
+          <t>Regularização</t>
+        </is>
+      </c>
+      <c r="C671" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D671" s="1" t="inlineStr">
+        <is>
+          <t>SANTOS - GC</t>
+        </is>
+      </c>
+      <c r="E671" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6533 - OFICIALMED BOM JESUS PRODUTOS FARMACÊUTICOS E APOIO ADMINISTRATIVO LTDA - Renovação do Alvará </t>
+        </is>
+      </c>
+      <c r="F671" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G671" s="1" t="n"/>
+      <c r="H671" s="1" t="inlineStr">
+        <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I670" s="1" t="inlineStr">
+      <c r="I671" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J670" s="2" t="n">
+      <c r="J671" s="2" t="n">
         <v>46265.38856802083</v>
       </c>
-      <c r="K670" s="2" t="n">
+      <c r="K671" s="2" t="n">
         <v>46267</v>
       </c>
-      <c r="L670" s="1" t="inlineStr">
+      <c r="L671" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M670" s="1" t="inlineStr">
+      <c r="M671" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N670" s="2" t="n">
+      <c r="N671" s="2" t="n">
         <v>46267.71143642361</v>
       </c>
-      <c r="O670" s="1" t="n"/>
-      <c r="P670" s="2" t="n">
+      <c r="O671" s="1" t="n"/>
+      <c r="P671" s="2" t="n">
         <v>46288.52680405093</v>
       </c>
-      <c r="Q670" s="1" t="inlineStr">
+      <c r="Q671" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="R670" s="1" t="inlineStr">
+      <c r="R671" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 Qual alvará?
 Atenciosamente,</t>
         </is>
       </c>
-      <c r="S670" s="1" t="inlineStr">
+      <c r="S671" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T670" s="1" t="n"/>
-      <c r="U670" s="1" t="inlineStr"/>
-    </row>
-    <row r="671">
-      <c r="A671" s="1" t="n">
+      <c r="T671" s="1" t="n"/>
+      <c r="U671" s="1" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" s="1" t="n">
         <v>83452</v>
       </c>
-      <c r="B671" s="1" t="inlineStr">
+      <c r="B672" s="1" t="inlineStr">
         <is>
           <t>Encerramento de Empresa</t>
         </is>
       </c>
-      <c r="C671" s="1" t="inlineStr">
+      <c r="C672" s="1" t="inlineStr">
         <is>
           <t>Eireli - Comércio</t>
         </is>
       </c>
-      <c r="D671" s="1" t="inlineStr">
+      <c r="D672" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E671" s="1" t="inlineStr">
+      <c r="E672" s="1" t="inlineStr">
         <is>
           <t>Pós Ata de reunião - 2876 -  BAR E LANCHES JUVENTUDE DE PRAIA GRANDE- EIRELI  Juventude	Encerramento Empresa 	O cliente solicitou o encerramento da empresa Juventude, ficando registrada a pendência para avaliação e condução dos procedimentos fiscais, cadastrais e societários necessários. 31/08/2026</t>
         </is>
       </c>
-      <c r="F671" s="1" t="n">
+      <c r="F672" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G671" s="1" t="n"/>
-      <c r="H671" s="1" t="inlineStr">
+      <c r="G672" s="1" t="n"/>
+      <c r="H672" s="1" t="inlineStr">
         <is>
           <t>Ronaldo Dias</t>
         </is>
       </c>
-      <c r="I671" s="1" t="inlineStr">
+      <c r="I672" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J671" s="2" t="n">
+      <c r="J672" s="2" t="n">
         <v>46267.40487928241</v>
       </c>
-      <c r="K671" s="2" t="n">
+      <c r="K672" s="2" t="n">
         <v>46269</v>
       </c>
-      <c r="L671" s="1" t="inlineStr">
+      <c r="L672" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M671" s="1" t="inlineStr">
+      <c r="M672" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N671" s="1" t="n"/>
-      <c r="O671" s="1" t="n"/>
-      <c r="P671" s="2" t="n">
+      <c r="N672" s="1" t="n"/>
+      <c r="O672" s="1" t="n"/>
+      <c r="P672" s="2" t="n">
         <v>46268.72386732639</v>
       </c>
-      <c r="Q671" s="1" t="inlineStr">
+      <c r="Q672" s="1" t="inlineStr">
         <is>
           <t>Ronaldo Dias</t>
         </is>
       </c>
-      <c r="R671" s="1" t="inlineStr">
+      <c r="R672" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Anexo proposta e abaixo as condições para dar andamento.
 1.	Quadro de pessoal: não possuir funcionários ativos — todos os contratos de trabalho devem estar encerrados e as obrigações trabalhistas devidamente quitadas;
@@ -51467,320 +51530,320 @@
 </t>
         </is>
       </c>
-      <c r="S671" s="1" t="inlineStr">
+      <c r="S672" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T671" s="1" t="n"/>
-      <c r="U671" s="1" t="inlineStr"/>
-    </row>
-    <row r="672">
-      <c r="A672" s="1" t="n">
+      <c r="T672" s="1" t="n"/>
+      <c r="U672" s="1" t="inlineStr"/>
+    </row>
+    <row r="673">
+      <c r="A673" s="1" t="n">
         <v>83530</v>
       </c>
-      <c r="B672" s="1" t="inlineStr">
+      <c r="B673" s="1" t="inlineStr">
         <is>
           <t>Parcelamento RFB</t>
         </is>
       </c>
-      <c r="C672" s="1" t="inlineStr">
+      <c r="C673" s="1" t="inlineStr">
         <is>
           <t>Simplificado</t>
         </is>
       </c>
-      <c r="D672" s="1" t="inlineStr">
+      <c r="D673" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E672" s="1" t="inlineStr">
+      <c r="E673" s="1" t="inlineStr">
         <is>
           <t>6296 - GRAND DIVINO COMERCIO DE ALIMENTOS LTDA - Por gentileza simular em 12 vezes os debitos em aberto na RFB. obrigada.</t>
         </is>
       </c>
-      <c r="F672" s="1" t="n">
+      <c r="F673" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G672" s="1" t="n"/>
-      <c r="H672" s="1" t="inlineStr">
+      <c r="G673" s="1" t="n"/>
+      <c r="H673" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="I672" s="1" t="inlineStr">
+      <c r="I673" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J672" s="2" t="n">
+      <c r="J673" s="2" t="n">
         <v>46267.7888037037</v>
       </c>
-      <c r="K672" s="2" t="n">
+      <c r="K673" s="2" t="n">
         <v>46272</v>
       </c>
-      <c r="L672" s="1" t="inlineStr">
+      <c r="L673" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M672" s="1" t="inlineStr">
+      <c r="M673" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N672" s="1" t="n"/>
-      <c r="O672" s="1" t="n"/>
-      <c r="P672" s="2" t="n">
+      <c r="N673" s="1" t="n"/>
+      <c r="O673" s="1" t="n"/>
+      <c r="P673" s="2" t="n">
         <v>46280.77879980324</v>
       </c>
-      <c r="Q672" s="1" t="inlineStr">
+      <c r="Q673" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R672" s="1" t="inlineStr">
+      <c r="R673" s="1" t="inlineStr">
         <is>
           <t>Rafa, boa tarde!
 Segue simulado e proposta em anexo.
 Por gentileza, verificar a omissão de DCTFWEB 12/2025.</t>
         </is>
       </c>
-      <c r="S672" s="1" t="inlineStr">
+      <c r="S673" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T672" s="1" t="n"/>
-      <c r="U672" s="1" t="inlineStr"/>
-    </row>
-    <row r="673">
-      <c r="A673" s="1" t="n">
+      <c r="T673" s="1" t="n"/>
+      <c r="U673" s="1" t="inlineStr"/>
+    </row>
+    <row r="674">
+      <c r="A674" s="1" t="n">
         <v>83563</v>
       </c>
-      <c r="B673" s="1" t="inlineStr">
+      <c r="B674" s="1" t="inlineStr">
         <is>
           <t>Processo de Prefeitura</t>
         </is>
       </c>
-      <c r="C673" s="1" t="inlineStr">
+      <c r="C674" s="1" t="inlineStr">
         <is>
           <t>Geral</t>
         </is>
       </c>
-      <c r="D673" s="1" t="inlineStr">
+      <c r="D674" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E673" s="1" t="inlineStr">
+      <c r="E674" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">3173 - Providenciar o Alvará/CLI por favor </t>
         </is>
       </c>
-      <c r="F673" s="1" t="n">
+      <c r="F674" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G673" s="1" t="n"/>
-      <c r="H673" s="1" t="inlineStr">
+      <c r="G674" s="1" t="n"/>
+      <c r="H674" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I673" s="1" t="inlineStr">
+      <c r="I674" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J673" s="2" t="n">
+      <c r="J674" s="2" t="n">
         <v>46268.54673834491</v>
       </c>
-      <c r="K673" s="2" t="n">
+      <c r="K674" s="2" t="n">
         <v>46273</v>
       </c>
-      <c r="L673" s="1" t="inlineStr">
+      <c r="L674" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M673" s="1" t="inlineStr">
+      <c r="M674" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N673" s="2" t="n">
+      <c r="N674" s="2" t="n">
         <v>46268.67929375</v>
       </c>
-      <c r="O673" s="1" t="n"/>
-      <c r="P673" s="2" t="n">
+      <c r="O674" s="1" t="n"/>
+      <c r="P674" s="2" t="n">
         <v>46275.64996585648</v>
       </c>
-      <c r="Q673" s="1" t="inlineStr">
+      <c r="Q674" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="R673" s="1" t="inlineStr">
+      <c r="R674" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 Providenciando a Viabilidade.
 Atenciosamente,</t>
         </is>
       </c>
-      <c r="S673" s="1" t="inlineStr">
+      <c r="S674" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T673" s="1" t="n"/>
-      <c r="U673" s="1" t="inlineStr"/>
-    </row>
-    <row r="674">
-      <c r="A674" s="1" t="n">
+      <c r="T674" s="1" t="n"/>
+      <c r="U674" s="1" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" s="1" t="n">
         <v>83564</v>
       </c>
-      <c r="B674" s="1" t="inlineStr">
+      <c r="B675" s="1" t="inlineStr">
         <is>
           <t>Processo de Prefeitura</t>
         </is>
       </c>
-      <c r="C674" s="1" t="inlineStr">
+      <c r="C675" s="1" t="inlineStr">
         <is>
           <t>Geral</t>
         </is>
       </c>
-      <c r="D674" s="1" t="inlineStr">
+      <c r="D675" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E674" s="1" t="inlineStr">
+      <c r="E675" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">3176 - renovar o Alvará/CLi por favor </t>
         </is>
       </c>
-      <c r="F674" s="1" t="n">
+      <c r="F675" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G674" s="1" t="n"/>
-      <c r="H674" s="1" t="inlineStr">
+      <c r="G675" s="1" t="n"/>
+      <c r="H675" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I674" s="1" t="inlineStr">
+      <c r="I675" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J674" s="2" t="n">
+      <c r="J675" s="2" t="n">
         <v>46268.54783070602</v>
       </c>
-      <c r="K674" s="2" t="n">
+      <c r="K675" s="2" t="n">
         <v>46273</v>
       </c>
-      <c r="L674" s="1" t="inlineStr">
+      <c r="L675" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M674" s="1" t="inlineStr">
+      <c r="M675" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N674" s="2" t="n">
+      <c r="N675" s="2" t="n">
         <v>46268.67942207176</v>
       </c>
-      <c r="O674" s="1" t="n"/>
-      <c r="P674" s="2" t="n">
+      <c r="O675" s="1" t="n"/>
+      <c r="P675" s="2" t="n">
         <v>46275.65324540509</v>
       </c>
-      <c r="Q674" s="1" t="inlineStr">
+      <c r="Q675" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="R674" s="1" t="inlineStr">
+      <c r="R675" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 Providenciando a Viabilidade.
 Atenciosamente,</t>
         </is>
       </c>
-      <c r="S674" s="1" t="inlineStr">
+      <c r="S675" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T674" s="1" t="n"/>
-      <c r="U674" s="1" t="inlineStr"/>
-    </row>
-    <row r="675">
-      <c r="A675" s="1" t="n">
+      <c r="T675" s="1" t="n"/>
+      <c r="U675" s="1" t="inlineStr"/>
+    </row>
+    <row r="676">
+      <c r="A676" s="1" t="n">
         <v>83565</v>
       </c>
-      <c r="B675" s="1" t="inlineStr">
+      <c r="B676" s="1" t="inlineStr">
         <is>
           <t>Processo de Prefeitura</t>
         </is>
       </c>
-      <c r="C675" s="1" t="inlineStr">
+      <c r="C676" s="1" t="inlineStr">
         <is>
           <t>Geral</t>
         </is>
       </c>
-      <c r="D675" s="1" t="inlineStr">
+      <c r="D676" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E675" s="1" t="inlineStr">
+      <c r="E676" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">3177 - Renovação de Alvará/cli por favor </t>
         </is>
       </c>
-      <c r="F675" s="1" t="n">
+      <c r="F676" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G675" s="1" t="n"/>
-      <c r="H675" s="1" t="inlineStr">
+      <c r="G676" s="1" t="n"/>
+      <c r="H676" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I675" s="1" t="inlineStr">
+      <c r="I676" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J675" s="2" t="n">
+      <c r="J676" s="2" t="n">
         <v>46268.54870725694</v>
       </c>
-      <c r="K675" s="2" t="n">
+      <c r="K676" s="2" t="n">
         <v>46273</v>
       </c>
-      <c r="L675" s="1" t="inlineStr">
+      <c r="L676" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M675" s="1" t="inlineStr">
+      <c r="M676" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N675" s="1" t="n"/>
-      <c r="O675" s="1" t="n"/>
-      <c r="P675" s="2" t="n">
+      <c r="N676" s="1" t="n"/>
+      <c r="O676" s="1" t="n"/>
+      <c r="P676" s="2" t="n">
         <v>46268.56602326389</v>
       </c>
-      <c r="Q675" s="1" t="inlineStr">
+      <c r="Q676" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="R675" s="1" t="inlineStr">
+      <c r="R676" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 O endereço do AVCB ( AVENIDA CABUÇU Nº: 377) e o endereço da empresa (RUA JOAO MARIANO, 193).
@@ -51788,164 +51851,87 @@
 Atenciosamente,</t>
         </is>
       </c>
-      <c r="S675" s="1" t="inlineStr">
+      <c r="S676" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T675" s="1" t="n"/>
-      <c r="U675" s="1" t="inlineStr"/>
-    </row>
-    <row r="676">
-      <c r="A676" s="1" t="n">
+      <c r="T676" s="1" t="n"/>
+      <c r="U676" s="1" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" s="1" t="n">
         <v>83583</v>
       </c>
-      <c r="B676" s="1" t="inlineStr">
+      <c r="B677" s="1" t="inlineStr">
         <is>
           <t>Processo de Prefeitura</t>
         </is>
       </c>
-      <c r="C676" s="1" t="inlineStr">
+      <c r="C677" s="1" t="inlineStr">
         <is>
           <t>Geral</t>
         </is>
       </c>
-      <c r="D676" s="1" t="inlineStr">
+      <c r="D677" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E676" s="1" t="inlineStr">
+      <c r="E677" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">3174 - Ronovação do Alvará/Cli por favor </t>
         </is>
       </c>
-      <c r="F676" s="1" t="n">
+      <c r="F677" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G676" s="1" t="n"/>
-      <c r="H676" s="1" t="inlineStr">
+      <c r="G677" s="1" t="n"/>
+      <c r="H677" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I676" s="1" t="inlineStr">
+      <c r="I677" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J676" s="2" t="n">
+      <c r="J677" s="2" t="n">
         <v>46268.69685413194</v>
       </c>
-      <c r="K676" s="2" t="n">
+      <c r="K677" s="2" t="n">
         <v>46273</v>
       </c>
-      <c r="L676" s="1" t="inlineStr">
+      <c r="L677" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M676" s="1" t="inlineStr">
+      <c r="M677" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N676" s="2" t="n">
+      <c r="N677" s="2" t="n">
         <v>46273.69585717592</v>
       </c>
-      <c r="O676" s="1" t="n"/>
-      <c r="P676" s="2" t="n">
+      <c r="O677" s="1" t="n"/>
+      <c r="P677" s="2" t="n">
         <v>46282.53441554398</v>
       </c>
-      <c r="Q676" s="1" t="inlineStr">
+      <c r="Q677" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="R676" s="1" t="inlineStr">
+      <c r="R677" s="1" t="inlineStr">
         <is>
           <t>Boa tarde,
 Aguardando a aprovação da viabilidade.
 Atenciosamente</t>
         </is>
       </c>
-      <c r="S676" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T676" s="1" t="n"/>
-      <c r="U676" s="1" t="inlineStr"/>
-    </row>
-    <row r="677">
-      <c r="A677" s="1" t="n">
-        <v>83704</v>
-      </c>
-      <c r="B677" s="1" t="inlineStr">
-        <is>
-          <t>Levantamento de Débitos Mensal</t>
-        </is>
-      </c>
-      <c r="C677" s="1" t="inlineStr">
-        <is>
-          <t>PGFN</t>
-        </is>
-      </c>
-      <c r="D677" s="1" t="inlineStr">
-        <is>
-          <t>SANTOS - GC</t>
-        </is>
-      </c>
-      <c r="E677" s="1" t="inlineStr">
-        <is>
-          <t>4200 - Henrique Leone- Por gentileza simular o parcelamento dos débitos que são mencionados na carta em anexo por favor.</t>
-        </is>
-      </c>
-      <c r="F677" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G677" s="1" t="n"/>
-      <c r="H677" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="I677" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J677" s="2" t="n">
-        <v>46274.42889741898</v>
-      </c>
-      <c r="K677" s="2" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L677" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M677" s="1" t="inlineStr">
-        <is>
-          <t>Rafaella Massuia</t>
-        </is>
-      </c>
-      <c r="N677" s="1" t="n"/>
-      <c r="O677" s="1" t="n"/>
-      <c r="P677" s="2" t="n">
-        <v>46275.83228032407</v>
-      </c>
-      <c r="Q677" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="R677" s="1" t="inlineStr">
-        <is>
-          <t>Segue proposta e simulado para parcelamento das inscrições 80 6 26 082503-45, 80 2 26 064060-04 e 80 2 26 064396-03, referente a notificação recebida.</t>
-        </is>
-      </c>
       <c r="S677" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -51956,26 +51942,26 @@
     </row>
     <row r="678">
       <c r="A678" s="1" t="n">
-        <v>83052</v>
+        <v>83704</v>
       </c>
       <c r="B678" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Levantamento de Débitos Mensal</t>
         </is>
       </c>
       <c r="C678" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa ICMS</t>
+          <t>PGFN</t>
         </is>
       </c>
       <c r="D678" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E678" s="1" t="inlineStr">
         <is>
-          <t>Empresa 6070 - Megacar. Há um débito na competência 05/2026, referente a um erro na transmissão da DeSTDA, em que foi informado indevidamente o valor de R$ 25.769,04.A declaração foi retificada em 20/08/2026, sem esse valor, porém a informação ainda não foi atualizada na SEFAZ.Solicito por gentileza que verifiquem se há alguma forma de agilizar a regularização dessa pendência.Seguem anexos o comprovante da DeSTDA retificada em 20/08/2026 e os registros que comprovam que não houve compras de fora do estado no período.</t>
+          <t>4200 - Henrique Leone- Por gentileza simular o parcelamento dos débitos que são mencionados na carta em anexo por favor.</t>
         </is>
       </c>
       <c r="F678" s="1" t="n">
@@ -51984,7 +51970,7 @@
       <c r="G678" s="1" t="n"/>
       <c r="H678" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I678" s="1" t="inlineStr">
@@ -51993,35 +51979,39 @@
         </is>
       </c>
       <c r="J678" s="2" t="n">
-        <v>46260.53714988426</v>
+        <v>46274.42889741898</v>
       </c>
       <c r="K678" s="2" t="n">
-        <v>46261</v>
+        <v>46276</v>
       </c>
       <c r="L678" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M678" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
-      <c r="N678" s="2" t="n">
-        <v>46288.64739603009</v>
-      </c>
+          <t>Rafaella Massuia</t>
+        </is>
+      </c>
+      <c r="N678" s="1" t="n"/>
       <c r="O678" s="1" t="n"/>
-      <c r="P678" s="1" t="n"/>
-      <c r="Q678" s="1" t="inlineStr"/>
+      <c r="P678" s="2" t="n">
+        <v>46275.83228032407</v>
+      </c>
+      <c r="Q678" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="R678" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por favor, verificar se foi aprovada a retificação. </t>
+          <t>Segue proposta e simulado para parcelamento das inscrições 80 6 26 082503-45, 80 2 26 064060-04 e 80 2 26 064396-03, referente a notificação recebida.</t>
         </is>
       </c>
       <c r="S678" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T678" s="1" t="n"/>
@@ -52029,11 +52019,11 @@
     </row>
     <row r="679">
       <c r="A679" s="1" t="n">
-        <v>83130</v>
+        <v>83052</v>
       </c>
       <c r="B679" s="1" t="inlineStr">
         <is>
-          <t>Levantamento de Débitos</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C679" s="1" t="inlineStr">
@@ -52043,12 +52033,12 @@
       </c>
       <c r="D679" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E679" s="1" t="inlineStr">
         <is>
-          <t>Cliente solicitou o levantamento de débitos da empresa 5551 - L.B. Hortifruti</t>
+          <t>Empresa 6070 - Megacar. Há um débito na competência 05/2026, referente a um erro na transmissão da DeSTDA, em que foi informado indevidamente o valor de R$ 25.769,04.A declaração foi retificada em 20/08/2026, sem esse valor, porém a informação ainda não foi atualizada na SEFAZ.Solicito por gentileza que verifiquem se há alguma forma de agilizar a regularização dessa pendência.Seguem anexos o comprovante da DeSTDA retificada em 20/08/2026 e os registros que comprovam que não houve compras de fora do estado no período.</t>
         </is>
       </c>
       <c r="F679" s="1" t="n">
@@ -52057,189 +52047,195 @@
       <c r="G679" s="1" t="n"/>
       <c r="H679" s="1" t="inlineStr">
         <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="I679" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J679" s="2" t="n">
+        <v>46260.53714988426</v>
+      </c>
+      <c r="K679" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="L679" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M679" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
+      <c r="N679" s="2" t="n">
+        <v>46288.64739603009</v>
+      </c>
+      <c r="O679" s="1" t="n"/>
+      <c r="P679" s="1" t="n"/>
+      <c r="Q679" s="1" t="inlineStr"/>
+      <c r="R679" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por favor, verificar se foi aprovada a retificação. </t>
+        </is>
+      </c>
+      <c r="S679" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T679" s="1" t="n"/>
+      <c r="U679" s="1" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" s="1" t="n">
+        <v>83130</v>
+      </c>
+      <c r="B680" s="1" t="inlineStr">
+        <is>
+          <t>Levantamento de Débitos</t>
+        </is>
+      </c>
+      <c r="C680" s="1" t="inlineStr">
+        <is>
+          <t>Divida Ativa ICMS</t>
+        </is>
+      </c>
+      <c r="D680" s="1" t="inlineStr">
+        <is>
+          <t>SANTOS - ADM</t>
+        </is>
+      </c>
+      <c r="E680" s="1" t="inlineStr">
+        <is>
+          <t>Cliente solicitou o levantamento de débitos da empresa 5551 - L.B. Hortifruti</t>
+        </is>
+      </c>
+      <c r="F680" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G680" s="1" t="n"/>
+      <c r="H680" s="1" t="inlineStr">
+        <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="I679" s="1" t="inlineStr">
+      <c r="I680" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J679" s="2" t="n">
+      <c r="J680" s="2" t="n">
         <v>46261.51850563657</v>
       </c>
-      <c r="K679" s="2" t="n">
+      <c r="K680" s="2" t="n">
         <v>46262</v>
       </c>
-      <c r="L679" s="1" t="inlineStr">
+      <c r="L680" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M679" s="1" t="inlineStr">
+      <c r="M680" s="1" t="inlineStr">
         <is>
           <t>Lidia Tavares</t>
         </is>
       </c>
-      <c r="N679" s="1" t="n"/>
-      <c r="O679" s="1" t="n"/>
-      <c r="P679" s="2" t="n">
+      <c r="N680" s="1" t="n"/>
+      <c r="O680" s="1" t="n"/>
+      <c r="P680" s="2" t="n">
         <v>46280.77373244213</v>
       </c>
-      <c r="Q679" s="1" t="inlineStr">
+      <c r="Q680" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R679" s="1" t="inlineStr">
+      <c r="R680" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lidia, bom dia!
 Essa empresa é filia, está correto a solicitação?
 Os débitos federais e estaduais são unificados com a matriz. </t>
         </is>
       </c>
-      <c r="S679" s="1" t="inlineStr">
+      <c r="S680" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="T679" s="1" t="n"/>
-      <c r="U679" s="1" t="inlineStr"/>
-    </row>
-    <row r="680">
-      <c r="A680" s="1" t="n">
+      <c r="T680" s="1" t="n"/>
+      <c r="U680" s="1" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" s="1" t="n">
         <v>83924</v>
       </c>
-      <c r="B680" s="1" t="inlineStr">
+      <c r="B681" s="1" t="inlineStr">
         <is>
           <t>Regularização</t>
         </is>
       </c>
-      <c r="C680" s="1" t="inlineStr">
+      <c r="C681" s="1" t="inlineStr">
         <is>
           <t>Prefeitura</t>
         </is>
       </c>
-      <c r="D680" s="1" t="inlineStr">
+      <c r="D681" s="1" t="inlineStr">
         <is>
           <t>SANTOS - GC</t>
         </is>
       </c>
-      <c r="E680" s="1" t="inlineStr">
+      <c r="E681" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">3828 - Supermercado Popular - Renovação do Cli </t>
         </is>
       </c>
-      <c r="F680" s="1" t="n">
+      <c r="F681" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G680" s="1" t="n"/>
-      <c r="H680" s="1" t="inlineStr">
+      <c r="G681" s="1" t="n"/>
+      <c r="H681" s="1" t="inlineStr">
         <is>
           <t>Edson Silva</t>
         </is>
       </c>
-      <c r="I680" s="1" t="inlineStr">
+      <c r="I681" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J680" s="2" t="n">
+      <c r="J681" s="2" t="n">
         <v>46279.40335633101</v>
       </c>
-      <c r="K680" s="2" t="n">
+      <c r="K681" s="2" t="n">
         <v>46281</v>
       </c>
-      <c r="L680" s="1" t="inlineStr">
+      <c r="L681" s="1" t="inlineStr">
         <is>
           <t>Em Atendimento</t>
         </is>
       </c>
-      <c r="M680" s="1" t="inlineStr">
+      <c r="M681" s="1" t="inlineStr">
         <is>
           <t>Rafaella Massuia</t>
         </is>
       </c>
-      <c r="N680" s="2" t="n">
+      <c r="N681" s="2" t="n">
         <v>46281.55550413195</v>
       </c>
-      <c r="O680" s="1" t="n"/>
-      <c r="P680" s="1" t="n"/>
-      <c r="Q680" s="1" t="inlineStr"/>
-      <c r="R680" s="1" t="inlineStr">
+      <c r="O681" s="1" t="n"/>
+      <c r="P681" s="1" t="n"/>
+      <c r="Q681" s="1" t="inlineStr"/>
+      <c r="R681" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 Aguardando o deferimento.
 Atenciosamente,</t>
         </is>
       </c>
-      <c r="S680" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T680" s="1" t="n"/>
-      <c r="U680" s="1" t="inlineStr"/>
-    </row>
-    <row r="681">
-      <c r="A681" s="1" t="n">
-        <v>83981</v>
-      </c>
-      <c r="B681" s="1" t="inlineStr">
-        <is>
-          <t>Regularização</t>
-        </is>
-      </c>
-      <c r="C681" s="1" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="D681" s="1" t="inlineStr">
-        <is>
-          <t>EF - INDUSTRIA</t>
-        </is>
-      </c>
-      <c r="E681" s="1" t="inlineStr">
-        <is>
-          <t>3262 - JCV - GNRE de ALPEC - AlagoasConforme solicitação no e-mail anexo, é necessário providenciar o preenchimento do REDAR, emissão da taxa e protocolar do processo junto à SEFAZ/AL.</t>
-        </is>
-      </c>
-      <c r="F681" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G681" s="1" t="n"/>
-      <c r="H681" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="I681" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J681" s="2" t="n">
-        <v>46280.38897322916</v>
-      </c>
-      <c r="K681" s="2" t="n">
-        <v>46282</v>
-      </c>
-      <c r="L681" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M681" s="1" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
-      <c r="N681" s="1" t="n"/>
-      <c r="O681" s="1" t="n"/>
-      <c r="P681" s="1" t="n"/>
-      <c r="Q681" s="1" t="inlineStr"/>
-      <c r="R681" s="1" t="inlineStr"/>
       <c r="S681" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52250,7 +52246,7 @@
     </row>
     <row r="682">
       <c r="A682" s="1" t="n">
-        <v>84060</v>
+        <v>83981</v>
       </c>
       <c r="B682" s="1" t="inlineStr">
         <is>
@@ -52269,7 +52265,7 @@
       </c>
       <c r="E682" s="1" t="inlineStr">
         <is>
-          <t>5132 - CABEXPRESS - Notificação GNRE UF MT.Nosso cliente recebeu uma notificação da SEFAZ de MT sobre o não pagamento da GNRE de uma venda referente à NF-e 45.008 que já havia sido recolhido em 04/09/2026, 10 dias antes da emissão do TAD em 14/09/2026.O valor principal cobrado no TAD é exatamente o mesmo valor que consta na GNRE paga R$ 1.204,18. Porém, o TAD indica que a fiscalização não reconheceu/localizou esse recolhimento no momento da abordagem, e por isso constituiu o débito e acrescentou multa.O documento informa a possibilidade de provar a regularidade, mas não apresenta de forma clara, um canal eletrônico específico, e-mail ou botão/link para enviar os comprovantes.Segue anexo o e-mail do cliente com a GNRE e o comprovante bancário para que vejam a possibilidade de solicitar a baixa/cancelamento da exigência TAD.</t>
+          <t>3262 - JCV - GNRE de ALPEC - AlagoasConforme solicitação no e-mail anexo, é necessário providenciar o preenchimento do REDAR, emissão da taxa e protocolar do processo junto à SEFAZ/AL.</t>
         </is>
       </c>
       <c r="F682" s="1" t="n">
@@ -52287,14 +52283,14 @@
         </is>
       </c>
       <c r="J682" s="2" t="n">
-        <v>46281.40508255787</v>
+        <v>46280.38897322916</v>
       </c>
       <c r="K682" s="2" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="L682" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M682" s="1" t="inlineStr">
@@ -52302,17 +52298,11 @@
           <t>Ricardo Fischer</t>
         </is>
       </c>
-      <c r="N682" s="2" t="n">
-        <v>46287.76335497685</v>
-      </c>
+      <c r="N682" s="1" t="n"/>
       <c r="O682" s="1" t="n"/>
       <c r="P682" s="1" t="n"/>
       <c r="Q682" s="1" t="inlineStr"/>
-      <c r="R682" s="1" t="inlineStr">
-        <is>
-          <t>Protocolado processo de baixa do auto, acompanhando o processo.</t>
-        </is>
-      </c>
+      <c r="R682" s="1" t="inlineStr"/>
       <c r="S682" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52323,26 +52313,26 @@
     </row>
     <row r="683">
       <c r="A683" s="1" t="n">
-        <v>84230</v>
+        <v>84060</v>
       </c>
       <c r="B683" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Guia</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C683" s="1" t="inlineStr">
         <is>
-          <t>DARF</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="D683" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL HOLDING</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E683" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde tudo bem?O cliente da empresa 1404 - ASMJ pagou um DARF referente ao mês 03/2026 no código incorreto, foi pago o DARF no valor de R$ 839,61 no código 2372 - CSLL, porem o correto seria o código 2089 - IRPJ Lucro presumido, se possível poderiam efetuar o REDARF por gentileza. Segue comprovante de arrecadação no código incorreto</t>
+          <t>5132 - CABEXPRESS - Notificação GNRE UF MT.Nosso cliente recebeu uma notificação da SEFAZ de MT sobre o não pagamento da GNRE de uma venda referente à NF-e 45.008 que já havia sido recolhido em 04/09/2026, 10 dias antes da emissão do TAD em 14/09/2026.O valor principal cobrado no TAD é exatamente o mesmo valor que consta na GNRE paga R$ 1.204,18. Porém, o TAD indica que a fiscalização não reconheceu/localizou esse recolhimento no momento da abordagem, e por isso constituiu o débito e acrescentou multa.O documento informa a possibilidade de provar a regularidade, mas não apresenta de forma clara, um canal eletrônico específico, e-mail ou botão/link para enviar os comprovantes.Segue anexo o e-mail do cliente com a GNRE e o comprovante bancário para que vejam a possibilidade de solicitar a baixa/cancelamento da exigência TAD.</t>
         </is>
       </c>
       <c r="F683" s="1" t="n">
@@ -52351,7 +52341,7 @@
       <c r="G683" s="1" t="n"/>
       <c r="H683" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I683" s="1" t="inlineStr">
@@ -52360,10 +52350,10 @@
         </is>
       </c>
       <c r="J683" s="2" t="n">
-        <v>46286.69414984954</v>
+        <v>46281.40508255787</v>
       </c>
       <c r="K683" s="2" t="n">
-        <v>46290</v>
+        <v>46283</v>
       </c>
       <c r="L683" s="1" t="inlineStr">
         <is>
@@ -52372,169 +52362,175 @@
       </c>
       <c r="M683" s="1" t="inlineStr">
         <is>
-          <t>Vitor de Souza</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="N683" s="2" t="n">
-        <v>46287.59273383102</v>
+        <v>46287.76335497685</v>
       </c>
       <c r="O683" s="1" t="n"/>
       <c r="P683" s="1" t="n"/>
       <c r="Q683" s="1" t="inlineStr"/>
       <c r="R683" s="1" t="inlineStr">
         <is>
+          <t>Protocolado processo de baixa do auto, acompanhando o processo.</t>
+        </is>
+      </c>
+      <c r="S683" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T683" s="1" t="n"/>
+      <c r="U683" s="1" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="1" t="n">
+        <v>84230</v>
+      </c>
+      <c r="B684" s="1" t="inlineStr">
+        <is>
+          <t>Retificação de Guia</t>
+        </is>
+      </c>
+      <c r="C684" s="1" t="inlineStr">
+        <is>
+          <t>DARF</t>
+        </is>
+      </c>
+      <c r="D684" s="1" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL HOLDING</t>
+        </is>
+      </c>
+      <c r="E684" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde tudo bem?O cliente da empresa 1404 - ASMJ pagou um DARF referente ao mês 03/2026 no código incorreto, foi pago o DARF no valor de R$ 839,61 no código 2372 - CSLL, porem o correto seria o código 2089 - IRPJ Lucro presumido, se possível poderiam efetuar o REDARF por gentileza. Segue comprovante de arrecadação no código incorreto</t>
+        </is>
+      </c>
+      <c r="F684" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G684" s="1" t="n"/>
+      <c r="H684" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="I684" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J684" s="2" t="n">
+        <v>46286.69414984954</v>
+      </c>
+      <c r="K684" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="L684" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M684" s="1" t="inlineStr">
+        <is>
+          <t>Vitor de Souza</t>
+        </is>
+      </c>
+      <c r="N684" s="2" t="n">
+        <v>46287.59273383102</v>
+      </c>
+      <c r="O684" s="1" t="n"/>
+      <c r="P684" s="1" t="n"/>
+      <c r="Q684" s="1" t="inlineStr"/>
+      <c r="R684" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Boa tarde!
 Redarf protocolado. </t>
         </is>
       </c>
-      <c r="S683" s="1" t="inlineStr">
+      <c r="S684" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T683" s="1" t="n"/>
-      <c r="U683" s="1" t="inlineStr"/>
-    </row>
-    <row r="684">
-      <c r="A684" s="1" t="n">
+      <c r="T684" s="1" t="n"/>
+      <c r="U684" s="1" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="1" t="n">
         <v>84244</v>
       </c>
-      <c r="B684" s="1" t="inlineStr">
+      <c r="B685" s="1" t="inlineStr">
         <is>
           <t>Parcelamento RFB</t>
         </is>
       </c>
-      <c r="C684" s="1" t="inlineStr">
+      <c r="C685" s="1" t="inlineStr">
         <is>
           <t>Simplificado</t>
         </is>
       </c>
-      <c r="D684" s="1" t="inlineStr">
+      <c r="D685" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
-      <c r="E684" s="1" t="inlineStr">
+      <c r="E685" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bom dia, por gentileza encaminhar extrato dos parcelamentos do grupo Medical Discovery, cliente quer saber as parcelas que já foram pagas e o que ainda consta em aberto. </t>
         </is>
       </c>
-      <c r="F684" s="1" t="n">
+      <c r="F685" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G684" s="1" t="n"/>
-      <c r="H684" s="1" t="inlineStr">
+      <c r="G685" s="1" t="n"/>
+      <c r="H685" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="I684" s="1" t="inlineStr">
+      <c r="I685" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J684" s="2" t="n">
+      <c r="J685" s="2" t="n">
         <v>46287.38990729167</v>
       </c>
-      <c r="K684" s="2" t="n">
+      <c r="K685" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="L684" s="1" t="inlineStr">
+      <c r="L685" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M684" s="1" t="inlineStr">
+      <c r="M685" s="1" t="inlineStr">
         <is>
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N684" s="1" t="n"/>
-      <c r="O684" s="1" t="n"/>
-      <c r="P684" s="2" t="n">
+      <c r="N685" s="1" t="n"/>
+      <c r="O685" s="1" t="n"/>
+      <c r="P685" s="2" t="n">
         <v>46287.7625866551</v>
       </c>
-      <c r="Q684" s="1" t="inlineStr">
+      <c r="Q685" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R684" s="1" t="inlineStr">
+      <c r="R685" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Boa noite!
 Segue. </t>
         </is>
       </c>
-      <c r="S684" s="1" t="inlineStr">
+      <c r="S685" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="T684" s="1" t="n"/>
-      <c r="U684" s="1" t="inlineStr"/>
-    </row>
-    <row r="685">
-      <c r="A685" s="1" t="n">
-        <v>84305</v>
-      </c>
-      <c r="B685" s="1" t="inlineStr">
-        <is>
-          <t>Senha</t>
-        </is>
-      </c>
-      <c r="C685" s="1" t="inlineStr">
-        <is>
-          <t>Prefeitura</t>
-        </is>
-      </c>
-      <c r="D685" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="E685" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde, por gentileza disponibilizar login e senha da prefeitura referente a empresa 6204 - Cucinare FL91.Obrigada!</t>
-        </is>
-      </c>
-      <c r="F685" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G685" s="1" t="n"/>
-      <c r="H685" s="1" t="inlineStr">
-        <is>
-          <t>Sarah Amaro</t>
-        </is>
-      </c>
-      <c r="I685" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J685" s="2" t="n">
-        <v>46287.64928989583</v>
-      </c>
-      <c r="K685" s="2" t="n">
-        <v>46289</v>
-      </c>
-      <c r="L685" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M685" s="1" t="inlineStr">
-        <is>
-          <t>Julia Medeiros</t>
-        </is>
-      </c>
-      <c r="N685" s="1" t="n"/>
-      <c r="O685" s="1" t="n"/>
-      <c r="P685" s="1" t="n"/>
-      <c r="Q685" s="1" t="inlineStr"/>
-      <c r="R685" s="1" t="inlineStr"/>
-      <c r="S685" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="T685" s="1" t="n"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-29 15:55
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1496,7 +1496,11 @@
           <t>Supermercado Kanashiro Ltda</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n"/>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -1510,7 +1514,7 @@
       </c>
       <c r="L13" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M13" s="1" t="inlineStr">
@@ -1519,17 +1523,23 @@
         </is>
       </c>
       <c r="N13" s="1" t="n"/>
-      <c r="O13" s="1" t="n"/>
+      <c r="O13" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P13" s="1" t="n"/>
       <c r="Q13" s="1" t="inlineStr"/>
-      <c r="R13" s="1" t="n"/>
+      <c r="R13" s="1" t="inlineStr"/>
       <c r="S13" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T13" s="1" t="n"/>
-      <c r="U13" s="1" t="inlineStr"/>
+      <c r="U13" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1677,7 +1687,9 @@
         </is>
       </c>
       <c r="N15" s="1" t="n"/>
-      <c r="O15" s="1" t="n"/>
+      <c r="O15" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P15" s="1" t="n"/>
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr"/>
@@ -1725,7 +1737,11 @@
           <t>BANDEIRANTES REFRIGERAÇÃO COMERCIAL LTDA</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n"/>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -1739,7 +1755,7 @@
       </c>
       <c r="L16" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M16" s="1" t="inlineStr">
@@ -1749,16 +1765,30 @@
       </c>
       <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
-      <c r="P16" s="1" t="n"/>
-      <c r="Q16" s="1" t="inlineStr"/>
-      <c r="R16" s="1" t="n"/>
+      <c r="P16" s="2" t="n">
+        <v>46294.63901493056</v>
+      </c>
+      <c r="Q16" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R16" s="1" t="inlineStr">
+        <is>
+          <t>Já foi ajustado e devolvido no analise.</t>
+        </is>
+      </c>
       <c r="S16" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T16" s="1" t="n"/>
-      <c r="U16" s="1" t="inlineStr"/>
+      <c r="U16" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -2363,7 +2393,11 @@
           <t>XERYU'S IMPORTADORA E DISTRIBUIDORA DE ARTIGOS PARA VESTUARIO LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n"/>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -2377,7 +2411,7 @@
       </c>
       <c r="L24" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M24" s="1" t="inlineStr">
@@ -2386,17 +2420,33 @@
         </is>
       </c>
       <c r="N24" s="1" t="n"/>
-      <c r="O24" s="1" t="n"/>
-      <c r="P24" s="1" t="n"/>
-      <c r="Q24" s="1" t="inlineStr"/>
-      <c r="R24" s="1" t="n"/>
+      <c r="O24" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>46294.65353996528</v>
+      </c>
+      <c r="Q24" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R24" s="1" t="inlineStr">
+        <is>
+          <t>respondido via email desde 11:20 da manha</t>
+        </is>
+      </c>
       <c r="S24" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T24" s="1" t="n"/>
-      <c r="U24" s="1" t="inlineStr"/>
+      <c r="U24" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -3272,7 +3322,11 @@
           <t>NALLINI MANUTENÇÃO DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H35" s="1" t="n"/>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
       <c r="I35" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -3286,7 +3340,7 @@
       </c>
       <c r="L35" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M35" s="1" t="inlineStr">
@@ -3295,17 +3349,23 @@
         </is>
       </c>
       <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
+      <c r="O35" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P35" s="1" t="n"/>
       <c r="Q35" s="1" t="inlineStr"/>
-      <c r="R35" s="1" t="n"/>
+      <c r="R35" s="1" t="inlineStr"/>
       <c r="S35" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T35" s="1" t="n"/>
-      <c r="U35" s="1" t="inlineStr"/>
+      <c r="U35" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -4441,7 +4501,7 @@
       </c>
       <c r="L49" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M49" s="1" t="inlineStr">
@@ -4449,12 +4509,20 @@
           <t>Simone Marques</t>
         </is>
       </c>
-      <c r="N49" s="1" t="n"/>
+      <c r="N49" s="2" t="n">
+        <v>46190.46143564815</v>
+      </c>
       <c r="O49" s="2" t="n">
         <v>46234</v>
       </c>
-      <c r="P49" s="1" t="n"/>
-      <c r="Q49" s="1" t="inlineStr"/>
+      <c r="P49" s="2" t="n">
+        <v>46294.6576278588</v>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="R49" s="1" t="inlineStr">
         <is>
           <t>Vai ser feito o levantamento</t>
@@ -4462,7 +4530,7 @@
       </c>
       <c r="S49" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T49" s="1" t="n"/>
@@ -6432,7 +6500,11 @@
           <t>V.B. MOREIRA LAVANDERIA</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n"/>
+      <c r="H73" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I73" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -6446,7 +6518,7 @@
       </c>
       <c r="L73" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M73" s="1" t="inlineStr">
@@ -6455,17 +6527,23 @@
         </is>
       </c>
       <c r="N73" s="1" t="n"/>
-      <c r="O73" s="1" t="n"/>
+      <c r="O73" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P73" s="1" t="n"/>
       <c r="Q73" s="1" t="inlineStr"/>
-      <c r="R73" s="1" t="n"/>
+      <c r="R73" s="1" t="inlineStr"/>
       <c r="S73" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T73" s="1" t="n"/>
-      <c r="U73" s="1" t="inlineStr"/>
+      <c r="U73" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -9333,7 +9411,11 @@
           <t>YARA DESIGN E DECORAÇÃO LTDA</t>
         </is>
       </c>
-      <c r="H107" s="1" t="n"/>
+      <c r="H107" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
       <c r="I107" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -9347,7 +9429,7 @@
       </c>
       <c r="L107" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M107" s="1" t="inlineStr">
@@ -9356,17 +9438,23 @@
         </is>
       </c>
       <c r="N107" s="1" t="n"/>
-      <c r="O107" s="1" t="n"/>
+      <c r="O107" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P107" s="1" t="n"/>
       <c r="Q107" s="1" t="inlineStr"/>
-      <c r="R107" s="1" t="n"/>
+      <c r="R107" s="1" t="inlineStr"/>
       <c r="S107" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T107" s="1" t="n"/>
-      <c r="U107" s="1" t="inlineStr"/>
+      <c r="U107" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -12999,7 +13087,11 @@
           <t>GHOST KITCHENS ALIMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H151" s="1" t="n"/>
+      <c r="H151" s="1" t="inlineStr">
+        <is>
+          <t>Edileide Dias</t>
+        </is>
+      </c>
       <c r="I151" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -13013,7 +13105,7 @@
       </c>
       <c r="L151" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M151" s="1" t="inlineStr">
@@ -13022,17 +13114,23 @@
         </is>
       </c>
       <c r="N151" s="1" t="n"/>
-      <c r="O151" s="1" t="n"/>
+      <c r="O151" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P151" s="1" t="n"/>
       <c r="Q151" s="1" t="inlineStr"/>
-      <c r="R151" s="1" t="n"/>
+      <c r="R151" s="1" t="inlineStr"/>
       <c r="S151" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T151" s="1" t="n"/>
-      <c r="U151" s="1" t="inlineStr"/>
+      <c r="U151" s="1" t="inlineStr">
+        <is>
+          <t>Edileide Dias</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -13066,7 +13164,11 @@
           <t>BLACK KITCHENS ALIMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H152" s="1" t="n"/>
+      <c r="H152" s="1" t="inlineStr">
+        <is>
+          <t>Edileide Dias</t>
+        </is>
+      </c>
       <c r="I152" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -13080,7 +13182,7 @@
       </c>
       <c r="L152" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M152" s="1" t="inlineStr">
@@ -13089,17 +13191,23 @@
         </is>
       </c>
       <c r="N152" s="1" t="n"/>
-      <c r="O152" s="1" t="n"/>
+      <c r="O152" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P152" s="1" t="n"/>
       <c r="Q152" s="1" t="inlineStr"/>
-      <c r="R152" s="1" t="n"/>
+      <c r="R152" s="1" t="inlineStr"/>
       <c r="S152" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T152" s="1" t="n"/>
-      <c r="U152" s="1" t="inlineStr"/>
+      <c r="U152" s="1" t="inlineStr">
+        <is>
+          <t>Edileide Dias</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -15080,7 +15188,7 @@
       </c>
       <c r="L176" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M176" s="1" t="inlineStr">
@@ -15088,12 +15196,20 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N176" s="1" t="n"/>
+      <c r="N176" s="2" t="n">
+        <v>46290.65051751157</v>
+      </c>
       <c r="O176" s="2" t="n">
         <v>46294</v>
       </c>
-      <c r="P176" s="1" t="n"/>
-      <c r="Q176" s="1" t="inlineStr"/>
+      <c r="P176" s="2" t="n">
+        <v>46294.64589545139</v>
+      </c>
+      <c r="Q176" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="R176" s="1" t="inlineStr">
         <is>
           <t>Analisando</t>
@@ -15101,7 +15217,7 @@
       </c>
       <c r="S176" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T176" s="1" t="n"/>
@@ -15301,7 +15417,11 @@
           <t>ESPETINHO VILA MARIANA LTDA</t>
         </is>
       </c>
-      <c r="H179" s="1" t="n"/>
+      <c r="H179" s="1" t="inlineStr">
+        <is>
+          <t>Lucas Fischer</t>
+        </is>
+      </c>
       <c r="I179" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -15315,7 +15435,7 @@
       </c>
       <c r="L179" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M179" s="1" t="inlineStr">
@@ -15324,17 +15444,23 @@
         </is>
       </c>
       <c r="N179" s="1" t="n"/>
-      <c r="O179" s="1" t="n"/>
+      <c r="O179" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P179" s="1" t="n"/>
       <c r="Q179" s="1" t="inlineStr"/>
-      <c r="R179" s="1" t="n"/>
+      <c r="R179" s="1" t="inlineStr"/>
       <c r="S179" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T179" s="1" t="n"/>
-      <c r="U179" s="1" t="inlineStr"/>
+      <c r="U179" s="1" t="inlineStr">
+        <is>
+          <t>Lucas Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -15936,7 +16062,11 @@
           <t>OBA OBA MIX LTDA</t>
         </is>
       </c>
-      <c r="H187" s="1" t="n"/>
+      <c r="H187" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I187" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -15950,7 +16080,7 @@
       </c>
       <c r="L187" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M187" s="1" t="inlineStr">
@@ -15959,17 +16089,23 @@
         </is>
       </c>
       <c r="N187" s="1" t="n"/>
-      <c r="O187" s="1" t="n"/>
+      <c r="O187" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P187" s="1" t="n"/>
       <c r="Q187" s="1" t="inlineStr"/>
-      <c r="R187" s="1" t="n"/>
+      <c r="R187" s="1" t="inlineStr"/>
       <c r="S187" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T187" s="1" t="n"/>
-      <c r="U187" s="1" t="inlineStr"/>
+      <c r="U187" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -16488,7 +16624,11 @@
           <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
         </is>
       </c>
-      <c r="H194" s="1" t="n"/>
+      <c r="H194" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I194" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -16502,7 +16642,7 @@
       </c>
       <c r="L194" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M194" s="1" t="inlineStr">
@@ -16511,17 +16651,33 @@
         </is>
       </c>
       <c r="N194" s="1" t="n"/>
-      <c r="O194" s="1" t="n"/>
-      <c r="P194" s="1" t="n"/>
-      <c r="Q194" s="1" t="inlineStr"/>
-      <c r="R194" s="1" t="n"/>
+      <c r="O194" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="P194" s="2" t="n">
+        <v>46294.65183695602</v>
+      </c>
+      <c r="Q194" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R194" s="1" t="inlineStr">
+        <is>
+          <t>Foi enviado por email, cliente solicita guias recalculadas ref outros anos mensalmente. ja foi enviado.</t>
+        </is>
+      </c>
       <c r="S194" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T194" s="1" t="n"/>
-      <c r="U194" s="1" t="inlineStr"/>
+      <c r="U194" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -17412,7 +17568,7 @@
       </c>
       <c r="L205" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M205" s="1" t="inlineStr">
@@ -17420,12 +17576,20 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N205" s="1" t="n"/>
+      <c r="N205" s="2" t="n">
+        <v>46290.6504658912</v>
+      </c>
       <c r="O205" s="2" t="n">
         <v>46295</v>
       </c>
-      <c r="P205" s="1" t="n"/>
-      <c r="Q205" s="1" t="inlineStr"/>
+      <c r="P205" s="2" t="n">
+        <v>46294.64073244213</v>
+      </c>
+      <c r="Q205" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="R205" s="1" t="inlineStr">
         <is>
           <t>Analisando</t>
@@ -17433,7 +17597,7 @@
       </c>
       <c r="S205" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T205" s="1" t="n"/>
@@ -18750,7 +18914,11 @@
           <t>BOMBEIROS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANÇA LTDA</t>
         </is>
       </c>
-      <c r="H221" s="1" t="n"/>
+      <c r="H221" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
       <c r="I221" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -18764,7 +18932,7 @@
       </c>
       <c r="L221" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M221" s="1" t="inlineStr">
@@ -18773,17 +18941,23 @@
         </is>
       </c>
       <c r="N221" s="1" t="n"/>
-      <c r="O221" s="1" t="n"/>
+      <c r="O221" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P221" s="1" t="n"/>
       <c r="Q221" s="1" t="inlineStr"/>
-      <c r="R221" s="1" t="n"/>
+      <c r="R221" s="1" t="inlineStr"/>
       <c r="S221" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T221" s="1" t="n"/>
-      <c r="U221" s="1" t="inlineStr"/>
+      <c r="U221" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -18817,7 +18991,11 @@
           <t>COMBATEAINCENDIOS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANCA LTDA</t>
         </is>
       </c>
-      <c r="H222" s="1" t="n"/>
+      <c r="H222" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
       <c r="I222" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -18831,7 +19009,7 @@
       </c>
       <c r="L222" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M222" s="1" t="inlineStr">
@@ -18840,17 +19018,23 @@
         </is>
       </c>
       <c r="N222" s="1" t="n"/>
-      <c r="O222" s="1" t="n"/>
+      <c r="O222" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P222" s="1" t="n"/>
       <c r="Q222" s="1" t="inlineStr"/>
-      <c r="R222" s="1" t="n"/>
+      <c r="R222" s="1" t="inlineStr"/>
       <c r="S222" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T222" s="1" t="n"/>
-      <c r="U222" s="1" t="inlineStr"/>
+      <c r="U222" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -20329,7 +20513,7 @@
       </c>
       <c r="L240" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M240" s="1" t="inlineStr">
@@ -20343,8 +20527,14 @@
       <c r="O240" s="2" t="n">
         <v>46295</v>
       </c>
-      <c r="P240" s="1" t="n"/>
-      <c r="Q240" s="1" t="inlineStr"/>
+      <c r="P240" s="2" t="n">
+        <v>46294.64758487268</v>
+      </c>
+      <c r="Q240" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="R240" s="1" t="inlineStr">
         <is>
           <t>Analisando</t>
@@ -20352,7 +20542,7 @@
       </c>
       <c r="S240" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T240" s="1" t="n"/>
@@ -20424,7 +20614,7 @@
         <v>46276.6543150463</v>
       </c>
       <c r="O241" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="P241" s="1" t="n"/>
       <c r="Q241" s="1" t="inlineStr"/>
@@ -64146,7 +64336,7 @@
       </c>
       <c r="L836" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M836" s="1" t="inlineStr">
@@ -64154,7 +64344,9 @@
           <t>Ney Barbosa</t>
         </is>
       </c>
-      <c r="N836" s="1" t="n"/>
+      <c r="N836" s="2" t="n">
+        <v>46294.64554829861</v>
+      </c>
       <c r="O836" s="1" t="n"/>
       <c r="P836" s="1" t="n"/>
       <c r="Q836" s="1" t="inlineStr"/>
@@ -67915,7 +68107,7 @@
       </c>
       <c r="L887" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M887" s="1" t="inlineStr">
@@ -67923,7 +68115,9 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N887" s="1" t="n"/>
+      <c r="N887" s="2" t="n">
+        <v>46261.69782774305</v>
+      </c>
       <c r="O887" s="2" t="n">
         <v>46297</v>
       </c>
@@ -68071,7 +68265,7 @@
       </c>
       <c r="L889" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M889" s="1" t="inlineStr">
@@ -68079,7 +68273,9 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N889" s="1" t="n"/>
+      <c r="N889" s="2" t="n">
+        <v>46261.69765454861</v>
+      </c>
       <c r="O889" s="2" t="n">
         <v>46283</v>
       </c>
@@ -68148,7 +68344,7 @@
       </c>
       <c r="L890" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M890" s="1" t="inlineStr">
@@ -68156,7 +68352,9 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N890" s="1" t="n"/>
+      <c r="N890" s="2" t="n">
+        <v>46261.69723422454</v>
+      </c>
       <c r="O890" s="2" t="n">
         <v>46283</v>
       </c>
@@ -68225,7 +68423,7 @@
       </c>
       <c r="L891" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M891" s="1" t="inlineStr">
@@ -68233,7 +68431,9 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N891" s="1" t="n"/>
+      <c r="N891" s="2" t="n">
+        <v>46259.7507258449</v>
+      </c>
       <c r="O891" s="2" t="n">
         <v>46297</v>
       </c>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-29 18:23
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -11250,7 +11250,11 @@
           <t>RJR INDUSTRIA DE ALIMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H129" s="1" t="n"/>
+      <c r="H129" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I129" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -11264,7 +11268,7 @@
       </c>
       <c r="L129" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M129" s="1" t="inlineStr">
@@ -11273,17 +11277,23 @@
         </is>
       </c>
       <c r="N129" s="1" t="n"/>
-      <c r="O129" s="1" t="n"/>
+      <c r="O129" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P129" s="1" t="n"/>
       <c r="Q129" s="1" t="inlineStr"/>
-      <c r="R129" s="1" t="n"/>
+      <c r="R129" s="1" t="inlineStr"/>
       <c r="S129" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T129" s="1" t="n"/>
-      <c r="U129" s="1" t="inlineStr"/>
+      <c r="U129" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -16141,7 +16151,11 @@
           <t>OBA OBA MIX LTDA</t>
         </is>
       </c>
-      <c r="H188" s="1" t="n"/>
+      <c r="H188" s="1" t="inlineStr">
+        <is>
+          <t>Kaique Souza</t>
+        </is>
+      </c>
       <c r="I188" s="1" t="inlineStr">
         <is>
           <t>DP - DEPTO. PESSOAL</t>
@@ -16155,7 +16169,7 @@
       </c>
       <c r="L188" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M188" s="1" t="inlineStr">
@@ -16163,18 +16177,28 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N188" s="1" t="n"/>
+      <c r="N188" s="2" t="n">
+        <v>46294.75443252315</v>
+      </c>
       <c r="O188" s="1" t="n"/>
       <c r="P188" s="1" t="n"/>
       <c r="Q188" s="1" t="inlineStr"/>
-      <c r="R188" s="1" t="n"/>
+      <c r="R188" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento.</t>
+        </is>
+      </c>
       <c r="S188" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T188" s="1" t="n"/>
-      <c r="U188" s="1" t="inlineStr"/>
+      <c r="U188" s="1" t="inlineStr">
+        <is>
+          <t>Sara Cavalheiro</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -18166,7 +18190,7 @@
       </c>
       <c r="I212" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J212" s="2" t="n">
@@ -18177,7 +18201,7 @@
       </c>
       <c r="L212" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M212" s="1" t="inlineStr">
@@ -18199,7 +18223,11 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T212" s="1" t="n"/>
+      <c r="T212" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
       <c r="U212" s="1" t="inlineStr">
         <is>
           <t>Sara Cavalheiro</t>
@@ -61287,7 +61315,7 @@
       </c>
       <c r="L796" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M796" s="1" t="inlineStr">
@@ -61299,7 +61327,12 @@
       <c r="O796" s="1" t="n"/>
       <c r="P796" s="1" t="n"/>
       <c r="Q796" s="1" t="inlineStr"/>
-      <c r="R796" s="1" t="inlineStr"/>
+      <c r="R796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde!
+As guias são recalculadas para o dia, verifique com o cliente quando ele deseja efetuar o pagamento, que enviaremos as guias no primeiro horario. </t>
+        </is>
+      </c>
       <c r="S796" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-13 13:07
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -9843,7 +9843,11 @@
           <t>YARA DESIGN E DECORAÇÃO LTDA</t>
         </is>
       </c>
-      <c r="H112" s="1" t="n"/>
+      <c r="H112" s="1" t="inlineStr">
+        <is>
+          <t>Eveny Silva</t>
+        </is>
+      </c>
       <c r="I112" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -9857,7 +9861,7 @@
       </c>
       <c r="L112" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M112" s="1" t="inlineStr">
@@ -9869,14 +9873,18 @@
       <c r="O112" s="1" t="n"/>
       <c r="P112" s="1" t="n"/>
       <c r="Q112" s="1" t="inlineStr"/>
-      <c r="R112" s="1" t="n"/>
+      <c r="R112" s="1" t="inlineStr"/>
       <c r="S112" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T112" s="1" t="n"/>
-      <c r="U112" s="1" t="inlineStr"/>
+      <c r="U112" s="1" t="inlineStr">
+        <is>
+          <t>Karina Fonseca</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -13768,7 +13776,7 @@
       </c>
       <c r="L159" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M159" s="1" t="inlineStr">
@@ -13778,12 +13786,22 @@
       </c>
       <c r="N159" s="1" t="n"/>
       <c r="O159" s="1" t="n"/>
-      <c r="P159" s="1" t="n"/>
-      <c r="Q159" s="1" t="inlineStr"/>
-      <c r="R159" s="1" t="inlineStr"/>
+      <c r="P159" s="2" t="n">
+        <v>46308.53981504629</v>
+      </c>
+      <c r="Q159" s="1" t="inlineStr">
+        <is>
+          <t>Eveny Silva</t>
+        </is>
+      </c>
+      <c r="R159" s="1" t="inlineStr">
+        <is>
+          <t>Despesas de agosto verificadas. Aguardando financeiro referente ao mês 09.</t>
+        </is>
+      </c>
       <c r="S159" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T159" s="1" t="n"/>

</xml_diff>